<commit_message>
Various Data Migration Improvements (#49)
* uat dataflow IDs have been udpated. We need to update the json to keep the new values

* uat updates

* updating dataflows to allow for mapping a legacy view in the admin view on Request.

* adding javascript to show/hide the legacy data on the admin view

* data changes to test fields that previously had no test data to migrate

* fixing mapping issue for Cons

* fixing issue with acquisition approach

* adding default and env var configs

* workbook updates

* adding comment back
</commit_message>
<xml_diff>
--- a/apps/it-governance/migrations/IT Governance Intake Request Mapping Workbook.xlsx
+++ b/apps/it-governance/migrations/IT Governance Intake Request Mapping Workbook.xlsx
@@ -2,19 +2,19 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="business_cases" sheetId="1" r:id="Raa2048d5864c45d8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="estimated_lifecycle_costs" sheetId="2" r:id="Rdeeb80f95031434a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="governance_request_feedback" sheetId="3" r:id="R88cf3fe092a946ce"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="system_intake_contacts" sheetId="4" r:id="Raed67096c69649c5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="system_intake_contract_numbers" sheetId="5" r:id="Re33d0de759dd4ad9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="system_intake_documents" sheetId="6" r:id="R9526d935c67e4d25"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="system_intake_funding_sources" sheetId="7" r:id="Rbc281eda52be4df4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="system_intake_systems" sheetId="8" r:id="Rca8f6e32fbfc4ff3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="system_intakes" sheetId="9" r:id="R15a31044fbbe49e2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="system_intake_grb_reviewers" sheetId="10" r:id="Rf77b121e0894415e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="system_intake_grb_presentation_" sheetId="11" r:id="Rbd6d46345c034856"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="system_intake_internal_grb_revi" sheetId="12" r:id="Ra01b189569024f90"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mapping Governance" sheetId="14" r:id="Rc5cb33ff034a49e8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="business_cases" sheetId="1" r:id="Rf649c00947fd4e20"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="estimated_lifecycle_costs" sheetId="2" r:id="Ra2f3542a3cd54e64"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="governance_request_feedback" sheetId="3" r:id="R347f91b2f04a4b62"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="system_intake_contacts" sheetId="4" r:id="R7495fbcf9d57476f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="system_intake_contract_numbers" sheetId="5" r:id="Ra23d57fbf20c477e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="system_intake_documents" sheetId="6" r:id="Re499d6d619664390"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="system_intake_funding_sources" sheetId="7" r:id="R354da069328e43b2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="system_intake_systems" sheetId="8" r:id="R721178315b424ca7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="system_intakes" sheetId="9" r:id="Re5cc73f08f0241a5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="system_intake_grb_reviewers" sheetId="10" r:id="R0389533f04144139"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="system_intake_grb_presentation_" sheetId="11" r:id="Rc6b44bc9cc0248bf"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="system_intake_internal_grb_revi" sheetId="12" r:id="Rea45f73267294503"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mapping Governance" sheetId="14" r:id="Rebda621c9be549ca"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -166,13 +166,7 @@
     <x:t xml:space="preserve">preferred_pros</x:t>
   </x:si>
   <x:si>
-    <x:t xml:space="preserve">cr69a_Pros</x:t>
-  </x:si>
-  <x:si>
     <x:t xml:space="preserve">preferred_cons</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">cr69a_Cons</x:t>
   </x:si>
   <x:si>
     <x:t xml:space="preserve">preferred_cost_savings</x:t>
@@ -2728,8 +2722,8 @@
       <x:c r="A21" s="1" t="s">
         <x:v>47</x:v>
       </x:c>
-      <x:c r="B21" s="1" t="s">
-        <x:v>48</x:v>
+      <x:c r="B21" s="1" t="str">
+        <x:v>cr69a_ProsMulti</x:v>
       </x:c>
       <x:c r="C21" s="1" t="s">
         <x:v>41</x:v>
@@ -2755,10 +2749,10 @@
     </x:row>
     <x:row r="22">
       <x:c r="A22" s="1" t="s">
-        <x:v>49</x:v>
-      </x:c>
-      <x:c r="B22" s="1" t="s">
-        <x:v>50</x:v>
+        <x:v>48</x:v>
+      </x:c>
+      <x:c r="B22" s="1" t="str">
+        <x:v>cr69a_ConsMulti</x:v>
       </x:c>
       <x:c r="C22" s="1" t="s">
         <x:v>41</x:v>
@@ -2784,10 +2778,10 @@
     </x:row>
     <x:row r="23">
       <x:c r="A23" s="1" t="s">
-        <x:v>51</x:v>
+        <x:v>49</x:v>
       </x:c>
       <x:c r="B23" s="1" t="s">
-        <x:v>52</x:v>
+        <x:v>50</x:v>
       </x:c>
       <x:c r="C23" s="1" t="s">
         <x:v>41</x:v>
@@ -2814,7 +2808,7 @@
     </x:row>
     <x:row r="24">
       <x:c r="A24" s="1" t="s">
-        <x:v>53</x:v>
+        <x:v>51</x:v>
       </x:c>
       <x:c r="B24" s="1" t="s">
         <x:v>40</x:v>
@@ -2841,7 +2835,7 @@
     </x:row>
     <x:row r="25">
       <x:c r="A25" s="1" t="s">
-        <x:v>54</x:v>
+        <x:v>52</x:v>
       </x:c>
       <x:c r="B25" s="1" t="s">
         <x:v>43</x:v>
@@ -2868,7 +2862,7 @@
     </x:row>
     <x:row r="26">
       <x:c r="A26" s="1" t="s">
-        <x:v>55</x:v>
+        <x:v>53</x:v>
       </x:c>
       <x:c r="B26" s="1" t="s">
         <x:v>45</x:v>
@@ -2898,10 +2892,10 @@
     </x:row>
     <x:row r="27">
       <x:c r="A27" s="1" t="s">
-        <x:v>56</x:v>
-      </x:c>
-      <x:c r="B27" s="1" t="s">
-        <x:v>48</x:v>
+        <x:v>54</x:v>
+      </x:c>
+      <x:c r="B27" s="1" t="str">
+        <x:v>cr69a_ProsMulti</x:v>
       </x:c>
       <x:c r="C27" s="1" t="s">
         <x:v>41</x:v>
@@ -2928,10 +2922,10 @@
     </x:row>
     <x:row r="28">
       <x:c r="A28" s="1" t="s">
-        <x:v>57</x:v>
-      </x:c>
-      <x:c r="B28" s="1" t="s">
-        <x:v>50</x:v>
+        <x:v>55</x:v>
+      </x:c>
+      <x:c r="B28" s="1" t="str">
+        <x:v>cr69a_ConsMulti</x:v>
       </x:c>
       <x:c r="C28" s="1" t="s">
         <x:v>41</x:v>
@@ -2958,10 +2952,10 @@
     </x:row>
     <x:row r="29">
       <x:c r="A29" s="1" t="s">
-        <x:v>58</x:v>
+        <x:v>56</x:v>
       </x:c>
       <x:c r="B29" s="1" t="s">
-        <x:v>52</x:v>
+        <x:v>50</x:v>
       </x:c>
       <x:c r="C29" s="1" t="s">
         <x:v>41</x:v>
@@ -2988,7 +2982,7 @@
     </x:row>
     <x:row r="30">
       <x:c r="A30" s="1" t="s">
-        <x:v>59</x:v>
+        <x:v>57</x:v>
       </x:c>
       <x:c r="B30" s="1" t="s">
         <x:v>40</x:v>
@@ -3015,7 +3009,7 @@
     </x:row>
     <x:row r="31">
       <x:c r="A31" s="1" t="s">
-        <x:v>60</x:v>
+        <x:v>58</x:v>
       </x:c>
       <x:c r="B31" s="1" t="s">
         <x:v>43</x:v>
@@ -3042,7 +3036,7 @@
     </x:row>
     <x:row r="32">
       <x:c r="A32" s="1" t="s">
-        <x:v>61</x:v>
+        <x:v>59</x:v>
       </x:c>
       <x:c r="B32" s="1" t="s">
         <x:v>45</x:v>
@@ -3072,10 +3066,10 @@
     </x:row>
     <x:row r="33">
       <x:c r="A33" s="1" t="s">
-        <x:v>62</x:v>
-      </x:c>
-      <x:c r="B33" s="1" t="s">
-        <x:v>48</x:v>
+        <x:v>60</x:v>
+      </x:c>
+      <x:c r="B33" s="1" t="str">
+        <x:v>cr69a_ProsMulti</x:v>
       </x:c>
       <x:c r="C33" s="1" t="s">
         <x:v>41</x:v>
@@ -3102,10 +3096,10 @@
     </x:row>
     <x:row r="34">
       <x:c r="A34" s="1" t="s">
-        <x:v>63</x:v>
-      </x:c>
-      <x:c r="B34" s="1" t="s">
-        <x:v>50</x:v>
+        <x:v>61</x:v>
+      </x:c>
+      <x:c r="B34" s="1" t="str">
+        <x:v>cr69a_ConsMulti</x:v>
       </x:c>
       <x:c r="C34" s="1" t="s">
         <x:v>41</x:v>
@@ -3132,10 +3126,10 @@
     </x:row>
     <x:row r="35">
       <x:c r="A35" s="1" t="s">
-        <x:v>64</x:v>
+        <x:v>62</x:v>
       </x:c>
       <x:c r="B35" s="1" t="s">
-        <x:v>52</x:v>
+        <x:v>50</x:v>
       </x:c>
       <x:c r="C35" s="1" t="s">
         <x:v>41</x:v>
@@ -3161,7 +3155,7 @@
     </x:row>
     <x:row r="36">
       <x:c r="A36" s="1" t="s">
-        <x:v>65</x:v>
+        <x:v>63</x:v>
       </x:c>
       <x:c r="B36" s="1" t="s">
         <x:v>19</x:v>
@@ -3171,7 +3165,7 @@
     </x:row>
     <x:row r="37">
       <x:c r="A37" s="1" t="s">
-        <x:v>66</x:v>
+        <x:v>64</x:v>
       </x:c>
       <x:c r="B37" s="1" t="s">
         <x:v>19</x:v>
@@ -3181,7 +3175,7 @@
     </x:row>
     <x:row r="38">
       <x:c r="A38" s="1" t="s">
-        <x:v>67</x:v>
+        <x:v>65</x:v>
       </x:c>
       <x:c r="B38" s="1" t="s">
         <x:v>19</x:v>
@@ -3191,36 +3185,36 @@
     </x:row>
     <x:row r="39">
       <x:c r="A39" s="1" t="s">
-        <x:v>68</x:v>
+        <x:v>66</x:v>
       </x:c>
       <x:c r="B39" s="1" t="s">
-        <x:v>69</x:v>
+        <x:v>67</x:v>
       </x:c>
       <x:c r="C39" s="16" t="s">
         <x:v>27</x:v>
       </x:c>
       <x:c r="D39" s="1" t="s">
+        <x:v>68</x:v>
+      </x:c>
+      <x:c r="E39" s="1" t="s">
+        <x:v>69</x:v>
+      </x:c>
+      <x:c r="F39" s="1" t="s">
         <x:v>70</x:v>
-      </x:c>
-      <x:c r="E39" s="1" t="s">
-        <x:v>71</x:v>
-      </x:c>
-      <x:c r="F39" s="1" t="s">
-        <x:v>72</x:v>
       </x:c>
       <x:c r="H39" s="5">
         <x:v>100.0</x:v>
       </x:c>
       <x:c r="I39" s="5" t="s">
-        <x:v>73</x:v>
+        <x:v>71</x:v>
       </x:c>
     </x:row>
     <x:row r="40">
       <x:c r="A40" s="1" t="s">
-        <x:v>74</x:v>
+        <x:v>72</x:v>
       </x:c>
       <x:c r="B40" s="1" t="s">
-        <x:v>75</x:v>
+        <x:v>73</x:v>
       </x:c>
       <x:c r="C40" s="1" t="s">
         <x:v>41</x:v>
@@ -3243,10 +3237,10 @@
     </x:row>
     <x:row r="41">
       <x:c r="A41" s="1" t="s">
-        <x:v>76</x:v>
+        <x:v>74</x:v>
       </x:c>
       <x:c r="B41" s="1" t="s">
-        <x:v>77</x:v>
+        <x:v>75</x:v>
       </x:c>
       <x:c r="C41" s="1" t="s">
         <x:v>41</x:v>
@@ -3269,10 +3263,10 @@
     </x:row>
     <x:row r="42">
       <x:c r="A42" s="1" t="s">
-        <x:v>78</x:v>
+        <x:v>76</x:v>
       </x:c>
       <x:c r="B42" s="1" t="s">
-        <x:v>79</x:v>
+        <x:v>77</x:v>
       </x:c>
       <x:c r="C42" s="1" t="s">
         <x:v>41</x:v>
@@ -3295,10 +3289,10 @@
     </x:row>
     <x:row r="43">
       <x:c r="A43" s="1" t="s">
-        <x:v>80</x:v>
+        <x:v>78</x:v>
       </x:c>
       <x:c r="B43" s="1" t="s">
-        <x:v>81</x:v>
+        <x:v>79</x:v>
       </x:c>
       <x:c r="C43" s="1" t="s">
         <x:v>41</x:v>
@@ -3321,10 +3315,10 @@
     </x:row>
     <x:row r="44">
       <x:c r="A44" s="1" t="s">
-        <x:v>82</x:v>
+        <x:v>80</x:v>
       </x:c>
       <x:c r="B44" s="1" t="s">
-        <x:v>75</x:v>
+        <x:v>73</x:v>
       </x:c>
       <x:c r="C44" s="1" t="s">
         <x:v>41</x:v>
@@ -3347,10 +3341,10 @@
     </x:row>
     <x:row r="45">
       <x:c r="A45" s="1" t="s">
-        <x:v>83</x:v>
+        <x:v>81</x:v>
       </x:c>
       <x:c r="B45" s="1" t="s">
-        <x:v>77</x:v>
+        <x:v>75</x:v>
       </x:c>
       <x:c r="C45" s="1" t="s">
         <x:v>41</x:v>
@@ -3373,10 +3367,10 @@
     </x:row>
     <x:row r="46">
       <x:c r="A46" s="1" t="s">
-        <x:v>84</x:v>
+        <x:v>82</x:v>
       </x:c>
       <x:c r="B46" s="1" t="s">
-        <x:v>79</x:v>
+        <x:v>77</x:v>
       </x:c>
       <x:c r="C46" s="1" t="s">
         <x:v>41</x:v>
@@ -3399,10 +3393,10 @@
     </x:row>
     <x:row r="47">
       <x:c r="A47" s="1" t="s">
-        <x:v>85</x:v>
+        <x:v>83</x:v>
       </x:c>
       <x:c r="B47" s="1" t="s">
-        <x:v>81</x:v>
+        <x:v>79</x:v>
       </x:c>
       <x:c r="C47" s="1" t="s">
         <x:v>41</x:v>
@@ -3425,10 +3419,10 @@
     </x:row>
     <x:row r="48">
       <x:c r="A48" s="1" t="s">
-        <x:v>86</x:v>
+        <x:v>84</x:v>
       </x:c>
       <x:c r="B48" s="1" t="s">
-        <x:v>75</x:v>
+        <x:v>73</x:v>
       </x:c>
       <x:c r="C48" s="1" t="s">
         <x:v>41</x:v>
@@ -3451,10 +3445,10 @@
     </x:row>
     <x:row r="49">
       <x:c r="A49" s="1" t="s">
-        <x:v>87</x:v>
+        <x:v>85</x:v>
       </x:c>
       <x:c r="B49" s="1" t="s">
-        <x:v>77</x:v>
+        <x:v>75</x:v>
       </x:c>
       <x:c r="C49" s="1" t="s">
         <x:v>41</x:v>
@@ -3477,10 +3471,10 @@
     </x:row>
     <x:row r="50">
       <x:c r="A50" s="1" t="s">
-        <x:v>88</x:v>
+        <x:v>86</x:v>
       </x:c>
       <x:c r="B50" s="1" t="s">
-        <x:v>79</x:v>
+        <x:v>77</x:v>
       </x:c>
       <x:c r="C50" s="1" t="s">
         <x:v>41</x:v>
@@ -3503,10 +3497,10 @@
     </x:row>
     <x:row r="51">
       <x:c r="A51" s="1" t="s">
-        <x:v>89</x:v>
+        <x:v>87</x:v>
       </x:c>
       <x:c r="B51" s="1" t="s">
-        <x:v>81</x:v>
+        <x:v>79</x:v>
       </x:c>
       <x:c r="C51" s="1" t="s">
         <x:v>41</x:v>
@@ -3529,7 +3523,7 @@
     </x:row>
     <x:row r="52">
       <x:c r="A52" s="1" t="s">
-        <x:v>90</x:v>
+        <x:v>88</x:v>
       </x:c>
       <x:c r="B52" s="1" t="s">
         <x:v>19</x:v>
@@ -3539,7 +3533,7 @@
     </x:row>
     <x:row r="53">
       <x:c r="A53" s="1" t="s">
-        <x:v>91</x:v>
+        <x:v>89</x:v>
       </x:c>
       <x:c r="B53" s="1" t="s">
         <x:v>19</x:v>
@@ -3549,7 +3543,7 @@
     </x:row>
     <x:row r="54">
       <x:c r="A54" s="1" t="s">
-        <x:v>92</x:v>
+        <x:v>90</x:v>
       </x:c>
       <x:c r="B54" s="1" t="s">
         <x:v>19</x:v>
@@ -3559,20 +3553,20 @@
     </x:row>
     <x:row r="55">
       <x:c r="A55" s="1" t="s">
-        <x:v>93</x:v>
+        <x:v>91</x:v>
       </x:c>
       <x:c r="B55" s="1" t="s">
-        <x:v>94</x:v>
+        <x:v>92</x:v>
       </x:c>
       <x:c r="H55" s="5"/>
       <x:c r="I55" s="5"/>
     </x:row>
     <x:row r="56">
       <x:c r="A56" s="1" t="s">
-        <x:v>95</x:v>
+        <x:v>93</x:v>
       </x:c>
       <x:c r="B56" s="1" t="s">
-        <x:v>96</x:v>
+        <x:v>94</x:v>
       </x:c>
       <x:c r="C56" s="1" t="s">
         <x:v>41</x:v>
@@ -3595,33 +3589,33 @@
     </x:row>
     <x:row r="57">
       <x:c r="A57" s="1" t="s">
-        <x:v>97</x:v>
+        <x:v>95</x:v>
       </x:c>
       <x:c r="B57" s="1" t="s">
-        <x:v>94</x:v>
+        <x:v>92</x:v>
       </x:c>
       <x:c r="C57" s="1" t="s">
         <x:v>41</x:v>
       </x:c>
       <x:c r="D57" s="1" t="s">
-        <x:v>98</x:v>
+        <x:v>96</x:v>
       </x:c>
       <x:c r="E57" s="1" t="s">
-        <x:v>98</x:v>
+        <x:v>96</x:v>
       </x:c>
       <x:c r="H57" s="5" t="s">
-        <x:v>73</x:v>
+        <x:v>71</x:v>
       </x:c>
       <x:c r="I57" s="5" t="s">
-        <x:v>73</x:v>
+        <x:v>71</x:v>
       </x:c>
     </x:row>
     <x:row r="58">
       <x:c r="A58" s="1" t="s">
-        <x:v>99</x:v>
+        <x:v>97</x:v>
       </x:c>
       <x:c r="B58" s="1" t="s">
-        <x:v>96</x:v>
+        <x:v>94</x:v>
       </x:c>
       <x:c r="C58" s="1" t="s">
         <x:v>41</x:v>
@@ -3644,33 +3638,33 @@
     </x:row>
     <x:row r="59">
       <x:c r="A59" s="1" t="s">
-        <x:v>100</x:v>
+        <x:v>98</x:v>
       </x:c>
       <x:c r="B59" s="1" t="s">
-        <x:v>94</x:v>
+        <x:v>92</x:v>
       </x:c>
       <x:c r="C59" s="1" t="s">
         <x:v>41</x:v>
       </x:c>
       <x:c r="D59" s="1" t="s">
-        <x:v>98</x:v>
+        <x:v>96</x:v>
       </x:c>
       <x:c r="E59" s="1" t="s">
-        <x:v>98</x:v>
+        <x:v>96</x:v>
       </x:c>
       <x:c r="H59" s="5" t="s">
-        <x:v>73</x:v>
+        <x:v>71</x:v>
       </x:c>
       <x:c r="I59" s="5" t="s">
-        <x:v>73</x:v>
+        <x:v>71</x:v>
       </x:c>
     </x:row>
     <x:row r="60">
       <x:c r="A60" s="1" t="s">
-        <x:v>101</x:v>
+        <x:v>99</x:v>
       </x:c>
       <x:c r="B60" s="1" t="s">
-        <x:v>96</x:v>
+        <x:v>94</x:v>
       </x:c>
       <x:c r="C60" s="1" t="s">
         <x:v>41</x:v>
@@ -3693,10 +3687,10 @@
     </x:row>
     <x:row r="61">
       <x:c r="A61" s="1" t="s">
-        <x:v>102</x:v>
+        <x:v>100</x:v>
       </x:c>
       <x:c r="B61" s="1" t="s">
-        <x:v>103</x:v>
+        <x:v>101</x:v>
       </x:c>
       <x:c r="C61" s="16" t="s">
         <x:v>27</x:v>
@@ -3719,7 +3713,7 @@
     </x:row>
     <x:row r="62">
       <x:c r="A62" s="1" t="s">
-        <x:v>104</x:v>
+        <x:v>102</x:v>
       </x:c>
       <x:c r="B62" s="1" t="s">
         <x:v>19</x:v>
@@ -3730,10 +3724,10 @@
     </x:row>
     <x:row r="63">
       <x:c r="A63" s="1" t="s">
-        <x:v>105</x:v>
+        <x:v>103</x:v>
       </x:c>
       <x:c r="B63" s="1" t="s">
-        <x:v>106</x:v>
+        <x:v>104</x:v>
       </x:c>
       <x:c r="C63" s="16" t="s">
         <x:v>27</x:v>
@@ -3756,56 +3750,56 @@
     </x:row>
     <x:row r="64">
       <x:c r="A64" s="1" t="s">
-        <x:v>107</x:v>
+        <x:v>105</x:v>
       </x:c>
       <x:c r="B64" s="1" t="s">
-        <x:v>108</x:v>
+        <x:v>106</x:v>
       </x:c>
       <x:c r="C64" s="1" t="s">
         <x:v>41</x:v>
       </x:c>
       <x:c r="D64" s="1" t="s">
-        <x:v>109</x:v>
+        <x:v>107</x:v>
       </x:c>
       <x:c r="E64" s="1" t="s">
-        <x:v>109</x:v>
+        <x:v>107</x:v>
       </x:c>
       <x:c r="H64" s="5" t="s">
-        <x:v>73</x:v>
+        <x:v>71</x:v>
       </x:c>
       <x:c r="I64" s="5" t="s">
-        <x:v>73</x:v>
+        <x:v>71</x:v>
       </x:c>
     </x:row>
     <x:row r="65">
       <x:c r="A65" s="1" t="s">
-        <x:v>110</x:v>
+        <x:v>108</x:v>
       </x:c>
       <x:c r="B65" s="1" t="s">
-        <x:v>111</x:v>
+        <x:v>109</x:v>
       </x:c>
       <x:c r="C65" s="1" t="s">
         <x:v>41</x:v>
       </x:c>
       <x:c r="D65" s="1" t="s">
-        <x:v>109</x:v>
+        <x:v>107</x:v>
       </x:c>
       <x:c r="E65" s="1" t="s">
-        <x:v>109</x:v>
+        <x:v>107</x:v>
       </x:c>
       <x:c r="H65" s="5" t="s">
-        <x:v>73</x:v>
+        <x:v>71</x:v>
       </x:c>
       <x:c r="I65" s="5" t="s">
-        <x:v>73</x:v>
+        <x:v>71</x:v>
       </x:c>
     </x:row>
     <x:row r="66">
       <x:c r="A66" s="1" t="s">
-        <x:v>112</x:v>
+        <x:v>110</x:v>
       </x:c>
       <x:c r="B66" s="1" t="s">
-        <x:v>113</x:v>
+        <x:v>111</x:v>
       </x:c>
       <x:c r="C66" s="1" t="s">
         <x:v>41</x:v>
@@ -3828,10 +3822,10 @@
     </x:row>
     <x:row r="67">
       <x:c r="A67" s="1" t="s">
-        <x:v>114</x:v>
+        <x:v>112</x:v>
       </x:c>
       <x:c r="B67" s="1" t="s">
-        <x:v>115</x:v>
+        <x:v>113</x:v>
       </x:c>
       <x:c r="C67" s="1" t="s">
         <x:v>41</x:v>
@@ -3854,10 +3848,10 @@
     </x:row>
     <x:row r="68">
       <x:c r="A68" s="1" t="s">
-        <x:v>116</x:v>
+        <x:v>114</x:v>
       </x:c>
       <x:c r="B68" s="1" t="s">
-        <x:v>117</x:v>
+        <x:v>115</x:v>
       </x:c>
       <x:c r="C68" s="1" t="s">
         <x:v>41</x:v>
@@ -3880,56 +3874,56 @@
     </x:row>
     <x:row r="69">
       <x:c r="A69" s="1" t="s">
-        <x:v>118</x:v>
+        <x:v>116</x:v>
       </x:c>
       <x:c r="B69" s="1" t="s">
-        <x:v>108</x:v>
+        <x:v>106</x:v>
       </x:c>
       <x:c r="C69" s="1" t="s">
         <x:v>41</x:v>
       </x:c>
       <x:c r="D69" s="1" t="s">
-        <x:v>109</x:v>
+        <x:v>107</x:v>
       </x:c>
       <x:c r="E69" s="1" t="s">
-        <x:v>109</x:v>
+        <x:v>107</x:v>
       </x:c>
       <x:c r="H69" s="5" t="s">
-        <x:v>73</x:v>
+        <x:v>71</x:v>
       </x:c>
       <x:c r="I69" s="5" t="s">
-        <x:v>73</x:v>
+        <x:v>71</x:v>
       </x:c>
     </x:row>
     <x:row r="70">
       <x:c r="A70" s="1" t="s">
-        <x:v>119</x:v>
+        <x:v>117</x:v>
       </x:c>
       <x:c r="B70" s="1" t="s">
-        <x:v>111</x:v>
+        <x:v>109</x:v>
       </x:c>
       <x:c r="C70" s="1" t="s">
         <x:v>41</x:v>
       </x:c>
       <x:c r="D70" s="1" t="s">
-        <x:v>109</x:v>
+        <x:v>107</x:v>
       </x:c>
       <x:c r="E70" s="1" t="s">
-        <x:v>109</x:v>
+        <x:v>107</x:v>
       </x:c>
       <x:c r="H70" s="5" t="s">
-        <x:v>73</x:v>
+        <x:v>71</x:v>
       </x:c>
       <x:c r="I70" s="5" t="s">
-        <x:v>73</x:v>
+        <x:v>71</x:v>
       </x:c>
     </x:row>
     <x:row r="71">
       <x:c r="A71" s="1" t="s">
-        <x:v>120</x:v>
+        <x:v>118</x:v>
       </x:c>
       <x:c r="B71" s="1" t="s">
-        <x:v>113</x:v>
+        <x:v>111</x:v>
       </x:c>
       <x:c r="C71" s="1" t="s">
         <x:v>41</x:v>
@@ -3952,10 +3946,10 @@
     </x:row>
     <x:row r="72">
       <x:c r="A72" s="1" t="s">
-        <x:v>121</x:v>
+        <x:v>119</x:v>
       </x:c>
       <x:c r="B72" s="1" t="s">
-        <x:v>115</x:v>
+        <x:v>113</x:v>
       </x:c>
       <x:c r="C72" s="1" t="s">
         <x:v>41</x:v>
@@ -3978,10 +3972,10 @@
     </x:row>
     <x:row r="73">
       <x:c r="A73" s="1" t="s">
-        <x:v>122</x:v>
+        <x:v>120</x:v>
       </x:c>
       <x:c r="B73" s="1" t="s">
-        <x:v>117</x:v>
+        <x:v>115</x:v>
       </x:c>
       <x:c r="C73" s="1" t="s">
         <x:v>41</x:v>
@@ -4004,56 +3998,56 @@
     </x:row>
     <x:row r="74">
       <x:c r="A74" s="1" t="s">
-        <x:v>123</x:v>
+        <x:v>121</x:v>
       </x:c>
       <x:c r="B74" s="1" t="s">
-        <x:v>108</x:v>
+        <x:v>106</x:v>
       </x:c>
       <x:c r="C74" s="1" t="s">
         <x:v>41</x:v>
       </x:c>
       <x:c r="D74" s="1" t="s">
-        <x:v>109</x:v>
+        <x:v>107</x:v>
       </x:c>
       <x:c r="E74" s="1" t="s">
-        <x:v>109</x:v>
+        <x:v>107</x:v>
       </x:c>
       <x:c r="H74" s="5" t="s">
-        <x:v>73</x:v>
+        <x:v>71</x:v>
       </x:c>
       <x:c r="I74" s="5" t="s">
-        <x:v>73</x:v>
+        <x:v>71</x:v>
       </x:c>
     </x:row>
     <x:row r="75">
       <x:c r="A75" s="1" t="s">
-        <x:v>124</x:v>
+        <x:v>122</x:v>
       </x:c>
       <x:c r="B75" s="1" t="s">
-        <x:v>111</x:v>
+        <x:v>109</x:v>
       </x:c>
       <x:c r="C75" s="1" t="s">
         <x:v>41</x:v>
       </x:c>
       <x:c r="D75" s="1" t="s">
-        <x:v>109</x:v>
+        <x:v>107</x:v>
       </x:c>
       <x:c r="E75" s="1" t="s">
-        <x:v>109</x:v>
+        <x:v>107</x:v>
       </x:c>
       <x:c r="H75" s="5" t="s">
-        <x:v>73</x:v>
+        <x:v>71</x:v>
       </x:c>
       <x:c r="I75" s="5" t="s">
-        <x:v>73</x:v>
+        <x:v>71</x:v>
       </x:c>
     </x:row>
     <x:row r="76">
       <x:c r="A76" s="1" t="s">
-        <x:v>125</x:v>
+        <x:v>123</x:v>
       </x:c>
       <x:c r="B76" s="1" t="s">
-        <x:v>113</x:v>
+        <x:v>111</x:v>
       </x:c>
       <x:c r="C76" s="1" t="s">
         <x:v>41</x:v>
@@ -4076,10 +4070,10 @@
     </x:row>
     <x:row r="77">
       <x:c r="A77" s="1" t="s">
-        <x:v>126</x:v>
+        <x:v>124</x:v>
       </x:c>
       <x:c r="B77" s="1" t="s">
-        <x:v>115</x:v>
+        <x:v>113</x:v>
       </x:c>
       <x:c r="C77" s="1" t="s">
         <x:v>41</x:v>
@@ -4102,10 +4096,10 @@
     </x:row>
     <x:row r="78">
       <x:c r="A78" s="1" t="s">
-        <x:v>127</x:v>
+        <x:v>125</x:v>
       </x:c>
       <x:c r="B78" s="1" t="s">
-        <x:v>117</x:v>
+        <x:v>115</x:v>
       </x:c>
       <x:c r="C78" s="1" t="s">
         <x:v>41</x:v>
@@ -7875,7 +7869,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="B1" s="2" t="s">
-        <x:v>423</x:v>
+        <x:v>421</x:v>
       </x:c>
       <x:c r="N1" s="1" t="s">
         <x:v>2</x:v>
@@ -7886,7 +7880,7 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="B2" s="2" t="s">
-        <x:v>424</x:v>
+        <x:v>422</x:v>
       </x:c>
     </x:row>
     <x:row r="3">
@@ -7931,7 +7925,7 @@
         <x:v>18</x:v>
       </x:c>
       <x:c r="D6" s="1" t="s">
-        <x:v>133</x:v>
+        <x:v>131</x:v>
       </x:c>
       <x:c r="E6" s="1" t="s">
         <x:v>28</x:v>
@@ -7939,10 +7933,10 @@
     </x:row>
     <x:row r="7">
       <x:c r="A7" s="1" t="s">
-        <x:v>184</x:v>
+        <x:v>182</x:v>
       </x:c>
       <x:c r="D7" s="1" t="s">
-        <x:v>133</x:v>
+        <x:v>131</x:v>
       </x:c>
       <x:c r="E7" s="1" t="s">
         <x:v>28</x:v>
@@ -7950,10 +7944,10 @@
     </x:row>
     <x:row r="8">
       <x:c r="A8" s="1" t="s">
-        <x:v>180</x:v>
+        <x:v>178</x:v>
       </x:c>
       <x:c r="D8" s="1" t="s">
-        <x:v>133</x:v>
+        <x:v>131</x:v>
       </x:c>
       <x:c r="E8" s="1" t="s">
         <x:v>28</x:v>
@@ -7961,38 +7955,38 @@
     </x:row>
     <x:row r="9">
       <x:c r="A9" s="1" t="s">
-        <x:v>425</x:v>
+        <x:v>423</x:v>
       </x:c>
       <x:c r="D9" s="1" t="s">
-        <x:v>426</x:v>
+        <x:v>424</x:v>
       </x:c>
       <x:c r="E9" s="1" t="s">
-        <x:v>71</x:v>
+        <x:v>69</x:v>
       </x:c>
       <x:c r="F9" s="1" t="s">
-        <x:v>139</x:v>
+        <x:v>137</x:v>
       </x:c>
     </x:row>
     <x:row r="10">
       <x:c r="A10" s="1" t="s">
-        <x:v>427</x:v>
+        <x:v>425</x:v>
       </x:c>
       <x:c r="D10" s="1" t="s">
-        <x:v>428</x:v>
+        <x:v>426</x:v>
       </x:c>
       <x:c r="E10" s="1" t="s">
-        <x:v>71</x:v>
+        <x:v>69</x:v>
       </x:c>
       <x:c r="F10" s="1" t="s">
-        <x:v>139</x:v>
+        <x:v>137</x:v>
       </x:c>
     </x:row>
     <x:row r="11">
       <x:c r="A11" s="1" t="s">
-        <x:v>164</x:v>
+        <x:v>162</x:v>
       </x:c>
       <x:c r="D11" s="1" t="s">
-        <x:v>133</x:v>
+        <x:v>131</x:v>
       </x:c>
       <x:c r="E11" s="1" t="s">
         <x:v>28</x:v>
@@ -8000,21 +7994,21 @@
     </x:row>
     <x:row r="12">
       <x:c r="A12" s="1" t="s">
-        <x:v>66</x:v>
+        <x:v>64</x:v>
       </x:c>
       <x:c r="D12" s="1" t="s">
-        <x:v>109</x:v>
+        <x:v>107</x:v>
       </x:c>
       <x:c r="E12" s="1" t="s">
-        <x:v>109</x:v>
+        <x:v>107</x:v>
       </x:c>
     </x:row>
     <x:row r="13">
       <x:c r="A13" s="1" t="s">
-        <x:v>167</x:v>
+        <x:v>165</x:v>
       </x:c>
       <x:c r="D13" s="1" t="s">
-        <x:v>133</x:v>
+        <x:v>131</x:v>
       </x:c>
       <x:c r="E13" s="1" t="s">
         <x:v>28</x:v>
@@ -8022,35 +8016,35 @@
     </x:row>
     <x:row r="14">
       <x:c r="A14" s="1" t="s">
-        <x:v>169</x:v>
+        <x:v>167</x:v>
       </x:c>
       <x:c r="D14" s="1" t="s">
-        <x:v>109</x:v>
+        <x:v>107</x:v>
       </x:c>
       <x:c r="E14" s="1" t="s">
-        <x:v>109</x:v>
+        <x:v>107</x:v>
       </x:c>
     </x:row>
     <x:row r="15">
       <x:c r="A15" s="1" t="s">
-        <x:v>429</x:v>
+        <x:v>427</x:v>
       </x:c>
       <x:c r="D15" s="1" t="s">
-        <x:v>430</x:v>
+        <x:v>428</x:v>
       </x:c>
       <x:c r="E15" s="1" t="s">
-        <x:v>71</x:v>
+        <x:v>69</x:v>
       </x:c>
       <x:c r="F15" s="1" t="s">
-        <x:v>139</x:v>
+        <x:v>137</x:v>
       </x:c>
     </x:row>
     <x:row r="16">
       <x:c r="A16" s="1" t="s">
-        <x:v>431</x:v>
+        <x:v>429</x:v>
       </x:c>
       <x:c r="D16" s="1" t="s">
-        <x:v>197</x:v>
+        <x:v>195</x:v>
       </x:c>
       <x:c r="E16" s="1" t="s">
         <x:v>28</x:v>
@@ -8058,13 +8052,13 @@
     </x:row>
     <x:row r="17">
       <x:c r="A17" s="1" t="s">
-        <x:v>432</x:v>
+        <x:v>430</x:v>
       </x:c>
       <x:c r="D17" s="1" t="s">
-        <x:v>109</x:v>
+        <x:v>107</x:v>
       </x:c>
       <x:c r="E17" s="1" t="s">
-        <x:v>109</x:v>
+        <x:v>107</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -8103,7 +8097,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="B1" s="2" t="s">
-        <x:v>433</x:v>
+        <x:v>431</x:v>
       </x:c>
       <x:c r="F1" s="4"/>
       <x:c r="G1" s="4"/>
@@ -8114,7 +8108,7 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="B2" s="2" t="s">
-        <x:v>434</x:v>
+        <x:v>432</x:v>
       </x:c>
       <x:c r="F2" s="4"/>
       <x:c r="G2" s="4"/>
@@ -8170,88 +8164,88 @@
         <x:v>18</x:v>
       </x:c>
       <x:c r="D6" s="1" t="s">
-        <x:v>133</x:v>
+        <x:v>131</x:v>
       </x:c>
       <x:c r="E6" s="1" t="s">
         <x:v>28</x:v>
       </x:c>
       <x:c r="F6" s="1" t="s">
-        <x:v>435</x:v>
+        <x:v>433</x:v>
       </x:c>
     </x:row>
     <x:row r="7">
       <x:c r="A7" s="1" t="s">
-        <x:v>164</x:v>
+        <x:v>162</x:v>
       </x:c>
       <x:c r="D7" s="1" t="s">
-        <x:v>133</x:v>
+        <x:v>131</x:v>
       </x:c>
       <x:c r="E7" s="1" t="s">
         <x:v>28</x:v>
       </x:c>
       <x:c r="F7" s="1" t="s">
-        <x:v>435</x:v>
+        <x:v>433</x:v>
       </x:c>
     </x:row>
     <x:row r="8">
       <x:c r="A8" s="1" t="s">
-        <x:v>66</x:v>
+        <x:v>64</x:v>
       </x:c>
       <x:c r="D8" s="1" t="s">
-        <x:v>109</x:v>
+        <x:v>107</x:v>
       </x:c>
       <x:c r="E8" s="1" t="s">
-        <x:v>109</x:v>
+        <x:v>107</x:v>
       </x:c>
       <x:c r="F8" s="1" t="s">
-        <x:v>435</x:v>
+        <x:v>433</x:v>
       </x:c>
     </x:row>
     <x:row r="9">
       <x:c r="A9" s="1" t="s">
-        <x:v>167</x:v>
+        <x:v>165</x:v>
       </x:c>
       <x:c r="D9" s="1" t="s">
-        <x:v>133</x:v>
+        <x:v>131</x:v>
       </x:c>
       <x:c r="E9" s="1" t="s">
         <x:v>28</x:v>
       </x:c>
       <x:c r="F9" s="1" t="s">
-        <x:v>435</x:v>
+        <x:v>433</x:v>
       </x:c>
     </x:row>
     <x:row r="10">
       <x:c r="A10" s="1" t="s">
-        <x:v>169</x:v>
+        <x:v>167</x:v>
       </x:c>
       <x:c r="D10" s="1" t="s">
-        <x:v>109</x:v>
+        <x:v>107</x:v>
       </x:c>
       <x:c r="E10" s="1" t="s">
-        <x:v>109</x:v>
+        <x:v>107</x:v>
       </x:c>
       <x:c r="F10" s="1" t="s">
-        <x:v>435</x:v>
+        <x:v>433</x:v>
       </x:c>
     </x:row>
     <x:row r="11">
       <x:c r="A11" s="1" t="s">
-        <x:v>180</x:v>
+        <x:v>178</x:v>
       </x:c>
       <x:c r="D11" s="1" t="s">
-        <x:v>133</x:v>
+        <x:v>131</x:v>
       </x:c>
       <x:c r="E11" s="1" t="s">
         <x:v>28</x:v>
       </x:c>
       <x:c r="F11" s="1" t="s">
-        <x:v>435</x:v>
+        <x:v>433</x:v>
       </x:c>
     </x:row>
     <x:row r="12">
       <x:c r="A12" s="1" t="s">
-        <x:v>436</x:v>
+        <x:v>434</x:v>
       </x:c>
       <x:c r="D12" s="1" t="s">
         <x:v>28</x:v>
@@ -8260,12 +8254,12 @@
         <x:v>28</x:v>
       </x:c>
       <x:c r="F12" s="1" t="s">
-        <x:v>435</x:v>
+        <x:v>433</x:v>
       </x:c>
     </x:row>
     <x:row r="13">
       <x:c r="A13" s="1" t="s">
-        <x:v>437</x:v>
+        <x:v>435</x:v>
       </x:c>
       <x:c r="D13" s="1" t="s">
         <x:v>28</x:v>
@@ -8274,12 +8268,12 @@
         <x:v>28</x:v>
       </x:c>
       <x:c r="F13" s="1" t="s">
-        <x:v>435</x:v>
+        <x:v>433</x:v>
       </x:c>
     </x:row>
     <x:row r="14">
       <x:c r="A14" s="1" t="s">
-        <x:v>438</x:v>
+        <x:v>436</x:v>
       </x:c>
       <x:c r="D14" s="1" t="s">
         <x:v>28</x:v>
@@ -8288,12 +8282,12 @@
         <x:v>28</x:v>
       </x:c>
       <x:c r="F14" s="1" t="s">
-        <x:v>435</x:v>
+        <x:v>433</x:v>
       </x:c>
     </x:row>
     <x:row r="15">
       <x:c r="A15" s="1" t="s">
-        <x:v>439</x:v>
+        <x:v>437</x:v>
       </x:c>
       <x:c r="D15" s="1" t="s">
         <x:v>28</x:v>
@@ -8302,12 +8296,12 @@
         <x:v>28</x:v>
       </x:c>
       <x:c r="F15" s="1" t="s">
-        <x:v>435</x:v>
+        <x:v>433</x:v>
       </x:c>
     </x:row>
     <x:row r="16">
       <x:c r="A16" s="1" t="s">
-        <x:v>440</x:v>
+        <x:v>438</x:v>
       </x:c>
       <x:c r="D16" s="1" t="s">
         <x:v>28</x:v>
@@ -8316,12 +8310,12 @@
         <x:v>28</x:v>
       </x:c>
       <x:c r="F16" s="1" t="s">
-        <x:v>435</x:v>
+        <x:v>433</x:v>
       </x:c>
     </x:row>
     <x:row r="17">
       <x:c r="A17" s="1" t="s">
-        <x:v>441</x:v>
+        <x:v>439</x:v>
       </x:c>
       <x:c r="D17" s="1" t="s">
         <x:v>28</x:v>
@@ -8330,12 +8324,12 @@
         <x:v>28</x:v>
       </x:c>
       <x:c r="F17" s="1" t="s">
-        <x:v>435</x:v>
+        <x:v>433</x:v>
       </x:c>
     </x:row>
     <x:row r="18">
       <x:c r="A18" s="1" t="s">
-        <x:v>442</x:v>
+        <x:v>440</x:v>
       </x:c>
       <x:c r="D18" s="1" t="s">
         <x:v>28</x:v>
@@ -8344,7 +8338,7 @@
         <x:v>28</x:v>
       </x:c>
       <x:c r="F18" s="1" t="s">
-        <x:v>435</x:v>
+        <x:v>433</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -8380,7 +8374,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="B1" s="2" t="s">
-        <x:v>443</x:v>
+        <x:v>441</x:v>
       </x:c>
       <x:c r="M1" s="1" t="s">
         <x:v>2</x:v>
@@ -8391,7 +8385,7 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="B2" s="2" t="s">
-        <x:v>444</x:v>
+        <x:v>442</x:v>
       </x:c>
     </x:row>
     <x:row r="3">
@@ -8436,7 +8430,7 @@
         <x:v>18</x:v>
       </x:c>
       <x:c r="D6" s="1" t="s">
-        <x:v>133</x:v>
+        <x:v>131</x:v>
       </x:c>
       <x:c r="E6" s="1" t="s">
         <x:v>28</x:v>
@@ -8444,7 +8438,7 @@
     </x:row>
     <x:row r="7">
       <x:c r="A7" s="1" t="s">
-        <x:v>445</x:v>
+        <x:v>443</x:v>
       </x:c>
       <x:c r="D7" s="1" t="s">
         <x:v>28</x:v>
@@ -8455,38 +8449,38 @@
     </x:row>
     <x:row r="8">
       <x:c r="A8" s="1" t="s">
-        <x:v>425</x:v>
+        <x:v>423</x:v>
       </x:c>
       <x:c r="D8" s="1" t="s">
-        <x:v>426</x:v>
+        <x:v>424</x:v>
       </x:c>
       <x:c r="E8" s="1" t="s">
-        <x:v>71</x:v>
+        <x:v>69</x:v>
       </x:c>
       <x:c r="F8" s="1" t="s">
-        <x:v>139</x:v>
+        <x:v>137</x:v>
       </x:c>
     </x:row>
     <x:row r="9">
       <x:c r="A9" s="1" t="s">
-        <x:v>427</x:v>
+        <x:v>425</x:v>
       </x:c>
       <x:c r="D9" s="1" t="s">
-        <x:v>428</x:v>
+        <x:v>426</x:v>
       </x:c>
       <x:c r="E9" s="1" t="s">
-        <x:v>71</x:v>
+        <x:v>69</x:v>
       </x:c>
       <x:c r="F9" s="1" t="s">
-        <x:v>139</x:v>
+        <x:v>137</x:v>
       </x:c>
     </x:row>
     <x:row r="10">
       <x:c r="A10" s="1" t="s">
-        <x:v>180</x:v>
+        <x:v>178</x:v>
       </x:c>
       <x:c r="D10" s="1" t="s">
-        <x:v>133</x:v>
+        <x:v>131</x:v>
       </x:c>
       <x:c r="E10" s="1" t="s">
         <x:v>28</x:v>
@@ -8494,10 +8488,10 @@
     </x:row>
     <x:row r="11">
       <x:c r="A11" s="1" t="s">
-        <x:v>446</x:v>
+        <x:v>444</x:v>
       </x:c>
       <x:c r="D11" s="1" t="s">
-        <x:v>133</x:v>
+        <x:v>131</x:v>
       </x:c>
       <x:c r="E11" s="1" t="s">
         <x:v>28</x:v>
@@ -8505,10 +8499,10 @@
     </x:row>
     <x:row r="12">
       <x:c r="A12" s="1" t="s">
-        <x:v>164</x:v>
+        <x:v>162</x:v>
       </x:c>
       <x:c r="D12" s="1" t="s">
-        <x:v>133</x:v>
+        <x:v>131</x:v>
       </x:c>
       <x:c r="E12" s="1" t="s">
         <x:v>28</x:v>
@@ -8516,21 +8510,21 @@
     </x:row>
     <x:row r="13">
       <x:c r="A13" s="1" t="s">
-        <x:v>66</x:v>
+        <x:v>64</x:v>
       </x:c>
       <x:c r="D13" s="1" t="s">
-        <x:v>109</x:v>
+        <x:v>107</x:v>
       </x:c>
       <x:c r="E13" s="1" t="s">
-        <x:v>109</x:v>
+        <x:v>107</x:v>
       </x:c>
     </x:row>
     <x:row r="14">
       <x:c r="A14" s="1" t="s">
-        <x:v>167</x:v>
+        <x:v>165</x:v>
       </x:c>
       <x:c r="D14" s="1" t="s">
-        <x:v>133</x:v>
+        <x:v>131</x:v>
       </x:c>
       <x:c r="E14" s="1" t="s">
         <x:v>28</x:v>
@@ -8538,27 +8532,27 @@
     </x:row>
     <x:row r="15">
       <x:c r="A15" s="1" t="s">
-        <x:v>169</x:v>
+        <x:v>167</x:v>
       </x:c>
       <x:c r="D15" s="1" t="s">
-        <x:v>109</x:v>
+        <x:v>107</x:v>
       </x:c>
       <x:c r="E15" s="1" t="s">
-        <x:v>109</x:v>
+        <x:v>107</x:v>
       </x:c>
     </x:row>
     <x:row r="16">
       <x:c r="A16" s="1" t="s">
-        <x:v>447</x:v>
+        <x:v>445</x:v>
       </x:c>
       <x:c r="D16" s="1" t="s">
-        <x:v>447</x:v>
+        <x:v>445</x:v>
       </x:c>
       <x:c r="E16" s="1" t="s">
-        <x:v>71</x:v>
+        <x:v>69</x:v>
       </x:c>
       <x:c r="F16" s="1" t="s">
-        <x:v>139</x:v>
+        <x:v>137</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -8923,12 +8917,12 @@
         <x:v>00-stage-business-cases.m; 05-create-business-cases-and-solutions.m</x:v>
       </x:c>
       <x:c r="D19" s="42" t="str">
-        <x:v>DEV validation: 57 Business Case rows; UnmappedIssues blank for all rows. Business Case solution preparation and final output each contain 171 rows (3 per Business Case); BusinessCaseSolutionQA=0. Golden Business Case 00f054be-25d8-455f-8cdc-67180f9fd068 verified flattened Request fields, Preferred Solution data, three Solution types, Request relationships, batch IDs, and Estimated Lifecycle Cost association. Confirmed Request fields: new_organizationalpriorityalignment, new_businessoruserneed, new_currentprocess, new_howwillcmsbenefit, and new_successcriteria. Mappings for new_internalorexternalsupportneeded and new_grt_feedback_implementation are configured but could not be exercised because the DEV export contains no source values. The DEV export also contains no populated Alternative A/B fields and only OPEN status values. Follow-up: build a richer UAT dataset after SharePoint write access is granted; verify Alternative A/B, additional statuses, the two unexercised Request fields, rerun duplicate safety, and whether staging retention is sufficient for historical requester EUA attribution.</x:v>
+        <x:v>DEV validation: 57 Business Case rows; UnmappedIssues blank for all rows. Business Case solution preparation and final output each contain 171 rows (3 per Business Case); BusinessCaseSolutionQA=0. Golden Request 1a261eb8-162d-46a6-afaf-b5c9507dedd1 verified flattened Request fields, three related Solution types, batch IDs, and solution details. Confirmed Request fields include new_organizationalpriorityalignment, new_businessoruserneed, new_currentprocess, new_howwillcmsbenefit, new_successcriteria, new_internalorexternalsupportneeded, and new_grt_feedback_implementation. OPEN, sparse DRAFT, and CLOSED Business Case statuses migrated correctly. Preferred, Alternative A, and Alternative B verified Target Contract Award, Target Completion, Summary, Pros, Has UI, Zero Trust, workforce training requirements, Cons, and Acquisition Approach. Cons values: Adds complexity to the current application; Longest procurement timeline and highest transition effort; Requires coordination with the enterprise platform team. Acquisition Approach values: Use the current delivery contract; Run a competitive procurement; Use an existing enterprise contract.</x:v>
       </x:c>
       <x:c r="E19" s="42" t="str"/>
       <x:c r="F19" s="42" t="str"/>
       <x:c r="G19" s="68" t="n">
-        <x:v>46262.75</x:v>
+        <x:v>46287</x:v>
       </x:c>
       <x:c r="H19" s="39"/>
       <x:c r="I19" s="39"/>
@@ -9235,7 +9229,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="B1" s="1" t="s">
-        <x:v>128</x:v>
+        <x:v>126</x:v>
       </x:c>
       <x:c r="H1" s="3"/>
       <x:c r="I1" s="3"/>
@@ -9245,7 +9239,7 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="B2" s="1" t="s">
-        <x:v>129</x:v>
+        <x:v>127</x:v>
       </x:c>
       <x:c r="H2" s="3"/>
       <x:c r="I2" s="3"/>
@@ -9291,7 +9285,7 @@
         <x:v>12</x:v>
       </x:c>
       <x:c r="F6" s="6" t="s">
-        <x:v>130</x:v>
+        <x:v>128</x:v>
       </x:c>
       <x:c r="G6" s="6" t="s">
         <x:v>14</x:v>
@@ -9314,13 +9308,13 @@
         <x:v>18</x:v>
       </x:c>
       <x:c r="B7" s="1" t="s">
+        <x:v>129</x:v>
+      </x:c>
+      <x:c r="C7" s="1" t="s">
+        <x:v>130</x:v>
+      </x:c>
+      <x:c r="D7" s="1" t="s">
         <x:v>131</x:v>
-      </x:c>
-      <x:c r="C7" s="1" t="s">
-        <x:v>132</x:v>
-      </x:c>
-      <x:c r="D7" s="1" t="s">
-        <x:v>133</x:v>
       </x:c>
       <x:c r="E7" s="1" t="s">
         <x:v>28</x:v>
@@ -9334,16 +9328,16 @@
     </x:row>
     <x:row r="8">
       <x:c r="A8" s="1" t="s">
-        <x:v>134</x:v>
+        <x:v>132</x:v>
       </x:c>
       <x:c r="B8" s="1" t="s">
+        <x:v>129</x:v>
+      </x:c>
+      <x:c r="C8" s="1" t="s">
+        <x:v>133</x:v>
+      </x:c>
+      <x:c r="D8" s="1" t="s">
         <x:v>131</x:v>
-      </x:c>
-      <x:c r="C8" s="1" t="s">
-        <x:v>135</x:v>
-      </x:c>
-      <x:c r="D8" s="1" t="s">
-        <x:v>133</x:v>
       </x:c>
       <x:c r="E8" s="1" t="s">
         <x:v>28</x:v>
@@ -9357,68 +9351,68 @@
     </x:row>
     <x:row r="9">
       <x:c r="A9" s="1" t="s">
+        <x:v>134</x:v>
+      </x:c>
+      <x:c r="B9" s="1" t="s">
+        <x:v>129</x:v>
+      </x:c>
+      <x:c r="C9" s="1" t="s">
+        <x:v>135</x:v>
+      </x:c>
+      <x:c r="D9" s="1" t="s">
         <x:v>136</x:v>
       </x:c>
-      <x:c r="B9" s="1" t="s">
-        <x:v>131</x:v>
-      </x:c>
-      <x:c r="C9" s="1" t="s">
+      <x:c r="E9" s="1" t="s">
+        <x:v>69</x:v>
+      </x:c>
+      <x:c r="F9" s="1" t="s">
         <x:v>137</x:v>
       </x:c>
-      <x:c r="D9" s="1" t="s">
-        <x:v>138</x:v>
-      </x:c>
-      <x:c r="E9" s="1" t="s">
+      <x:c r="H9" s="14" t="s">
         <x:v>71</x:v>
       </x:c>
-      <x:c r="F9" s="1" t="s">
-        <x:v>139</x:v>
-      </x:c>
-      <x:c r="H9" s="14" t="s">
-        <x:v>73</x:v>
-      </x:c>
       <x:c r="I9" s="14" t="s">
-        <x:v>73</x:v>
+        <x:v>71</x:v>
       </x:c>
     </x:row>
     <x:row r="10">
       <x:c r="A10" s="1" t="s">
+        <x:v>138</x:v>
+      </x:c>
+      <x:c r="B10" s="1" t="s">
+        <x:v>129</x:v>
+      </x:c>
+      <x:c r="C10" s="1" t="s">
+        <x:v>139</x:v>
+      </x:c>
+      <x:c r="D10" s="1" t="s">
         <x:v>140</x:v>
       </x:c>
-      <x:c r="B10" s="1" t="s">
-        <x:v>131</x:v>
-      </x:c>
-      <x:c r="C10" s="1" t="s">
-        <x:v>141</x:v>
-      </x:c>
-      <x:c r="D10" s="1" t="s">
-        <x:v>142</x:v>
-      </x:c>
       <x:c r="E10" s="1" t="s">
+        <x:v>69</x:v>
+      </x:c>
+      <x:c r="F10" s="1" t="s">
+        <x:v>137</x:v>
+      </x:c>
+      <x:c r="H10" s="5" t="s">
         <x:v>71</x:v>
       </x:c>
-      <x:c r="F10" s="1" t="s">
-        <x:v>139</x:v>
-      </x:c>
-      <x:c r="H10" s="5" t="s">
-        <x:v>73</x:v>
-      </x:c>
       <x:c r="I10" s="5" t="s">
-        <x:v>73</x:v>
+        <x:v>71</x:v>
       </x:c>
     </x:row>
     <x:row r="11">
       <x:c r="A11" s="1" t="s">
+        <x:v>141</x:v>
+      </x:c>
+      <x:c r="B11" s="1" t="s">
+        <x:v>129</x:v>
+      </x:c>
+      <x:c r="C11" s="1" t="s">
+        <x:v>142</x:v>
+      </x:c>
+      <x:c r="D11" s="1" t="s">
         <x:v>143</x:v>
-      </x:c>
-      <x:c r="B11" s="1" t="s">
-        <x:v>131</x:v>
-      </x:c>
-      <x:c r="C11" s="1" t="s">
-        <x:v>144</x:v>
-      </x:c>
-      <x:c r="D11" s="1" t="s">
-        <x:v>145</x:v>
       </x:c>
       <x:c r="E11" s="1" t="s">
         <x:v>28</x:v>
@@ -9432,22 +9426,22 @@
     </x:row>
     <x:row r="12">
       <x:c r="A12" s="1" t="s">
+        <x:v>144</x:v>
+      </x:c>
+      <x:c r="B12" s="1" t="s">
+        <x:v>129</x:v>
+      </x:c>
+      <x:c r="C12" s="1" t="s">
+        <x:v>145</x:v>
+      </x:c>
+      <x:c r="D12" s="1" t="s">
         <x:v>146</x:v>
       </x:c>
-      <x:c r="B12" s="1" t="s">
-        <x:v>131</x:v>
-      </x:c>
-      <x:c r="C12" s="1" t="s">
-        <x:v>147</x:v>
-      </x:c>
-      <x:c r="D12" s="1" t="s">
-        <x:v>148</x:v>
-      </x:c>
       <x:c r="E12" s="1" t="s">
-        <x:v>71</x:v>
+        <x:v>69</x:v>
       </x:c>
       <x:c r="F12" s="1" t="s">
-        <x:v>139</x:v>
+        <x:v>137</x:v>
       </x:c>
       <x:c r="H12" s="5">
         <x:v>100.0</x:v>
@@ -13460,7 +13454,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="B1" s="1" t="s">
-        <x:v>149</x:v>
+        <x:v>147</x:v>
       </x:c>
       <x:c r="H1" s="3"/>
       <x:c r="I1" s="3"/>
@@ -13473,7 +13467,7 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="B2" s="1" t="s">
-        <x:v>150</x:v>
+        <x:v>148</x:v>
       </x:c>
       <x:c r="H2" s="3"/>
       <x:c r="I2" s="3"/>
@@ -13483,7 +13477,7 @@
         <x:v>5</x:v>
       </x:c>
       <x:c r="B3" s="1" t="s">
-        <x:v>151</x:v>
+        <x:v>149</x:v>
       </x:c>
       <x:c r="I3" s="3"/>
     </x:row>
@@ -13512,7 +13506,7 @@
         <x:v>12</x:v>
       </x:c>
       <x:c r="F6" s="6" t="s">
-        <x:v>130</x:v>
+        <x:v>128</x:v>
       </x:c>
       <x:c r="G6" s="6" t="s">
         <x:v>14</x:v>
@@ -13535,13 +13529,13 @@
         <x:v>18</x:v>
       </x:c>
       <x:c r="B7" s="1" t="s">
-        <x:v>152</x:v>
+        <x:v>150</x:v>
       </x:c>
       <x:c r="C7" s="1" t="s">
-        <x:v>153</x:v>
+        <x:v>151</x:v>
       </x:c>
       <x:c r="D7" s="1" t="s">
-        <x:v>133</x:v>
+        <x:v>131</x:v>
       </x:c>
       <x:c r="E7" s="1" t="s">
         <x:v>28</x:v>
@@ -13555,16 +13549,16 @@
     </x:row>
     <x:row r="8">
       <x:c r="A8" s="1" t="s">
-        <x:v>154</x:v>
+        <x:v>152</x:v>
       </x:c>
       <x:c r="B8" s="1" t="s">
-        <x:v>152</x:v>
+        <x:v>150</x:v>
       </x:c>
       <x:c r="C8" s="1" t="s">
-        <x:v>155</x:v>
+        <x:v>153</x:v>
       </x:c>
       <x:c r="D8" s="1" t="s">
-        <x:v>133</x:v>
+        <x:v>131</x:v>
       </x:c>
       <x:c r="E8" s="1" t="s">
         <x:v>28</x:v>
@@ -13573,18 +13567,18 @@
         <x:v>100.0</x:v>
       </x:c>
       <x:c r="I8" s="5" t="s">
-        <x:v>73</x:v>
+        <x:v>71</x:v>
       </x:c>
     </x:row>
     <x:row r="9">
       <x:c r="A9" s="1" t="s">
-        <x:v>156</x:v>
+        <x:v>154</x:v>
       </x:c>
       <x:c r="B9" s="1" t="s">
-        <x:v>152</x:v>
+        <x:v>150</x:v>
       </x:c>
       <x:c r="C9" s="1" t="s">
-        <x:v>157</x:v>
+        <x:v>155</x:v>
       </x:c>
       <x:c r="D9" s="1" t="s">
         <x:v>28</x:v>
@@ -13601,65 +13595,65 @@
     </x:row>
     <x:row r="10">
       <x:c r="A10" s="1" t="s">
+        <x:v>156</x:v>
+      </x:c>
+      <x:c r="B10" s="1" t="s">
+        <x:v>150</x:v>
+      </x:c>
+      <x:c r="C10" s="1" t="s">
+        <x:v>157</x:v>
+      </x:c>
+      <x:c r="D10" s="1" t="s">
         <x:v>158</x:v>
       </x:c>
-      <x:c r="B10" s="1" t="s">
-        <x:v>152</x:v>
-      </x:c>
-      <x:c r="C10" s="1" t="s">
-        <x:v>159</x:v>
-      </x:c>
-      <x:c r="D10" s="1" t="s">
-        <x:v>160</x:v>
-      </x:c>
       <x:c r="E10" s="1" t="s">
-        <x:v>71</x:v>
+        <x:v>69</x:v>
       </x:c>
       <x:c r="F10" s="1" t="s">
-        <x:v>139</x:v>
+        <x:v>137</x:v>
       </x:c>
       <x:c r="H10" s="5">
         <x:v>100.0</x:v>
       </x:c>
       <x:c r="I10" s="5" t="s">
-        <x:v>73</x:v>
+        <x:v>71</x:v>
       </x:c>
     </x:row>
     <x:row r="11">
       <x:c r="A11" s="1" t="s">
+        <x:v>159</x:v>
+      </x:c>
+      <x:c r="B11" s="1" t="s">
+        <x:v>150</x:v>
+      </x:c>
+      <x:c r="C11" s="1" t="s">
+        <x:v>160</x:v>
+      </x:c>
+      <x:c r="D11" s="1" t="s">
         <x:v>161</x:v>
       </x:c>
-      <x:c r="B11" s="1" t="s">
-        <x:v>152</x:v>
-      </x:c>
-      <x:c r="C11" s="1" t="s">
-        <x:v>162</x:v>
-      </x:c>
-      <x:c r="D11" s="1" t="s">
-        <x:v>163</x:v>
-      </x:c>
       <x:c r="E11" s="1" t="s">
-        <x:v>71</x:v>
+        <x:v>69</x:v>
       </x:c>
       <x:c r="F11" s="1" t="s">
-        <x:v>139</x:v>
+        <x:v>137</x:v>
       </x:c>
       <x:c r="H11" s="5">
         <x:v>100.0</x:v>
       </x:c>
       <x:c r="I11" s="5" t="s">
-        <x:v>73</x:v>
+        <x:v>71</x:v>
       </x:c>
     </x:row>
     <x:row r="12">
       <x:c r="A12" s="1" t="s">
-        <x:v>164</x:v>
+        <x:v>162</x:v>
       </x:c>
       <x:c r="B12" s="1" t="s">
-        <x:v>152</x:v>
+        <x:v>150</x:v>
       </x:c>
       <x:c r="C12" s="1" t="s">
-        <x:v>165</x:v>
+        <x:v>163</x:v>
       </x:c>
       <x:c r="D12" s="1" t="s">
         <x:v>28</x:v>
@@ -13676,36 +13670,36 @@
     </x:row>
     <x:row r="13">
       <x:c r="A13" s="1" t="s">
-        <x:v>66</x:v>
+        <x:v>64</x:v>
       </x:c>
       <x:c r="B13" s="1" t="s">
-        <x:v>152</x:v>
+        <x:v>150</x:v>
       </x:c>
       <x:c r="C13" s="1" t="s">
-        <x:v>166</x:v>
+        <x:v>164</x:v>
       </x:c>
       <x:c r="D13" s="1" t="s">
-        <x:v>109</x:v>
+        <x:v>107</x:v>
       </x:c>
       <x:c r="E13" s="1" t="s">
-        <x:v>109</x:v>
+        <x:v>107</x:v>
       </x:c>
       <x:c r="H13" s="5" t="s">
-        <x:v>73</x:v>
+        <x:v>71</x:v>
       </x:c>
       <x:c r="I13" s="5" t="s">
-        <x:v>73</x:v>
+        <x:v>71</x:v>
       </x:c>
     </x:row>
     <x:row r="14">
       <x:c r="A14" s="1" t="s">
-        <x:v>167</x:v>
+        <x:v>165</x:v>
       </x:c>
       <x:c r="B14" s="1" t="s">
-        <x:v>152</x:v>
+        <x:v>150</x:v>
       </x:c>
       <x:c r="C14" s="1" t="s">
-        <x:v>168</x:v>
+        <x:v>166</x:v>
       </x:c>
       <x:c r="D14" s="1" t="s">
         <x:v>28</x:v>
@@ -13722,54 +13716,54 @@
     </x:row>
     <x:row r="15">
       <x:c r="A15" s="1" t="s">
-        <x:v>169</x:v>
+        <x:v>167</x:v>
       </x:c>
       <x:c r="B15" s="1" t="s">
-        <x:v>152</x:v>
+        <x:v>150</x:v>
       </x:c>
       <x:c r="C15" s="1" t="s">
-        <x:v>170</x:v>
+        <x:v>168</x:v>
       </x:c>
       <x:c r="D15" s="1" t="s">
-        <x:v>109</x:v>
+        <x:v>107</x:v>
       </x:c>
       <x:c r="E15" s="1" t="s">
-        <x:v>109</x:v>
+        <x:v>107</x:v>
       </x:c>
       <x:c r="H15" s="5" t="s">
-        <x:v>73</x:v>
+        <x:v>71</x:v>
       </x:c>
       <x:c r="I15" s="5" t="s">
-        <x:v>73</x:v>
+        <x:v>71</x:v>
       </x:c>
     </x:row>
     <x:row r="16">
       <x:c r="A16" s="1" t="s">
+        <x:v>169</x:v>
+      </x:c>
+      <x:c r="B16" s="1" t="s">
+        <x:v>150</x:v>
+      </x:c>
+      <x:c r="C16" s="1" t="s">
+        <x:v>170</x:v>
+      </x:c>
+      <x:c r="D16" s="1" t="s">
         <x:v>171</x:v>
       </x:c>
-      <x:c r="B16" s="1" t="s">
-        <x:v>152</x:v>
-      </x:c>
-      <x:c r="C16" s="1" t="s">
-        <x:v>172</x:v>
-      </x:c>
-      <x:c r="D16" s="1" t="s">
-        <x:v>173</x:v>
-      </x:c>
       <x:c r="E16" s="1" t="s">
-        <x:v>71</x:v>
+        <x:v>69</x:v>
       </x:c>
       <x:c r="F16" s="1" t="s">
-        <x:v>139</x:v>
+        <x:v>137</x:v>
       </x:c>
       <x:c r="H16" s="5">
         <x:v>100.0</x:v>
       </x:c>
       <x:c r="I16" s="5" t="s">
-        <x:v>73</x:v>
+        <x:v>71</x:v>
       </x:c>
       <x:c r="J16" s="1" t="s">
-        <x:v>174</x:v>
+        <x:v>172</x:v>
       </x:c>
     </x:row>
     <x:row r="17" ht="30" customHeight="1">
@@ -17819,7 +17813,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="B1" s="2" t="s">
-        <x:v>175</x:v>
+        <x:v>173</x:v>
       </x:c>
       <x:c r="F1" s="4"/>
       <x:c r="G1" s="4"/>
@@ -17831,7 +17825,7 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="B2" s="2" t="s">
-        <x:v>176</x:v>
+        <x:v>174</x:v>
       </x:c>
       <x:c r="F2" s="4"/>
       <x:c r="G2" s="4"/>
@@ -17843,7 +17837,7 @@
         <x:v>5</x:v>
       </x:c>
       <x:c r="B3" s="1" t="s">
-        <x:v>177</x:v>
+        <x:v>175</x:v>
       </x:c>
       <x:c r="D3" s="1"/>
       <x:c r="E3" s="1"/>
@@ -17900,13 +17894,13 @@
         <x:v>18</x:v>
       </x:c>
       <x:c r="B6" s="1" t="s">
-        <x:v>178</x:v>
+        <x:v>176</x:v>
       </x:c>
       <x:c r="C6" s="1" t="s">
-        <x:v>179</x:v>
+        <x:v>177</x:v>
       </x:c>
       <x:c r="D6" s="1" t="s">
-        <x:v>133</x:v>
+        <x:v>131</x:v>
       </x:c>
       <x:c r="E6" s="1" t="s">
         <x:v>28</x:v>
@@ -17918,16 +17912,16 @@
     </x:row>
     <x:row r="7" ht="15.75" hidden="0" customHeight="1">
       <x:c r="A7" s="1" t="s">
-        <x:v>180</x:v>
+        <x:v>178</x:v>
       </x:c>
       <x:c r="B7" s="1" t="s">
-        <x:v>155</x:v>
+        <x:v>153</x:v>
       </x:c>
       <x:c r="C7" s="1" t="s">
-        <x:v>179</x:v>
+        <x:v>177</x:v>
       </x:c>
       <x:c r="D7" s="1" t="s">
-        <x:v>133</x:v>
+        <x:v>131</x:v>
       </x:c>
       <x:c r="E7" s="1" t="s">
         <x:v>28</x:v>
@@ -17939,22 +17933,22 @@
     </x:row>
     <x:row r="8" ht="15.75" hidden="0" customHeight="1">
       <x:c r="A8" s="1" t="s">
+        <x:v>179</x:v>
+      </x:c>
+      <x:c r="B8" s="1" t="s">
+        <x:v>180</x:v>
+      </x:c>
+      <x:c r="C8" s="1" t="s">
+        <x:v>177</x:v>
+      </x:c>
+      <x:c r="D8" s="1" t="s">
         <x:v>181</x:v>
       </x:c>
-      <x:c r="B8" s="1" t="s">
-        <x:v>182</x:v>
-      </x:c>
-      <x:c r="C8" s="1" t="s">
-        <x:v>179</x:v>
-      </x:c>
-      <x:c r="D8" s="1" t="s">
-        <x:v>183</x:v>
-      </x:c>
       <x:c r="E8" s="1" t="s">
-        <x:v>71</x:v>
+        <x:v>69</x:v>
       </x:c>
       <x:c r="F8" s="1" t="s">
-        <x:v>139</x:v>
+        <x:v>137</x:v>
       </x:c>
       <x:c r="H8" s="5">
         <x:v>100.0</x:v>
@@ -17964,58 +17958,58 @@
     </x:row>
     <x:row r="9" ht="15.75" hidden="0" customHeight="1">
       <x:c r="A9" s="1" t="s">
-        <x:v>66</x:v>
+        <x:v>64</x:v>
       </x:c>
       <x:c r="B9" s="1" t="s">
-        <x:v>166</x:v>
+        <x:v>164</x:v>
       </x:c>
       <x:c r="C9" s="1" t="s">
-        <x:v>179</x:v>
+        <x:v>177</x:v>
       </x:c>
       <x:c r="D9" s="1" t="s">
-        <x:v>109</x:v>
+        <x:v>107</x:v>
       </x:c>
       <x:c r="E9" s="1" t="s">
-        <x:v>109</x:v>
+        <x:v>107</x:v>
       </x:c>
       <x:c r="H9" s="5" t="s">
-        <x:v>73</x:v>
+        <x:v>71</x:v>
       </x:c>
       <x:c r="I9" s="3"/>
     </x:row>
     <x:row r="10" ht="15.75" hidden="0" customHeight="1">
       <x:c r="A10" s="1" t="s">
-        <x:v>169</x:v>
+        <x:v>167</x:v>
       </x:c>
       <x:c r="B10" s="1" t="s">
-        <x:v>170</x:v>
+        <x:v>168</x:v>
       </x:c>
       <x:c r="C10" s="1" t="s">
-        <x:v>179</x:v>
+        <x:v>177</x:v>
       </x:c>
       <x:c r="D10" s="1" t="s">
-        <x:v>109</x:v>
+        <x:v>107</x:v>
       </x:c>
       <x:c r="E10" s="1" t="s">
-        <x:v>109</x:v>
+        <x:v>107</x:v>
       </x:c>
       <x:c r="H10" s="5" t="s">
-        <x:v>73</x:v>
+        <x:v>71</x:v>
       </x:c>
       <x:c r="I10" s="3"/>
     </x:row>
     <x:row r="11" ht="15.75" hidden="0" customHeight="1">
       <x:c r="A11" s="1" t="s">
-        <x:v>184</x:v>
+        <x:v>182</x:v>
       </x:c>
       <x:c r="B11" s="1" t="s">
-        <x:v>185</x:v>
+        <x:v>183</x:v>
       </x:c>
       <x:c r="C11" s="1" t="s">
-        <x:v>179</x:v>
+        <x:v>177</x:v>
       </x:c>
       <x:c r="D11" s="1" t="s">
-        <x:v>133</x:v>
+        <x:v>131</x:v>
       </x:c>
       <x:c r="E11" s="1" t="s">
         <x:v>28</x:v>
@@ -18027,16 +18021,16 @@
     </x:row>
     <x:row r="12" ht="36" hidden="0" customHeight="1">
       <x:c r="A12" s="1" t="s">
+        <x:v>184</x:v>
+      </x:c>
+      <x:c r="B12" s="1" t="s">
+        <x:v>185</x:v>
+      </x:c>
+      <x:c r="C12" s="1" t="s">
+        <x:v>177</x:v>
+      </x:c>
+      <x:c r="D12" s="1" t="s">
         <x:v>186</x:v>
-      </x:c>
-      <x:c r="B12" s="1" t="s">
-        <x:v>187</x:v>
-      </x:c>
-      <x:c r="C12" s="1" t="s">
-        <x:v>179</x:v>
-      </x:c>
-      <x:c r="D12" s="1" t="s">
-        <x:v>188</x:v>
       </x:c>
       <x:c r="E12" s="1" t="str">
         <x:v>multi-select choice</x:v>
@@ -18054,37 +18048,37 @@
     </x:row>
     <x:row r="13" ht="15.75" hidden="0" customHeight="1">
       <x:c r="A13" s="1" t="s">
-        <x:v>189</x:v>
+        <x:v>187</x:v>
       </x:c>
       <x:c r="B13" s="1" t="s">
-        <x:v>190</x:v>
+        <x:v>188</x:v>
       </x:c>
       <x:c r="C13" s="1" t="s">
-        <x:v>179</x:v>
+        <x:v>177</x:v>
       </x:c>
       <x:c r="D13" s="1" t="s">
-        <x:v>98</x:v>
+        <x:v>96</x:v>
       </x:c>
       <x:c r="E13" s="1" t="s">
-        <x:v>98</x:v>
+        <x:v>96</x:v>
       </x:c>
       <x:c r="H13" s="5" t="s">
-        <x:v>73</x:v>
+        <x:v>71</x:v>
       </x:c>
       <x:c r="I13" s="3"/>
     </x:row>
     <x:row r="14" ht="15.75" hidden="0" customHeight="1">
       <x:c r="A14" s="1" t="s">
-        <x:v>164</x:v>
+        <x:v>162</x:v>
       </x:c>
       <x:c r="B14" s="1" t="s">
-        <x:v>165</x:v>
+        <x:v>163</x:v>
       </x:c>
       <x:c r="C14" s="1" t="s">
-        <x:v>179</x:v>
+        <x:v>177</x:v>
       </x:c>
       <x:c r="D14" s="1" t="s">
-        <x:v>133</x:v>
+        <x:v>131</x:v>
       </x:c>
       <x:c r="E14" s="1" t="s">
         <x:v>28</x:v>
@@ -18096,16 +18090,16 @@
     </x:row>
     <x:row r="15" ht="15.75" hidden="0" customHeight="1">
       <x:c r="A15" s="1" t="s">
-        <x:v>167</x:v>
+        <x:v>165</x:v>
       </x:c>
       <x:c r="B15" s="1" t="s">
-        <x:v>168</x:v>
+        <x:v>166</x:v>
       </x:c>
       <x:c r="C15" s="1" t="s">
-        <x:v>179</x:v>
+        <x:v>177</x:v>
       </x:c>
       <x:c r="D15" s="1" t="s">
-        <x:v>133</x:v>
+        <x:v>131</x:v>
       </x:c>
       <x:c r="E15" s="1" t="s">
         <x:v>28</x:v>
@@ -22085,7 +22079,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="B1" s="2" t="s">
-        <x:v>191</x:v>
+        <x:v>189</x:v>
       </x:c>
       <x:c r="G1" s="4"/>
       <x:c r="H1" s="1"/>
@@ -22098,7 +22092,7 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="B2" s="2" t="s">
-        <x:v>192</x:v>
+        <x:v>190</x:v>
       </x:c>
       <x:c r="G2" s="4"/>
       <x:c r="H2" s="1"/>
@@ -22150,13 +22144,13 @@
         <x:v>18</x:v>
       </x:c>
       <x:c r="B5" s="2" t="s">
-        <x:v>193</x:v>
+        <x:v>191</x:v>
       </x:c>
       <x:c r="C5" s="2" t="s">
-        <x:v>194</x:v>
+        <x:v>192</x:v>
       </x:c>
       <x:c r="D5" s="2" t="s">
-        <x:v>133</x:v>
+        <x:v>131</x:v>
       </x:c>
       <x:c r="E5" s="2" t="s">
         <x:v>28</x:v>
@@ -22167,21 +22161,21 @@
         <x:v>850.0</x:v>
       </x:c>
       <x:c r="I5" s="5" t="s">
-        <x:v>73</x:v>
+        <x:v>71</x:v>
       </x:c>
     </x:row>
     <x:row r="6">
       <x:c r="A6" s="1" t="s">
-        <x:v>180</x:v>
+        <x:v>178</x:v>
       </x:c>
       <x:c r="B6" s="2" t="s">
-        <x:v>195</x:v>
+        <x:v>193</x:v>
       </x:c>
       <x:c r="C6" s="2" t="s">
-        <x:v>194</x:v>
+        <x:v>192</x:v>
       </x:c>
       <x:c r="D6" s="2" t="s">
-        <x:v>133</x:v>
+        <x:v>131</x:v>
       </x:c>
       <x:c r="E6" s="2" t="s">
         <x:v>28</x:v>
@@ -22192,24 +22186,24 @@
         <x:v>100.0</x:v>
       </x:c>
       <x:c r="I6" s="5" t="s">
-        <x:v>73</x:v>
+        <x:v>71</x:v>
       </x:c>
     </x:row>
     <x:row r="7">
       <x:c r="A7" s="1" t="s">
+        <x:v>194</x:v>
+      </x:c>
+      <x:c r="B7" s="1" t="s">
+        <x:v>192</x:v>
+      </x:c>
+      <x:c r="C7" s="2" t="s">
+        <x:v>192</x:v>
+      </x:c>
+      <x:c r="D7" s="1" t="s">
+        <x:v>195</x:v>
+      </x:c>
+      <x:c r="E7" s="2" t="s">
         <x:v>196</x:v>
-      </x:c>
-      <x:c r="B7" s="1" t="s">
-        <x:v>194</x:v>
-      </x:c>
-      <x:c r="C7" s="2" t="s">
-        <x:v>194</x:v>
-      </x:c>
-      <x:c r="D7" s="1" t="s">
-        <x:v>197</x:v>
-      </x:c>
-      <x:c r="E7" s="2" t="s">
-        <x:v>198</x:v>
       </x:c>
       <x:c r="H7" s="5">
         <x:v>100.0</x:v>
@@ -22220,16 +22214,16 @@
     </x:row>
     <x:row r="8">
       <x:c r="A8" s="1" t="s">
-        <x:v>164</x:v>
+        <x:v>162</x:v>
       </x:c>
       <x:c r="B8" s="1" t="s">
-        <x:v>199</x:v>
+        <x:v>197</x:v>
       </x:c>
       <x:c r="C8" s="2" t="s">
-        <x:v>194</x:v>
+        <x:v>192</x:v>
       </x:c>
       <x:c r="D8" s="1" t="s">
-        <x:v>133</x:v>
+        <x:v>131</x:v>
       </x:c>
       <x:c r="E8" s="2" t="s">
         <x:v>28</x:v>
@@ -22246,39 +22240,39 @@
     </x:row>
     <x:row r="9">
       <x:c r="A9" s="1" t="s">
-        <x:v>66</x:v>
+        <x:v>64</x:v>
       </x:c>
       <x:c r="B9" s="1" t="s">
-        <x:v>200</x:v>
+        <x:v>198</x:v>
       </x:c>
       <x:c r="C9" s="2" t="s">
-        <x:v>194</x:v>
+        <x:v>192</x:v>
       </x:c>
       <x:c r="D9" s="1" t="s">
-        <x:v>109</x:v>
+        <x:v>107</x:v>
       </x:c>
       <x:c r="E9" s="1" t="s">
-        <x:v>109</x:v>
+        <x:v>107</x:v>
       </x:c>
       <x:c r="H9" s="5" t="s">
-        <x:v>73</x:v>
+        <x:v>71</x:v>
       </x:c>
       <x:c r="I9" s="5" t="s">
-        <x:v>73</x:v>
+        <x:v>71</x:v>
       </x:c>
     </x:row>
     <x:row r="10">
       <x:c r="A10" s="1" t="s">
-        <x:v>167</x:v>
+        <x:v>165</x:v>
       </x:c>
       <x:c r="B10" s="1" t="s">
-        <x:v>201</x:v>
+        <x:v>199</x:v>
       </x:c>
       <x:c r="C10" s="2" t="s">
-        <x:v>194</x:v>
+        <x:v>192</x:v>
       </x:c>
       <x:c r="D10" s="1" t="s">
-        <x:v>133</x:v>
+        <x:v>131</x:v>
       </x:c>
       <x:c r="E10" s="2" t="s">
         <x:v>28</x:v>
@@ -22292,25 +22286,25 @@
     </x:row>
     <x:row r="11">
       <x:c r="A11" s="1" t="s">
-        <x:v>169</x:v>
+        <x:v>167</x:v>
       </x:c>
       <x:c r="B11" s="1" t="s">
-        <x:v>202</x:v>
+        <x:v>200</x:v>
       </x:c>
       <x:c r="C11" s="2" t="s">
-        <x:v>194</x:v>
+        <x:v>192</x:v>
       </x:c>
       <x:c r="D11" s="1" t="s">
-        <x:v>109</x:v>
+        <x:v>107</x:v>
       </x:c>
       <x:c r="E11" s="1" t="s">
-        <x:v>109</x:v>
+        <x:v>107</x:v>
       </x:c>
       <x:c r="H11" s="5" t="s">
-        <x:v>73</x:v>
+        <x:v>71</x:v>
       </x:c>
       <x:c r="I11" s="5" t="s">
-        <x:v>73</x:v>
+        <x:v>71</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -22347,7 +22341,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="B1" s="2" t="s">
-        <x:v>203</x:v>
+        <x:v>201</x:v>
       </x:c>
       <x:c r="G1" s="4"/>
       <x:c r="H1" s="1"/>
@@ -22360,17 +22354,17 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="B2" s="2" t="s">
-        <x:v>204</x:v>
+        <x:v>202</x:v>
       </x:c>
       <x:c r="G2" s="4"/>
       <x:c r="H2" s="1"/>
     </x:row>
     <x:row r="3">
       <x:c r="A3" s="1" t="s">
-        <x:v>205</x:v>
+        <x:v>203</x:v>
       </x:c>
       <x:c r="B3" s="1" t="s">
-        <x:v>206</x:v>
+        <x:v>204</x:v>
       </x:c>
       <x:c r="C3" s="1"/>
       <x:c r="D3" s="1"/>
@@ -22416,13 +22410,13 @@
         <x:v>18</x:v>
       </x:c>
       <x:c r="B6" s="1" t="s">
-        <x:v>207</x:v>
+        <x:v>205</x:v>
       </x:c>
       <x:c r="C6" s="1" t="s">
-        <x:v>206</x:v>
+        <x:v>204</x:v>
       </x:c>
       <x:c r="D6" s="1" t="s">
-        <x:v>133</x:v>
+        <x:v>131</x:v>
       </x:c>
       <x:c r="E6" s="1" t="s">
         <x:v>28</x:v>
@@ -22432,21 +22426,21 @@
         <x:v>850.0</x:v>
       </x:c>
       <x:c r="I6" s="5" t="s">
-        <x:v>73</x:v>
+        <x:v>71</x:v>
       </x:c>
     </x:row>
     <x:row r="7">
       <x:c r="A7" s="1" t="s">
-        <x:v>180</x:v>
+        <x:v>178</x:v>
       </x:c>
       <x:c r="B7" s="1" t="s">
-        <x:v>208</x:v>
+        <x:v>206</x:v>
       </x:c>
       <x:c r="C7" s="1" t="s">
-        <x:v>206</x:v>
+        <x:v>204</x:v>
       </x:c>
       <x:c r="D7" s="1" t="s">
-        <x:v>133</x:v>
+        <x:v>131</x:v>
       </x:c>
       <x:c r="E7" s="1" t="s">
         <x:v>28</x:v>
@@ -22456,18 +22450,18 @@
         <x:v>100.0</x:v>
       </x:c>
       <x:c r="I7" s="12" t="s">
-        <x:v>73</x:v>
+        <x:v>71</x:v>
       </x:c>
     </x:row>
     <x:row r="8">
       <x:c r="A8" s="1" t="s">
-        <x:v>209</x:v>
+        <x:v>207</x:v>
       </x:c>
       <x:c r="B8" s="1" t="s">
-        <x:v>210</x:v>
+        <x:v>208</x:v>
       </x:c>
       <x:c r="C8" s="1" t="s">
-        <x:v>206</x:v>
+        <x:v>204</x:v>
       </x:c>
       <x:c r="D8" s="1" t="s">
         <x:v>28</x:v>
@@ -22485,40 +22479,40 @@
     </x:row>
     <x:row r="9">
       <x:c r="A9" s="15" t="s">
+        <x:v>209</x:v>
+      </x:c>
+      <x:c r="B9" s="1" t="s">
+        <x:v>210</x:v>
+      </x:c>
+      <x:c r="C9" s="1" t="s">
+        <x:v>204</x:v>
+      </x:c>
+      <x:c r="D9" s="1" t="s">
         <x:v>211</x:v>
       </x:c>
-      <x:c r="B9" s="1" t="s">
-        <x:v>212</x:v>
-      </x:c>
-      <x:c r="C9" s="1" t="s">
-        <x:v>206</x:v>
-      </x:c>
-      <x:c r="D9" s="1" t="s">
-        <x:v>213</x:v>
-      </x:c>
       <x:c r="E9" s="1" t="s">
-        <x:v>71</x:v>
+        <x:v>69</x:v>
       </x:c>
       <x:c r="F9" s="1" t="s">
-        <x:v>72</x:v>
+        <x:v>70</x:v>
       </x:c>
       <x:c r="G9" s="3"/>
       <x:c r="H9" s="5">
         <x:v>100.0</x:v>
       </x:c>
       <x:c r="I9" s="12" t="s">
-        <x:v>73</x:v>
+        <x:v>71</x:v>
       </x:c>
     </x:row>
     <x:row r="10">
       <x:c r="A10" s="1" t="s">
-        <x:v>214</x:v>
+        <x:v>212</x:v>
       </x:c>
       <x:c r="B10" s="1" t="s">
-        <x:v>215</x:v>
+        <x:v>213</x:v>
       </x:c>
       <x:c r="C10" s="1" t="s">
-        <x:v>206</x:v>
+        <x:v>204</x:v>
       </x:c>
       <x:c r="D10" s="1" t="s">
         <x:v>28</x:v>
@@ -22536,13 +22530,13 @@
     </x:row>
     <x:row r="11">
       <x:c r="A11" s="1" t="s">
-        <x:v>216</x:v>
+        <x:v>214</x:v>
       </x:c>
       <x:c r="B11" s="1" t="s">
-        <x:v>217</x:v>
+        <x:v>215</x:v>
       </x:c>
       <x:c r="C11" s="1" t="s">
-        <x:v>206</x:v>
+        <x:v>204</x:v>
       </x:c>
       <x:c r="D11" s="1" t="s">
         <x:v>28</x:v>
@@ -22560,13 +22554,13 @@
     </x:row>
     <x:row r="12">
       <x:c r="A12" s="1" t="s">
-        <x:v>218</x:v>
+        <x:v>216</x:v>
       </x:c>
       <x:c r="B12" s="1" t="s">
-        <x:v>219</x:v>
+        <x:v>217</x:v>
       </x:c>
       <x:c r="C12" s="1" t="s">
-        <x:v>206</x:v>
+        <x:v>204</x:v>
       </x:c>
       <x:c r="D12" s="1" t="s">
         <x:v>28</x:v>
@@ -22584,13 +22578,13 @@
     </x:row>
     <x:row r="13">
       <x:c r="A13" s="1" t="s">
-        <x:v>164</x:v>
+        <x:v>162</x:v>
       </x:c>
       <x:c r="B13" s="1" t="s">
-        <x:v>220</x:v>
+        <x:v>218</x:v>
       </x:c>
       <x:c r="C13" s="1" t="s">
-        <x:v>206</x:v>
+        <x:v>204</x:v>
       </x:c>
       <x:c r="D13" s="1" t="s">
         <x:v>28</x:v>
@@ -22608,37 +22602,37 @@
     </x:row>
     <x:row r="14">
       <x:c r="A14" s="1" t="s">
-        <x:v>66</x:v>
+        <x:v>64</x:v>
       </x:c>
       <x:c r="B14" s="1" t="s">
-        <x:v>221</x:v>
+        <x:v>219</x:v>
       </x:c>
       <x:c r="C14" s="1" t="s">
-        <x:v>206</x:v>
+        <x:v>204</x:v>
       </x:c>
       <x:c r="D14" s="1" t="s">
-        <x:v>109</x:v>
+        <x:v>107</x:v>
       </x:c>
       <x:c r="E14" s="1" t="s">
-        <x:v>109</x:v>
+        <x:v>107</x:v>
       </x:c>
       <x:c r="G14" s="3"/>
       <x:c r="H14" s="5" t="s">
-        <x:v>73</x:v>
+        <x:v>71</x:v>
       </x:c>
       <x:c r="I14" s="5" t="s">
-        <x:v>73</x:v>
+        <x:v>71</x:v>
       </x:c>
     </x:row>
     <x:row r="15">
       <x:c r="A15" s="1" t="s">
-        <x:v>167</x:v>
+        <x:v>165</x:v>
       </x:c>
       <x:c r="B15" s="1" t="s">
-        <x:v>222</x:v>
+        <x:v>220</x:v>
       </x:c>
       <x:c r="C15" s="1" t="s">
-        <x:v>206</x:v>
+        <x:v>204</x:v>
       </x:c>
       <x:c r="D15" s="1" t="s">
         <x:v>28</x:v>
@@ -22656,67 +22650,67 @@
     </x:row>
     <x:row r="16">
       <x:c r="A16" s="1" t="s">
-        <x:v>169</x:v>
+        <x:v>167</x:v>
       </x:c>
       <x:c r="B16" s="1" t="s">
-        <x:v>223</x:v>
+        <x:v>221</x:v>
       </x:c>
       <x:c r="C16" s="1" t="s">
-        <x:v>206</x:v>
+        <x:v>204</x:v>
       </x:c>
       <x:c r="D16" s="1" t="s">
-        <x:v>109</x:v>
+        <x:v>107</x:v>
       </x:c>
       <x:c r="E16" s="1" t="s">
-        <x:v>109</x:v>
+        <x:v>107</x:v>
       </x:c>
       <x:c r="G16" s="3"/>
       <x:c r="H16" s="5" t="s">
-        <x:v>73</x:v>
+        <x:v>71</x:v>
       </x:c>
       <x:c r="I16" s="5" t="s">
-        <x:v>73</x:v>
+        <x:v>71</x:v>
       </x:c>
     </x:row>
     <x:row r="17">
       <x:c r="A17" s="1" t="s">
+        <x:v>222</x:v>
+      </x:c>
+      <x:c r="B17" s="1" t="s">
+        <x:v>223</x:v>
+      </x:c>
+      <x:c r="C17" s="1" t="s">
+        <x:v>204</x:v>
+      </x:c>
+      <x:c r="D17" s="1" t="s">
         <x:v>224</x:v>
       </x:c>
-      <x:c r="B17" s="1" t="s">
-        <x:v>225</x:v>
-      </x:c>
-      <x:c r="C17" s="1" t="s">
-        <x:v>206</x:v>
-      </x:c>
-      <x:c r="D17" s="1" t="s">
-        <x:v>226</x:v>
-      </x:c>
       <x:c r="E17" s="1" t="s">
-        <x:v>71</x:v>
+        <x:v>69</x:v>
       </x:c>
       <x:c r="F17" s="1" t="s">
-        <x:v>72</x:v>
+        <x:v>70</x:v>
       </x:c>
       <x:c r="G17" s="3"/>
       <x:c r="H17" s="5">
         <x:v>100.0</x:v>
       </x:c>
       <x:c r="I17" s="5" t="s">
-        <x:v>73</x:v>
+        <x:v>71</x:v>
       </x:c>
     </x:row>
     <x:row r="18">
       <x:c r="A18" s="1" t="s">
+        <x:v>225</x:v>
+      </x:c>
+      <x:c r="B18" s="1" t="s">
+        <x:v>226</x:v>
+      </x:c>
+      <x:c r="C18" s="1" t="s">
+        <x:v>204</x:v>
+      </x:c>
+      <x:c r="D18" s="1" t="s">
         <x:v>227</x:v>
-      </x:c>
-      <x:c r="B18" s="1" t="s">
-        <x:v>228</x:v>
-      </x:c>
-      <x:c r="C18" s="1" t="s">
-        <x:v>206</x:v>
-      </x:c>
-      <x:c r="D18" s="1" t="s">
-        <x:v>229</x:v>
       </x:c>
       <x:c r="E18" s="1" t="s">
         <x:v>28</x:v>
@@ -22760,7 +22754,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="B1" s="2" t="s">
-        <x:v>230</x:v>
+        <x:v>228</x:v>
       </x:c>
       <x:c r="D1" s="4"/>
       <x:c r="E1" s="4"/>
@@ -22825,13 +22819,13 @@
         <x:v>18</x:v>
       </x:c>
       <x:c r="B5" s="1" t="s">
-        <x:v>231</x:v>
+        <x:v>229</x:v>
       </x:c>
       <x:c r="C5" s="1" t="s">
-        <x:v>232</x:v>
+        <x:v>230</x:v>
       </x:c>
       <x:c r="D5" s="1" t="s">
-        <x:v>133</x:v>
+        <x:v>131</x:v>
       </x:c>
       <x:c r="E5" s="1" t="s">
         <x:v>28</x:v>
@@ -22845,16 +22839,16 @@
     </x:row>
     <x:row r="6">
       <x:c r="A6" s="1" t="s">
-        <x:v>180</x:v>
+        <x:v>178</x:v>
       </x:c>
       <x:c r="B6" s="1" t="s">
-        <x:v>155</x:v>
+        <x:v>153</x:v>
       </x:c>
       <x:c r="C6" s="1" t="s">
-        <x:v>232</x:v>
+        <x:v>230</x:v>
       </x:c>
       <x:c r="D6" s="1" t="s">
-        <x:v>133</x:v>
+        <x:v>131</x:v>
       </x:c>
       <x:c r="E6" s="1" t="s">
         <x:v>28</x:v>
@@ -22866,47 +22860,47 @@
         <x:v>100.0</x:v>
       </x:c>
       <x:c r="I6" s="13" t="s">
-        <x:v>233</x:v>
+        <x:v>231</x:v>
       </x:c>
     </x:row>
     <x:row r="7">
       <x:c r="A7" s="1" t="s">
-        <x:v>234</x:v>
+        <x:v>232</x:v>
       </x:c>
       <x:c r="B7" s="1" t="s">
-        <x:v>235</x:v>
+        <x:v>233</x:v>
       </x:c>
       <x:c r="C7" s="1" t="s">
-        <x:v>232</x:v>
+        <x:v>230</x:v>
       </x:c>
       <x:c r="D7" s="1" t="s">
         <x:v>28</x:v>
       </x:c>
       <x:c r="E7" s="1" t="s">
-        <x:v>71</x:v>
+        <x:v>69</x:v>
       </x:c>
       <x:c r="F7" s="1" t="s">
-        <x:v>139</x:v>
+        <x:v>137</x:v>
       </x:c>
       <x:c r="G7" s="5">
         <x:v>26.0</x:v>
       </x:c>
       <x:c r="H7" s="5" t="s">
-        <x:v>73</x:v>
+        <x:v>71</x:v>
       </x:c>
       <x:c r="I7" s="1" t="s">
-        <x:v>236</x:v>
+        <x:v>234</x:v>
       </x:c>
     </x:row>
     <x:row r="8">
       <x:c r="A8" s="1" t="s">
-        <x:v>237</x:v>
+        <x:v>235</x:v>
       </x:c>
       <x:c r="B8" s="1" t="s">
-        <x:v>238</x:v>
+        <x:v>236</x:v>
       </x:c>
       <x:c r="C8" s="1" t="s">
-        <x:v>232</x:v>
+        <x:v>230</x:v>
       </x:c>
       <x:c r="D8" s="1" t="s">
         <x:v>28</x:v>
@@ -22923,25 +22917,25 @@
     </x:row>
     <x:row r="9">
       <x:c r="A9" s="1" t="s">
-        <x:v>66</x:v>
+        <x:v>64</x:v>
       </x:c>
       <x:c r="B9" s="1" t="s">
-        <x:v>239</x:v>
+        <x:v>237</x:v>
       </x:c>
       <x:c r="C9" s="1" t="s">
-        <x:v>232</x:v>
+        <x:v>230</x:v>
       </x:c>
       <x:c r="D9" s="1" t="s">
-        <x:v>109</x:v>
+        <x:v>107</x:v>
       </x:c>
       <x:c r="E9" s="1" t="s">
-        <x:v>109</x:v>
+        <x:v>107</x:v>
       </x:c>
       <x:c r="G9" s="5" t="s">
-        <x:v>73</x:v>
+        <x:v>71</x:v>
       </x:c>
       <x:c r="H9" s="5" t="s">
-        <x:v>73</x:v>
+        <x:v>71</x:v>
       </x:c>
     </x:row>
     <x:row r="12">
@@ -22983,7 +22977,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="B1" s="2" t="s">
-        <x:v>240</x:v>
+        <x:v>238</x:v>
       </x:c>
       <x:c r="H1" s="1"/>
       <x:c r="K1" s="1" t="s">
@@ -22995,7 +22989,7 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="B2" s="2" t="s">
-        <x:v>241</x:v>
+        <x:v>239</x:v>
       </x:c>
       <x:c r="F2" s="4"/>
       <x:c r="G2" s="4"/>
@@ -23006,7 +23000,7 @@
         <x:v>5</x:v>
       </x:c>
       <x:c r="B3" s="1" t="s">
-        <x:v>242</x:v>
+        <x:v>240</x:v>
       </x:c>
       <x:c r="H3" s="1"/>
     </x:row>
@@ -23058,31 +23052,31 @@
         <x:v>18</x:v>
       </x:c>
       <x:c r="B6" s="1" t="s">
-        <x:v>243</x:v>
+        <x:v>241</x:v>
       </x:c>
       <x:c r="D6" s="1" t="s">
-        <x:v>133</x:v>
+        <x:v>131</x:v>
       </x:c>
       <x:c r="E6" s="1" t="s">
-        <x:v>133</x:v>
+        <x:v>131</x:v>
       </x:c>
       <x:c r="G6" s="3"/>
       <x:c r="H6" s="5">
         <x:v>100.0</x:v>
       </x:c>
       <x:c r="I6" s="5" t="s">
-        <x:v>73</x:v>
+        <x:v>71</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="15.75" hidden="0" customHeight="1">
       <x:c r="A7" s="1" t="s">
-        <x:v>180</x:v>
+        <x:v>178</x:v>
       </x:c>
       <x:c r="B7" s="1" t="s">
-        <x:v>244</x:v>
+        <x:v>242</x:v>
       </x:c>
       <x:c r="D7" s="1" t="s">
-        <x:v>133</x:v>
+        <x:v>131</x:v>
       </x:c>
       <x:c r="E7" s="1" t="s">
         <x:v>28</x:v>
@@ -23092,39 +23086,39 @@
         <x:v>100.0</x:v>
       </x:c>
       <x:c r="I7" s="5" t="s">
-        <x:v>73</x:v>
+        <x:v>71</x:v>
       </x:c>
     </x:row>
     <x:row r="8" ht="15.75" hidden="0" customHeight="1">
       <x:c r="A8" s="1" t="s">
-        <x:v>245</x:v>
+        <x:v>243</x:v>
       </x:c>
       <x:c r="D8" s="1" t="s">
-        <x:v>197</x:v>
+        <x:v>195</x:v>
       </x:c>
       <x:c r="E8" s="1" t="s">
-        <x:v>246</x:v>
+        <x:v>244</x:v>
       </x:c>
       <x:c r="G8" s="3"/>
       <x:c r="H8" s="5">
         <x:v>100.0</x:v>
       </x:c>
       <x:c r="I8" s="5" t="s">
-        <x:v>73</x:v>
+        <x:v>71</x:v>
       </x:c>
       <x:c r="J8" s="1" t="s">
-        <x:v>247</x:v>
+        <x:v>245</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="15.75" hidden="0" customHeight="1">
       <x:c r="A9" s="1" t="s">
-        <x:v>164</x:v>
+        <x:v>162</x:v>
       </x:c>
       <x:c r="B9" s="1" t="s">
-        <x:v>165</x:v>
+        <x:v>163</x:v>
       </x:c>
       <x:c r="D9" s="1" t="s">
-        <x:v>133</x:v>
+        <x:v>131</x:v>
       </x:c>
       <x:c r="E9" s="1" t="s">
         <x:v>28</x:v>
@@ -23139,34 +23133,34 @@
     </x:row>
     <x:row r="10" ht="15.75" hidden="0" customHeight="1">
       <x:c r="A10" s="1" t="s">
-        <x:v>66</x:v>
+        <x:v>64</x:v>
       </x:c>
       <x:c r="B10" s="1" t="s">
-        <x:v>166</x:v>
+        <x:v>164</x:v>
       </x:c>
       <x:c r="D10" s="1" t="s">
-        <x:v>109</x:v>
+        <x:v>107</x:v>
       </x:c>
       <x:c r="E10" s="1" t="s">
-        <x:v>109</x:v>
+        <x:v>107</x:v>
       </x:c>
       <x:c r="G10" s="3"/>
       <x:c r="H10" s="5" t="s">
-        <x:v>73</x:v>
+        <x:v>71</x:v>
       </x:c>
       <x:c r="I10" s="5" t="s">
-        <x:v>73</x:v>
+        <x:v>71</x:v>
       </x:c>
     </x:row>
     <x:row r="11" ht="15.75" hidden="0" customHeight="1">
       <x:c r="A11" s="1" t="s">
-        <x:v>167</x:v>
+        <x:v>165</x:v>
       </x:c>
       <x:c r="B11" s="1" t="s">
-        <x:v>168</x:v>
+        <x:v>166</x:v>
       </x:c>
       <x:c r="D11" s="1" t="s">
-        <x:v>133</x:v>
+        <x:v>131</x:v>
       </x:c>
       <x:c r="E11" s="1" t="s">
         <x:v>28</x:v>
@@ -23181,34 +23175,34 @@
     </x:row>
     <x:row r="12" ht="15.75" hidden="0" customHeight="1">
       <x:c r="A12" s="1" t="s">
-        <x:v>169</x:v>
+        <x:v>167</x:v>
       </x:c>
       <x:c r="B12" s="1" t="s">
-        <x:v>170</x:v>
+        <x:v>168</x:v>
       </x:c>
       <x:c r="D12" s="1" t="s">
-        <x:v>109</x:v>
+        <x:v>107</x:v>
       </x:c>
       <x:c r="E12" s="1" t="s">
-        <x:v>109</x:v>
+        <x:v>107</x:v>
       </x:c>
       <x:c r="G12" s="3"/>
       <x:c r="H12" s="5" t="s">
-        <x:v>73</x:v>
+        <x:v>71</x:v>
       </x:c>
       <x:c r="I12" s="5" t="s">
-        <x:v>73</x:v>
+        <x:v>71</x:v>
       </x:c>
     </x:row>
     <x:row r="13" ht="48" hidden="0" customHeight="1">
       <x:c r="A13" s="1" t="s">
+        <x:v>246</x:v>
+      </x:c>
+      <x:c r="B13" s="1" t="s">
+        <x:v>247</x:v>
+      </x:c>
+      <x:c r="D13" s="1" t="s">
         <x:v>248</x:v>
-      </x:c>
-      <x:c r="B13" s="1" t="s">
-        <x:v>249</x:v>
-      </x:c>
-      <x:c r="D13" s="1" t="s">
-        <x:v>250</x:v>
       </x:c>
       <x:c r="E13" s="1" t="str">
         <x:v>multi-select choice</x:v>
@@ -23221,7 +23215,7 @@
         <x:v>100.0</x:v>
       </x:c>
       <x:c r="I13" s="5" t="s">
-        <x:v>73</x:v>
+        <x:v>71</x:v>
       </x:c>
       <x:c r="J13" s="22" t="str">
         <x:v>Mapped by 05-create-system-links.m through relationship_type_dataverse_format. QA reports every unknown relationship token; reconcile each System Link and its complete set of selections.</x:v>
@@ -23229,16 +23223,16 @@
     </x:row>
     <x:row r="14" ht="15.75" hidden="0" customHeight="1">
       <x:c r="A14" s="1" t="s">
-        <x:v>251</x:v>
+        <x:v>249</x:v>
       </x:c>
       <x:c r="B14" s="1" t="s">
-        <x:v>252</x:v>
+        <x:v>250</x:v>
       </x:c>
       <x:c r="D14" s="1" t="s">
-        <x:v>197</x:v>
+        <x:v>195</x:v>
       </x:c>
       <x:c r="E14" s="1" t="s">
-        <x:v>246</x:v>
+        <x:v>244</x:v>
       </x:c>
       <x:c r="H14" s="1">
         <x:v>100.0</x:v>
@@ -23356,7 +23350,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="B1" s="2" t="s">
-        <x:v>253</x:v>
+        <x:v>251</x:v>
       </x:c>
       <x:c r="CK1" s="1" t="s">
         <x:v>2</x:v>
@@ -23367,10 +23361,10 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="B2" s="2" t="s">
-        <x:v>254</x:v>
+        <x:v>252</x:v>
       </x:c>
       <x:c r="BC2" s="1" t="s">
-        <x:v>255</x:v>
+        <x:v>253</x:v>
       </x:c>
     </x:row>
     <x:row r="3">
@@ -23378,7 +23372,7 @@
         <x:v>5</x:v>
       </x:c>
       <x:c r="BC3" s="1" t="s">
-        <x:v>256</x:v>
+        <x:v>254</x:v>
       </x:c>
     </x:row>
     <x:row r="4">
@@ -23425,7 +23419,7 @@
         <x:v>17</x:v>
       </x:c>
       <x:c r="BC5" s="1" t="s">
-        <x:v>257</x:v>
+        <x:v>255</x:v>
       </x:c>
     </x:row>
     <x:row r="6">
@@ -23436,10 +23430,10 @@
         <x:v>27</x:v>
       </x:c>
       <x:c r="C6" s="1" t="s">
-        <x:v>258</x:v>
+        <x:v>256</x:v>
       </x:c>
       <x:c r="D6" s="1" t="s">
-        <x:v>133</x:v>
+        <x:v>131</x:v>
       </x:c>
       <x:c r="E6" s="1" t="s">
         <x:v>28</x:v>
@@ -23450,13 +23444,13 @@
         <x:v>18</x:v>
       </x:c>
       <x:c r="B7" s="1" t="s">
-        <x:v>259</x:v>
+        <x:v>257</x:v>
       </x:c>
       <x:c r="C7" s="1" t="s">
-        <x:v>260</x:v>
+        <x:v>258</x:v>
       </x:c>
       <x:c r="D7" s="1" t="s">
-        <x:v>133</x:v>
+        <x:v>131</x:v>
       </x:c>
       <x:c r="E7" s="1" t="s">
         <x:v>28</x:v>
@@ -23471,10 +23465,10 @@
         <x:v>27</x:v>
       </x:c>
       <x:c r="C8" s="1" t="s">
-        <x:v>261</x:v>
+        <x:v>259</x:v>
       </x:c>
       <x:c r="D8" s="1" t="s">
-        <x:v>133</x:v>
+        <x:v>131</x:v>
       </x:c>
       <x:c r="E8" s="1" t="s">
         <x:v>28</x:v>
@@ -23489,7 +23483,7 @@
         <x:v>27</x:v>
       </x:c>
       <x:c r="C9" s="1" t="s">
-        <x:v>262</x:v>
+        <x:v>260</x:v>
       </x:c>
       <x:c r="D9" s="1" t="s">
         <x:v>28</x:v>
@@ -23498,7 +23492,7 @@
         <x:v>28</x:v>
       </x:c>
       <x:c r="K9" s="1" t="s">
-        <x:v>263</x:v>
+        <x:v>261</x:v>
       </x:c>
     </x:row>
     <x:row r="10">
@@ -23509,7 +23503,7 @@
         <x:v>27</x:v>
       </x:c>
       <x:c r="C10" s="1" t="s">
-        <x:v>264</x:v>
+        <x:v>262</x:v>
       </x:c>
       <x:c r="D10" s="1" t="s">
         <x:v>28</x:v>
@@ -23520,13 +23514,13 @@
     </x:row>
     <x:row r="11">
       <x:c r="A11" s="1" t="s">
-        <x:v>181</x:v>
+        <x:v>179</x:v>
       </x:c>
       <x:c r="B11" s="1" t="s">
         <x:v>27</x:v>
       </x:c>
       <x:c r="C11" s="1" t="s">
-        <x:v>265</x:v>
+        <x:v>263</x:v>
       </x:c>
       <x:c r="D11" s="1" t="s">
         <x:v>28</x:v>
@@ -23544,7 +23538,7 @@
         <x:v>27</x:v>
       </x:c>
       <x:c r="C12" s="1" t="s">
-        <x:v>266</x:v>
+        <x:v>264</x:v>
       </x:c>
       <x:c r="D12" s="1" t="s">
         <x:v>28</x:v>
@@ -23555,13 +23549,13 @@
     </x:row>
     <x:row r="13">
       <x:c r="A13" s="1" t="s">
-        <x:v>267</x:v>
+        <x:v>265</x:v>
       </x:c>
       <x:c r="B13" s="1" t="s">
         <x:v>27</x:v>
       </x:c>
       <x:c r="C13" s="1" t="s">
-        <x:v>268</x:v>
+        <x:v>266</x:v>
       </x:c>
       <x:c r="D13" s="1" t="s">
         <x:v>28</x:v>
@@ -23572,13 +23566,13 @@
     </x:row>
     <x:row r="14">
       <x:c r="A14" s="1" t="s">
-        <x:v>269</x:v>
+        <x:v>267</x:v>
       </x:c>
       <x:c r="B14" s="1" t="s">
         <x:v>27</x:v>
       </x:c>
       <x:c r="C14" s="1" t="s">
-        <x:v>270</x:v>
+        <x:v>268</x:v>
       </x:c>
       <x:c r="D14" s="1" t="s">
         <x:v>28</x:v>
@@ -23589,13 +23583,13 @@
     </x:row>
     <x:row r="15">
       <x:c r="A15" s="1" t="s">
-        <x:v>271</x:v>
+        <x:v>269</x:v>
       </x:c>
       <x:c r="B15" s="1" t="s">
         <x:v>27</x:v>
       </x:c>
       <x:c r="C15" s="1" t="s">
-        <x:v>272</x:v>
+        <x:v>270</x:v>
       </x:c>
       <x:c r="D15" s="1" t="s">
         <x:v>28</x:v>
@@ -23606,13 +23600,13 @@
     </x:row>
     <x:row r="16">
       <x:c r="A16" s="1" t="s">
-        <x:v>273</x:v>
+        <x:v>271</x:v>
       </x:c>
       <x:c r="B16" s="1" t="s">
         <x:v>27</x:v>
       </x:c>
       <x:c r="C16" s="1" t="s">
-        <x:v>274</x:v>
+        <x:v>272</x:v>
       </x:c>
       <x:c r="D16" s="1" t="s">
         <x:v>28</x:v>
@@ -23623,13 +23617,13 @@
     </x:row>
     <x:row r="17">
       <x:c r="A17" s="1" t="s">
-        <x:v>275</x:v>
+        <x:v>273</x:v>
       </x:c>
       <x:c r="B17" s="1" t="s">
         <x:v>27</x:v>
       </x:c>
       <x:c r="C17" s="1" t="s">
-        <x:v>276</x:v>
+        <x:v>274</x:v>
       </x:c>
       <x:c r="D17" s="1" t="s">
         <x:v>28</x:v>
@@ -23640,13 +23634,13 @@
     </x:row>
     <x:row r="18">
       <x:c r="A18" s="1" t="s">
-        <x:v>277</x:v>
+        <x:v>275</x:v>
       </x:c>
       <x:c r="B18" s="1" t="s">
         <x:v>27</x:v>
       </x:c>
       <x:c r="C18" s="1" t="s">
-        <x:v>278</x:v>
+        <x:v>276</x:v>
       </x:c>
       <x:c r="D18" s="1" t="s">
         <x:v>28</x:v>
@@ -23657,13 +23651,13 @@
     </x:row>
     <x:row r="19">
       <x:c r="A19" s="1" t="s">
-        <x:v>279</x:v>
+        <x:v>277</x:v>
       </x:c>
       <x:c r="B19" s="1" t="s">
         <x:v>27</x:v>
       </x:c>
       <x:c r="C19" s="1" t="s">
-        <x:v>280</x:v>
+        <x:v>278</x:v>
       </x:c>
       <x:c r="D19" s="1" t="s">
         <x:v>28</x:v>
@@ -23680,7 +23674,7 @@
         <x:v>27</x:v>
       </x:c>
       <x:c r="C20" s="1" t="s">
-        <x:v>281</x:v>
+        <x:v>279</x:v>
       </x:c>
       <x:c r="D20" s="1" t="s">
         <x:v>28</x:v>
@@ -23691,30 +23685,30 @@
     </x:row>
     <x:row r="21">
       <x:c r="A21" s="1" t="s">
-        <x:v>282</x:v>
+        <x:v>280</x:v>
       </x:c>
       <x:c r="B21" s="1" t="s">
         <x:v>27</x:v>
       </x:c>
       <x:c r="C21" s="1" t="s">
-        <x:v>283</x:v>
+        <x:v>281</x:v>
       </x:c>
       <x:c r="D21" s="1" t="s">
-        <x:v>98</x:v>
+        <x:v>96</x:v>
       </x:c>
       <x:c r="E21" s="1" t="s">
-        <x:v>284</x:v>
+        <x:v>282</x:v>
       </x:c>
     </x:row>
     <x:row r="22">
       <x:c r="A22" s="1" t="s">
-        <x:v>285</x:v>
+        <x:v>283</x:v>
       </x:c>
       <x:c r="B22" s="1" t="s">
         <x:v>27</x:v>
       </x:c>
       <x:c r="C22" s="1" t="s">
-        <x:v>286</x:v>
+        <x:v>284</x:v>
       </x:c>
       <x:c r="D22" s="1" t="s">
         <x:v>28</x:v>
@@ -23731,7 +23725,7 @@
         <x:v>27</x:v>
       </x:c>
       <x:c r="C23" s="1" t="s">
-        <x:v>287</x:v>
+        <x:v>285</x:v>
       </x:c>
       <x:c r="D23" s="1" t="s">
         <x:v>28</x:v>
@@ -23742,13 +23736,13 @@
     </x:row>
     <x:row r="24">
       <x:c r="A24" s="1" t="s">
-        <x:v>146</x:v>
+        <x:v>144</x:v>
       </x:c>
       <x:c r="B24" s="1" t="s">
         <x:v>27</x:v>
       </x:c>
       <x:c r="C24" s="1" t="s">
-        <x:v>147</x:v>
+        <x:v>145</x:v>
       </x:c>
       <x:c r="D24" s="1" t="s">
         <x:v>28</x:v>
@@ -23759,13 +23753,13 @@
     </x:row>
     <x:row r="25">
       <x:c r="A25" s="1" t="s">
-        <x:v>288</x:v>
+        <x:v>286</x:v>
       </x:c>
       <x:c r="B25" s="1" t="s">
         <x:v>27</x:v>
       </x:c>
       <x:c r="C25" s="1" t="s">
-        <x:v>289</x:v>
+        <x:v>287</x:v>
       </x:c>
       <x:c r="D25" s="1" t="s">
         <x:v>28</x:v>
@@ -23776,81 +23770,81 @@
     </x:row>
     <x:row r="26">
       <x:c r="A26" s="1" t="s">
-        <x:v>290</x:v>
+        <x:v>288</x:v>
       </x:c>
       <x:c r="B26" s="1" t="s">
         <x:v>27</x:v>
       </x:c>
       <x:c r="C26" s="1" t="s">
-        <x:v>291</x:v>
+        <x:v>289</x:v>
       </x:c>
       <x:c r="D26" s="1" t="s">
-        <x:v>98</x:v>
+        <x:v>96</x:v>
       </x:c>
       <x:c r="E26" s="1" t="s">
-        <x:v>98</x:v>
+        <x:v>96</x:v>
       </x:c>
     </x:row>
     <x:row r="27">
       <x:c r="A27" s="1" t="s">
-        <x:v>292</x:v>
+        <x:v>290</x:v>
       </x:c>
       <x:c r="B27" s="1" t="s">
         <x:v>27</x:v>
       </x:c>
       <x:c r="C27" s="1" t="s">
-        <x:v>293</x:v>
+        <x:v>291</x:v>
       </x:c>
       <x:c r="D27" s="1" t="s">
         <x:v>28</x:v>
       </x:c>
       <x:c r="E27" s="1" t="s">
-        <x:v>71</x:v>
+        <x:v>69</x:v>
       </x:c>
     </x:row>
     <x:row r="28">
       <x:c r="A28" s="1" t="s">
-        <x:v>67</x:v>
+        <x:v>65</x:v>
       </x:c>
       <x:c r="B28" s="1" t="s">
         <x:v>27</x:v>
       </x:c>
       <x:c r="C28" s="1" t="s">
-        <x:v>294</x:v>
+        <x:v>292</x:v>
       </x:c>
       <x:c r="D28" s="1" t="s">
-        <x:v>109</x:v>
+        <x:v>107</x:v>
       </x:c>
       <x:c r="E28" s="1" t="s">
-        <x:v>109</x:v>
+        <x:v>107</x:v>
       </x:c>
     </x:row>
     <x:row r="29">
       <x:c r="A29" s="1" t="s">
-        <x:v>295</x:v>
+        <x:v>293</x:v>
       </x:c>
       <x:c r="B29" s="1" t="s">
         <x:v>27</x:v>
       </x:c>
       <x:c r="C29" s="1" t="s">
-        <x:v>296</x:v>
+        <x:v>294</x:v>
       </x:c>
       <x:c r="D29" s="1" t="s">
-        <x:v>109</x:v>
+        <x:v>107</x:v>
       </x:c>
       <x:c r="E29" s="1" t="s">
-        <x:v>109</x:v>
+        <x:v>107</x:v>
       </x:c>
     </x:row>
     <x:row r="30">
       <x:c r="A30" s="1" t="s">
-        <x:v>297</x:v>
+        <x:v>295</x:v>
       </x:c>
       <x:c r="B30" s="1" t="s">
         <x:v>27</x:v>
       </x:c>
       <x:c r="C30" s="1" t="s">
-        <x:v>298</x:v>
+        <x:v>296</x:v>
       </x:c>
       <x:c r="D30" s="1" t="s">
         <x:v>28</x:v>
@@ -23861,24 +23855,24 @@
     </x:row>
     <x:row r="31">
       <x:c r="A31" s="1" t="s">
-        <x:v>66</x:v>
+        <x:v>64</x:v>
       </x:c>
       <x:c r="B31" s="1" t="s">
         <x:v>27</x:v>
       </x:c>
       <x:c r="C31" s="1" t="s">
-        <x:v>166</x:v>
+        <x:v>164</x:v>
       </x:c>
       <x:c r="D31" s="1" t="s">
-        <x:v>109</x:v>
+        <x:v>107</x:v>
       </x:c>
       <x:c r="E31" s="1" t="s">
-        <x:v>109</x:v>
+        <x:v>107</x:v>
       </x:c>
     </x:row>
     <x:row r="32">
       <x:c r="A32" s="1" t="s">
-        <x:v>299</x:v>
+        <x:v>297</x:v>
       </x:c>
       <x:c r="B32" s="20"/>
       <x:c r="D32" s="1" t="s">
@@ -23890,13 +23884,13 @@
     </x:row>
     <x:row r="33">
       <x:c r="A33" s="1" t="s">
-        <x:v>300</x:v>
+        <x:v>298</x:v>
       </x:c>
       <x:c r="B33" s="1" t="s">
         <x:v>27</x:v>
       </x:c>
       <x:c r="C33" s="1" t="s">
-        <x:v>301</x:v>
+        <x:v>299</x:v>
       </x:c>
       <x:c r="D33" s="1" t="s">
         <x:v>28</x:v>
@@ -23907,47 +23901,47 @@
     </x:row>
     <x:row r="34">
       <x:c r="A34" s="1" t="s">
-        <x:v>302</x:v>
+        <x:v>300</x:v>
       </x:c>
       <x:c r="B34" s="1" t="s">
         <x:v>27</x:v>
       </x:c>
       <x:c r="C34" s="1" t="s">
-        <x:v>303</x:v>
+        <x:v>301</x:v>
       </x:c>
       <x:c r="D34" s="1" t="s">
-        <x:v>109</x:v>
+        <x:v>107</x:v>
       </x:c>
       <x:c r="E34" s="1" t="s">
-        <x:v>109</x:v>
+        <x:v>107</x:v>
       </x:c>
     </x:row>
     <x:row r="35">
       <x:c r="A35" s="1" t="s">
-        <x:v>92</x:v>
+        <x:v>90</x:v>
       </x:c>
       <x:c r="B35" s="1" t="s">
         <x:v>27</x:v>
       </x:c>
       <x:c r="C35" s="1" t="s">
-        <x:v>304</x:v>
+        <x:v>302</x:v>
       </x:c>
       <x:c r="D35" s="1" t="s">
-        <x:v>109</x:v>
+        <x:v>107</x:v>
       </x:c>
       <x:c r="E35" s="1" t="s">
-        <x:v>109</x:v>
+        <x:v>107</x:v>
       </x:c>
     </x:row>
     <x:row r="36">
       <x:c r="A36" s="1" t="s">
-        <x:v>305</x:v>
+        <x:v>303</x:v>
       </x:c>
       <x:c r="B36" s="1" t="s">
         <x:v>27</x:v>
       </x:c>
       <x:c r="C36" s="1" t="s">
-        <x:v>306</x:v>
+        <x:v>304</x:v>
       </x:c>
       <x:c r="D36" s="1" t="s">
         <x:v>28</x:v>
@@ -23958,13 +23952,13 @@
     </x:row>
     <x:row r="37">
       <x:c r="A37" s="1" t="s">
-        <x:v>307</x:v>
+        <x:v>305</x:v>
       </x:c>
       <x:c r="B37" s="1" t="s">
         <x:v>27</x:v>
       </x:c>
       <x:c r="C37" s="1" t="s">
-        <x:v>308</x:v>
+        <x:v>306</x:v>
       </x:c>
       <x:c r="D37" s="1" t="s">
         <x:v>28</x:v>
@@ -23975,13 +23969,13 @@
     </x:row>
     <x:row r="38">
       <x:c r="A38" s="1" t="s">
-        <x:v>309</x:v>
+        <x:v>307</x:v>
       </x:c>
       <x:c r="B38" s="1" t="s">
-        <x:v>259</x:v>
+        <x:v>257</x:v>
       </x:c>
       <x:c r="C38" s="1" t="s">
-        <x:v>310</x:v>
+        <x:v>308</x:v>
       </x:c>
       <x:c r="D38" s="1" t="s">
         <x:v>28</x:v>
@@ -23995,30 +23989,30 @@
     </x:row>
     <x:row r="39">
       <x:c r="A39" s="1" t="s">
-        <x:v>311</x:v>
+        <x:v>309</x:v>
       </x:c>
       <x:c r="B39" s="1" t="s">
-        <x:v>259</x:v>
+        <x:v>257</x:v>
       </x:c>
       <x:c r="C39" s="1" t="s">
-        <x:v>312</x:v>
+        <x:v>310</x:v>
       </x:c>
       <x:c r="D39" s="1" t="s">
-        <x:v>109</x:v>
+        <x:v>107</x:v>
       </x:c>
       <x:c r="E39" s="1" t="s">
-        <x:v>109</x:v>
+        <x:v>107</x:v>
       </x:c>
     </x:row>
     <x:row r="40">
       <x:c r="A40" s="1" t="s">
-        <x:v>313</x:v>
+        <x:v>311</x:v>
       </x:c>
       <x:c r="B40" s="1" t="s">
-        <x:v>259</x:v>
+        <x:v>257</x:v>
       </x:c>
       <x:c r="C40" s="1" t="s">
-        <x:v>314</x:v>
+        <x:v>312</x:v>
       </x:c>
       <x:c r="D40" s="1" t="s">
         <x:v>28</x:v>
@@ -24032,13 +24026,13 @@
     </x:row>
     <x:row r="41">
       <x:c r="A41" s="1" t="s">
-        <x:v>315</x:v>
+        <x:v>313</x:v>
       </x:c>
       <x:c r="B41" s="1" t="s">
         <x:v>27</x:v>
       </x:c>
       <x:c r="C41" s="1" t="s">
-        <x:v>316</x:v>
+        <x:v>314</x:v>
       </x:c>
       <x:c r="D41" s="1" t="s">
         <x:v>28</x:v>
@@ -24049,13 +24043,13 @@
     </x:row>
     <x:row r="42">
       <x:c r="A42" s="1" t="s">
-        <x:v>317</x:v>
+        <x:v>315</x:v>
       </x:c>
       <x:c r="B42" s="1" t="s">
         <x:v>27</x:v>
       </x:c>
       <x:c r="C42" s="1" t="s">
-        <x:v>318</x:v>
+        <x:v>316</x:v>
       </x:c>
       <x:c r="D42" s="1" t="s">
         <x:v>28</x:v>
@@ -24066,13 +24060,13 @@
     </x:row>
     <x:row r="43">
       <x:c r="A43" s="1" t="s">
-        <x:v>319</x:v>
+        <x:v>317</x:v>
       </x:c>
       <x:c r="B43" s="1" t="s">
         <x:v>27</x:v>
       </x:c>
       <x:c r="C43" s="1" t="s">
-        <x:v>320</x:v>
+        <x:v>318</x:v>
       </x:c>
       <x:c r="D43" s="1" t="s">
         <x:v>28</x:v>
@@ -24083,13 +24077,13 @@
     </x:row>
     <x:row r="44">
       <x:c r="A44" s="1" t="s">
-        <x:v>321</x:v>
+        <x:v>319</x:v>
       </x:c>
       <x:c r="B44" s="1" t="s">
         <x:v>27</x:v>
       </x:c>
       <x:c r="C44" s="1" t="s">
-        <x:v>322</x:v>
+        <x:v>320</x:v>
       </x:c>
       <x:c r="D44" s="1" t="s">
         <x:v>28</x:v>
@@ -24100,13 +24094,13 @@
     </x:row>
     <x:row r="45">
       <x:c r="A45" s="1" t="s">
-        <x:v>323</x:v>
+        <x:v>321</x:v>
       </x:c>
       <x:c r="B45" s="1" t="s">
         <x:v>27</x:v>
       </x:c>
       <x:c r="C45" s="1" t="s">
-        <x:v>324</x:v>
+        <x:v>322</x:v>
       </x:c>
       <x:c r="D45" s="1" t="s">
         <x:v>28</x:v>
@@ -24117,13 +24111,13 @@
     </x:row>
     <x:row r="46">
       <x:c r="A46" s="1" t="s">
-        <x:v>325</x:v>
+        <x:v>323</x:v>
       </x:c>
       <x:c r="B46" s="1" t="s">
         <x:v>27</x:v>
       </x:c>
       <x:c r="C46" s="1" t="s">
-        <x:v>326</x:v>
+        <x:v>324</x:v>
       </x:c>
       <x:c r="D46" s="1" t="s">
         <x:v>28</x:v>
@@ -24134,13 +24128,13 @@
     </x:row>
     <x:row r="47">
       <x:c r="A47" s="1" t="s">
-        <x:v>327</x:v>
+        <x:v>325</x:v>
       </x:c>
       <x:c r="B47" s="1" t="s">
         <x:v>27</x:v>
       </x:c>
       <x:c r="C47" s="1" t="s">
-        <x:v>328</x:v>
+        <x:v>326</x:v>
       </x:c>
       <x:c r="D47" s="1" t="s">
         <x:v>28</x:v>
@@ -24151,34 +24145,34 @@
     </x:row>
     <x:row r="48">
       <x:c r="A48" s="1" t="s">
-        <x:v>329</x:v>
+        <x:v>327</x:v>
       </x:c>
       <x:c r="B48" s="1" t="s">
         <x:v>27</x:v>
       </x:c>
       <x:c r="C48" s="1" t="s">
-        <x:v>330</x:v>
+        <x:v>328</x:v>
       </x:c>
       <x:c r="D48" s="1" t="s">
-        <x:v>331</x:v>
+        <x:v>329</x:v>
       </x:c>
       <x:c r="E48" s="1" t="s">
-        <x:v>71</x:v>
+        <x:v>69</x:v>
       </x:c>
       <x:c r="F48" s="1" t="s">
-        <x:v>72</x:v>
+        <x:v>70</x:v>
       </x:c>
       <x:c r="G48" s="1"/>
     </x:row>
     <x:row r="49">
       <x:c r="A49" s="1" t="s">
-        <x:v>104</x:v>
+        <x:v>102</x:v>
       </x:c>
       <x:c r="B49" s="1" t="s">
         <x:v>27</x:v>
       </x:c>
       <x:c r="C49" s="1" t="s">
-        <x:v>332</x:v>
+        <x:v>330</x:v>
       </x:c>
       <x:c r="D49" s="1" t="s">
         <x:v>28</x:v>
@@ -24192,41 +24186,41 @@
     </x:row>
     <x:row r="50">
       <x:c r="A50" s="1" t="s">
+        <x:v>331</x:v>
+      </x:c>
+      <x:c r="B50" s="1" t="s">
+        <x:v>332</x:v>
+      </x:c>
+      <x:c r="C50" s="1" t="s">
         <x:v>333</x:v>
       </x:c>
-      <x:c r="B50" s="1" t="s">
-        <x:v>334</x:v>
-      </x:c>
-      <x:c r="C50" s="1" t="s">
-        <x:v>335</x:v>
-      </x:c>
       <x:c r="D50" s="1" t="s">
-        <x:v>109</x:v>
+        <x:v>107</x:v>
       </x:c>
       <x:c r="E50" s="1" t="s">
-        <x:v>109</x:v>
+        <x:v>107</x:v>
       </x:c>
     </x:row>
     <x:row r="51">
       <x:c r="A51" s="1" t="s">
-        <x:v>336</x:v>
+        <x:v>334</x:v>
       </x:c>
       <x:c r="B51" s="1" t="s">
-        <x:v>334</x:v>
+        <x:v>332</x:v>
       </x:c>
       <x:c r="C51" s="1" t="s">
-        <x:v>337</x:v>
+        <x:v>335</x:v>
       </x:c>
       <x:c r="D51" s="1" t="s">
-        <x:v>109</x:v>
+        <x:v>107</x:v>
       </x:c>
       <x:c r="E51" s="1" t="s">
-        <x:v>109</x:v>
+        <x:v>107</x:v>
       </x:c>
     </x:row>
     <x:row r="52">
       <x:c r="A52" s="1" t="s">
-        <x:v>338</x:v>
+        <x:v>336</x:v>
       </x:c>
       <x:c r="B52" s="20"/>
       <x:c r="D52" s="1" t="s">
@@ -24238,7 +24232,7 @@
     </x:row>
     <x:row r="53">
       <x:c r="A53" s="1" t="s">
-        <x:v>339</x:v>
+        <x:v>337</x:v>
       </x:c>
       <x:c r="B53" s="20"/>
       <x:c r="D53" s="1" t="s">
@@ -24250,13 +24244,13 @@
     </x:row>
     <x:row r="54">
       <x:c r="A54" s="1" t="s">
-        <x:v>340</x:v>
+        <x:v>338</x:v>
       </x:c>
       <x:c r="B54" s="1" t="s">
         <x:v>27</x:v>
       </x:c>
       <x:c r="C54" s="1" t="s">
-        <x:v>341</x:v>
+        <x:v>339</x:v>
       </x:c>
       <x:c r="D54" s="1" t="s">
         <x:v>28</x:v>
@@ -24267,13 +24261,13 @@
     </x:row>
     <x:row r="55">
       <x:c r="A55" s="1" t="s">
-        <x:v>342</x:v>
+        <x:v>340</x:v>
       </x:c>
       <x:c r="B55" s="1" t="s">
         <x:v>27</x:v>
       </x:c>
       <x:c r="C55" s="1" t="s">
-        <x:v>343</x:v>
+        <x:v>341</x:v>
       </x:c>
       <x:c r="D55" s="1" t="s">
         <x:v>28</x:v>
@@ -24284,13 +24278,13 @@
     </x:row>
     <x:row r="56">
       <x:c r="A56" s="1" t="s">
-        <x:v>344</x:v>
+        <x:v>342</x:v>
       </x:c>
       <x:c r="B56" s="1" t="s">
         <x:v>27</x:v>
       </x:c>
       <x:c r="C56" s="1" t="s">
-        <x:v>345</x:v>
+        <x:v>343</x:v>
       </x:c>
       <x:c r="D56" s="1" t="s">
         <x:v>28</x:v>
@@ -24301,13 +24295,13 @@
     </x:row>
     <x:row r="57">
       <x:c r="A57" s="1" t="s">
-        <x:v>346</x:v>
+        <x:v>344</x:v>
       </x:c>
       <x:c r="B57" s="1" t="s">
         <x:v>27</x:v>
       </x:c>
       <x:c r="C57" s="1" t="s">
-        <x:v>347</x:v>
+        <x:v>345</x:v>
       </x:c>
       <x:c r="D57" s="1" t="s">
         <x:v>28</x:v>
@@ -24318,13 +24312,13 @@
     </x:row>
     <x:row r="58">
       <x:c r="A58" s="1" t="s">
-        <x:v>348</x:v>
+        <x:v>346</x:v>
       </x:c>
       <x:c r="B58" s="1" t="s">
         <x:v>27</x:v>
       </x:c>
       <x:c r="C58" s="1" t="s">
-        <x:v>349</x:v>
+        <x:v>347</x:v>
       </x:c>
       <x:c r="D58" s="1" t="s">
         <x:v>28</x:v>
@@ -24335,47 +24329,47 @@
     </x:row>
     <x:row r="59">
       <x:c r="A59" s="1" t="s">
-        <x:v>350</x:v>
+        <x:v>348</x:v>
       </x:c>
       <x:c r="B59" s="1" t="s">
         <x:v>27</x:v>
       </x:c>
       <x:c r="C59" s="1" t="s">
-        <x:v>351</x:v>
+        <x:v>349</x:v>
       </x:c>
       <x:c r="D59" s="1" t="s">
-        <x:v>352</x:v>
+        <x:v>350</x:v>
       </x:c>
       <x:c r="E59" s="1" t="s">
-        <x:v>352</x:v>
+        <x:v>350</x:v>
       </x:c>
     </x:row>
     <x:row r="60">
       <x:c r="A60" s="1" t="s">
-        <x:v>353</x:v>
+        <x:v>351</x:v>
       </x:c>
       <x:c r="B60" s="1" t="s">
         <x:v>27</x:v>
       </x:c>
       <x:c r="C60" s="1" t="s">
-        <x:v>354</x:v>
+        <x:v>352</x:v>
       </x:c>
       <x:c r="D60" s="1" t="s">
-        <x:v>352</x:v>
+        <x:v>350</x:v>
       </x:c>
       <x:c r="E60" s="1" t="s">
-        <x:v>352</x:v>
+        <x:v>350</x:v>
       </x:c>
     </x:row>
     <x:row r="61">
       <x:c r="A61" s="1" t="s">
-        <x:v>355</x:v>
+        <x:v>353</x:v>
       </x:c>
       <x:c r="B61" s="1" t="s">
-        <x:v>259</x:v>
+        <x:v>257</x:v>
       </x:c>
       <x:c r="C61" s="1" t="s">
-        <x:v>356</x:v>
+        <x:v>354</x:v>
       </x:c>
       <x:c r="D61" s="1" t="s">
         <x:v>28</x:v>
@@ -24389,13 +24383,13 @@
     </x:row>
     <x:row r="62">
       <x:c r="A62" s="21" t="s">
-        <x:v>357</x:v>
+        <x:v>355</x:v>
       </x:c>
       <x:c r="B62" s="21" t="s">
         <x:v>27</x:v>
       </x:c>
       <x:c r="C62" s="1" t="s">
-        <x:v>358</x:v>
+        <x:v>356</x:v>
       </x:c>
       <x:c r="D62" s="1" t="s">
         <x:v>28</x:v>
@@ -24404,173 +24398,173 @@
         <x:v>28</x:v>
       </x:c>
       <x:c r="J62" s="1" t="s">
-        <x:v>359</x:v>
+        <x:v>357</x:v>
       </x:c>
     </x:row>
     <x:row r="63">
       <x:c r="A63" s="1" t="s">
-        <x:v>360</x:v>
+        <x:v>358</x:v>
       </x:c>
       <x:c r="B63" s="1" t="s">
-        <x:v>259</x:v>
+        <x:v>257</x:v>
       </x:c>
       <x:c r="C63" s="1" t="s">
-        <x:v>361</x:v>
+        <x:v>359</x:v>
       </x:c>
       <x:c r="D63" s="1" t="s">
-        <x:v>109</x:v>
+        <x:v>107</x:v>
       </x:c>
       <x:c r="E63" s="1" t="s">
-        <x:v>109</x:v>
+        <x:v>107</x:v>
       </x:c>
     </x:row>
     <x:row r="64">
       <x:c r="A64" s="1" t="s">
-        <x:v>362</x:v>
+        <x:v>360</x:v>
       </x:c>
       <x:c r="B64" s="1" t="s">
         <x:v>27</x:v>
       </x:c>
       <x:c r="C64" s="1" t="s">
-        <x:v>363</x:v>
+        <x:v>361</x:v>
       </x:c>
       <x:c r="D64" s="1" t="s">
-        <x:v>98</x:v>
+        <x:v>96</x:v>
       </x:c>
       <x:c r="E64" s="1" t="s">
-        <x:v>98</x:v>
+        <x:v>96</x:v>
       </x:c>
     </x:row>
     <x:row r="65">
       <x:c r="A65" s="1" t="s">
-        <x:v>364</x:v>
+        <x:v>362</x:v>
       </x:c>
       <x:c r="B65" s="1" t="s">
         <x:v>27</x:v>
       </x:c>
       <x:c r="C65" s="1" t="s">
-        <x:v>365</x:v>
+        <x:v>363</x:v>
       </x:c>
       <x:c r="D65" s="1" t="s">
-        <x:v>366</x:v>
+        <x:v>364</x:v>
       </x:c>
       <x:c r="E65" s="1" t="s">
-        <x:v>71</x:v>
+        <x:v>69</x:v>
       </x:c>
       <x:c r="F65" s="1" t="s">
-        <x:v>72</x:v>
+        <x:v>70</x:v>
       </x:c>
     </x:row>
     <x:row r="66">
       <x:c r="A66" s="1" t="s">
-        <x:v>367</x:v>
+        <x:v>365</x:v>
       </x:c>
       <x:c r="B66" s="1" t="s">
         <x:v>27</x:v>
       </x:c>
       <x:c r="C66" s="1" t="s">
-        <x:v>368</x:v>
+        <x:v>366</x:v>
       </x:c>
       <x:c r="D66" s="1" t="s">
-        <x:v>366</x:v>
+        <x:v>364</x:v>
       </x:c>
       <x:c r="E66" s="1" t="s">
-        <x:v>71</x:v>
+        <x:v>69</x:v>
       </x:c>
       <x:c r="F66" s="1" t="s">
-        <x:v>72</x:v>
+        <x:v>70</x:v>
       </x:c>
     </x:row>
     <x:row r="67">
       <x:c r="A67" s="1" t="s">
-        <x:v>369</x:v>
+        <x:v>367</x:v>
       </x:c>
       <x:c r="B67" s="1" t="s">
         <x:v>27</x:v>
       </x:c>
       <x:c r="C67" s="1" t="s">
-        <x:v>370</x:v>
+        <x:v>368</x:v>
       </x:c>
       <x:c r="D67" s="1" t="s">
-        <x:v>366</x:v>
+        <x:v>364</x:v>
       </x:c>
       <x:c r="E67" s="1" t="s">
-        <x:v>71</x:v>
+        <x:v>69</x:v>
       </x:c>
       <x:c r="F67" s="1" t="s">
-        <x:v>72</x:v>
+        <x:v>70</x:v>
       </x:c>
     </x:row>
     <x:row r="68">
       <x:c r="A68" s="1" t="s">
-        <x:v>371</x:v>
+        <x:v>369</x:v>
       </x:c>
       <x:c r="B68" s="1" t="s">
         <x:v>27</x:v>
       </x:c>
       <x:c r="C68" s="1" t="s">
-        <x:v>372</x:v>
+        <x:v>370</x:v>
       </x:c>
       <x:c r="D68" s="1" t="s">
-        <x:v>373</x:v>
+        <x:v>371</x:v>
       </x:c>
       <x:c r="E68" s="1" t="s">
-        <x:v>71</x:v>
+        <x:v>69</x:v>
       </x:c>
       <x:c r="F68" s="1" t="s">
-        <x:v>72</x:v>
+        <x:v>70</x:v>
       </x:c>
     </x:row>
     <x:row r="69">
       <x:c r="A69" s="1" t="s">
-        <x:v>374</x:v>
+        <x:v>372</x:v>
       </x:c>
       <x:c r="B69" s="1" t="s">
         <x:v>27</x:v>
       </x:c>
       <x:c r="C69" s="1" t="s">
-        <x:v>375</x:v>
+        <x:v>373</x:v>
       </x:c>
       <x:c r="D69" s="1" t="s">
-        <x:v>376</x:v>
+        <x:v>374</x:v>
       </x:c>
       <x:c r="E69" s="1" t="s">
-        <x:v>71</x:v>
+        <x:v>69</x:v>
       </x:c>
       <x:c r="F69" s="1" t="s">
-        <x:v>72</x:v>
+        <x:v>70</x:v>
       </x:c>
     </x:row>
     <x:row r="70">
       <x:c r="A70" s="1" t="s">
-        <x:v>377</x:v>
+        <x:v>375</x:v>
       </x:c>
       <x:c r="B70" s="1" t="s">
         <x:v>27</x:v>
       </x:c>
       <x:c r="C70" s="1" t="s">
-        <x:v>378</x:v>
+        <x:v>376</x:v>
       </x:c>
       <x:c r="D70" s="1" t="s">
-        <x:v>379</x:v>
+        <x:v>377</x:v>
       </x:c>
       <x:c r="E70" s="1" t="s">
-        <x:v>71</x:v>
+        <x:v>69</x:v>
       </x:c>
       <x:c r="F70" s="1" t="s">
-        <x:v>72</x:v>
+        <x:v>70</x:v>
       </x:c>
       <x:c r="G70" s="1"/>
     </x:row>
     <x:row r="71">
       <x:c r="A71" s="1" t="s">
-        <x:v>380</x:v>
+        <x:v>378</x:v>
       </x:c>
       <x:c r="B71" s="1" t="s">
         <x:v>27</x:v>
       </x:c>
       <x:c r="C71" s="1" t="s">
-        <x:v>381</x:v>
+        <x:v>379</x:v>
       </x:c>
       <x:c r="D71" s="1" t="s">
         <x:v>28</x:v>
@@ -24581,13 +24575,13 @@
     </x:row>
     <x:row r="72">
       <x:c r="A72" s="1" t="s">
-        <x:v>382</x:v>
+        <x:v>380</x:v>
       </x:c>
       <x:c r="B72" s="1" t="s">
         <x:v>27</x:v>
       </x:c>
       <x:c r="C72" s="1" t="s">
-        <x:v>383</x:v>
+        <x:v>381</x:v>
       </x:c>
       <x:c r="D72" s="1" t="s">
         <x:v>28</x:v>
@@ -24598,70 +24592,70 @@
     </x:row>
     <x:row r="73">
       <x:c r="A73" s="1" t="s">
-        <x:v>384</x:v>
+        <x:v>382</x:v>
       </x:c>
       <x:c r="B73" s="1" t="s">
         <x:v>27</x:v>
       </x:c>
       <x:c r="C73" s="1" t="s">
-        <x:v>385</x:v>
+        <x:v>383</x:v>
       </x:c>
       <x:c r="D73" s="1" t="s">
-        <x:v>386</x:v>
+        <x:v>384</x:v>
       </x:c>
       <x:c r="E73" s="1" t="s">
-        <x:v>71</x:v>
+        <x:v>69</x:v>
       </x:c>
       <x:c r="F73" s="1" t="s">
-        <x:v>72</x:v>
+        <x:v>70</x:v>
       </x:c>
     </x:row>
     <x:row r="74">
       <x:c r="A74" s="1" t="s">
-        <x:v>387</x:v>
+        <x:v>385</x:v>
       </x:c>
       <x:c r="B74" s="1" t="s">
-        <x:v>259</x:v>
+        <x:v>257</x:v>
       </x:c>
       <x:c r="C74" s="1" t="s">
-        <x:v>388</x:v>
+        <x:v>386</x:v>
       </x:c>
       <x:c r="D74" s="1" t="s">
-        <x:v>109</x:v>
+        <x:v>107</x:v>
       </x:c>
       <x:c r="E74" s="1" t="s">
-        <x:v>109</x:v>
+        <x:v>107</x:v>
       </x:c>
     </x:row>
     <x:row r="75">
       <x:c r="A75" s="1" t="s">
-        <x:v>389</x:v>
+        <x:v>387</x:v>
       </x:c>
       <x:c r="B75" s="1" t="s">
-        <x:v>259</x:v>
+        <x:v>257</x:v>
       </x:c>
       <x:c r="C75" s="1" t="s">
-        <x:v>390</x:v>
+        <x:v>388</x:v>
       </x:c>
       <x:c r="D75" s="1" t="s">
-        <x:v>109</x:v>
+        <x:v>107</x:v>
       </x:c>
       <x:c r="E75" s="1" t="s">
-        <x:v>109</x:v>
+        <x:v>107</x:v>
       </x:c>
     </x:row>
     <x:row r="76">
       <x:c r="A76" s="1" t="s">
-        <x:v>391</x:v>
+        <x:v>389</x:v>
       </x:c>
       <x:c r="B76" s="1" t="s">
         <x:v>27</x:v>
       </x:c>
       <x:c r="C76" s="1" t="s">
-        <x:v>392</x:v>
+        <x:v>390</x:v>
       </x:c>
       <x:c r="D76" s="1" t="s">
-        <x:v>197</x:v>
+        <x:v>195</x:v>
       </x:c>
       <x:c r="E76" s="1" t="s">
         <x:v>28</x:v>
@@ -24669,13 +24663,13 @@
     </x:row>
     <x:row r="77">
       <x:c r="A77" s="1" t="s">
-        <x:v>393</x:v>
+        <x:v>391</x:v>
       </x:c>
       <x:c r="B77" s="1" t="s">
         <x:v>27</x:v>
       </x:c>
       <x:c r="C77" s="1" t="s">
-        <x:v>394</x:v>
+        <x:v>392</x:v>
       </x:c>
       <x:c r="D77" s="1" t="s">
         <x:v>28</x:v>
@@ -24686,13 +24680,13 @@
     </x:row>
     <x:row r="78">
       <x:c r="A78" s="1" t="s">
-        <x:v>395</x:v>
+        <x:v>393</x:v>
       </x:c>
       <x:c r="B78" s="1" t="s">
         <x:v>27</x:v>
       </x:c>
       <x:c r="C78" s="1" t="s">
-        <x:v>396</x:v>
+        <x:v>394</x:v>
       </x:c>
       <x:c r="D78" s="1" t="s">
         <x:v>28</x:v>
@@ -24703,62 +24697,62 @@
     </x:row>
     <x:row r="79" ht="15.75" hidden="0" customHeight="1">
       <x:c r="A79" s="1" t="s">
-        <x:v>397</x:v>
+        <x:v>395</x:v>
       </x:c>
       <x:c r="B79" s="1" t="s">
         <x:v>27</x:v>
       </x:c>
       <x:c r="C79" s="1" t="s">
-        <x:v>398</x:v>
+        <x:v>396</x:v>
       </x:c>
       <x:c r="D79" s="1" t="s">
-        <x:v>399</x:v>
+        <x:v>397</x:v>
       </x:c>
       <x:c r="E79" s="1" t="s">
-        <x:v>71</x:v>
+        <x:v>69</x:v>
       </x:c>
       <x:c r="F79" s="1" t="s">
-        <x:v>72</x:v>
+        <x:v>70</x:v>
       </x:c>
     </x:row>
     <x:row r="80" ht="15.75" hidden="0" customHeight="1">
       <x:c r="A80" s="1" t="s">
-        <x:v>400</x:v>
+        <x:v>398</x:v>
       </x:c>
       <x:c r="B80" s="1" t="s">
         <x:v>27</x:v>
       </x:c>
       <x:c r="C80" s="1" t="s">
-        <x:v>401</x:v>
+        <x:v>399</x:v>
       </x:c>
       <x:c r="D80" s="1" t="s">
-        <x:v>98</x:v>
+        <x:v>96</x:v>
       </x:c>
       <x:c r="E80" s="1" t="s">
-        <x:v>98</x:v>
+        <x:v>96</x:v>
       </x:c>
     </x:row>
     <x:row r="81" ht="15.75" hidden="0" customHeight="1">
       <x:c r="A81" s="1" t="s">
-        <x:v>402</x:v>
+        <x:v>400</x:v>
       </x:c>
       <x:c r="B81" s="20"/>
       <x:c r="D81" s="1" t="s">
-        <x:v>109</x:v>
+        <x:v>107</x:v>
       </x:c>
       <x:c r="E81" s="1" t="s">
-        <x:v>109</x:v>
+        <x:v>107</x:v>
       </x:c>
     </x:row>
     <x:row r="82" ht="15.75" hidden="0" customHeight="1">
       <x:c r="A82" s="1" t="s">
-        <x:v>403</x:v>
+        <x:v>401</x:v>
       </x:c>
       <x:c r="B82" s="1" t="s">
         <x:v>27</x:v>
       </x:c>
       <x:c r="C82" s="1" t="s">
-        <x:v>404</x:v>
+        <x:v>402</x:v>
       </x:c>
       <x:c r="D82" s="1" t="s">
         <x:v>28</x:v>
@@ -24769,16 +24763,16 @@
     </x:row>
     <x:row r="83" ht="60" hidden="0" customHeight="1">
       <x:c r="A83" s="1" t="s">
-        <x:v>405</x:v>
+        <x:v>403</x:v>
       </x:c>
       <x:c r="B83" s="1" t="s">
         <x:v>27</x:v>
       </x:c>
       <x:c r="C83" s="1" t="s">
-        <x:v>406</x:v>
+        <x:v>404</x:v>
       </x:c>
       <x:c r="D83" s="1" t="s">
-        <x:v>407</x:v>
+        <x:v>405</x:v>
       </x:c>
       <x:c r="E83" s="1" t="str">
         <x:v>multi-select choice</x:v>
@@ -24793,100 +24787,100 @@
     </x:row>
     <x:row r="84" ht="15.75" hidden="0" customHeight="1">
       <x:c r="A84" s="1" t="s">
-        <x:v>408</x:v>
+        <x:v>406</x:v>
       </x:c>
       <x:c r="B84" s="21"/>
       <x:c r="D84" s="1" t="s">
-        <x:v>408</x:v>
+        <x:v>406</x:v>
       </x:c>
       <x:c r="E84" s="1" t="s">
-        <x:v>71</x:v>
+        <x:v>69</x:v>
       </x:c>
       <x:c r="F84" s="1" t="s">
-        <x:v>72</x:v>
+        <x:v>70</x:v>
       </x:c>
     </x:row>
     <x:row r="85" ht="15.75" hidden="0" customHeight="1">
       <x:c r="A85" s="1" t="s">
-        <x:v>409</x:v>
+        <x:v>407</x:v>
       </x:c>
       <x:c r="B85" s="20"/>
       <x:c r="D85" s="1" t="s">
-        <x:v>109</x:v>
+        <x:v>107</x:v>
       </x:c>
       <x:c r="E85" s="1" t="s">
-        <x:v>109</x:v>
+        <x:v>107</x:v>
       </x:c>
     </x:row>
     <x:row r="86">
       <x:c r="A86" s="1" t="s">
-        <x:v>410</x:v>
+        <x:v>408</x:v>
       </x:c>
       <x:c r="B86" s="20"/>
       <x:c r="D86" s="1" t="s">
-        <x:v>109</x:v>
+        <x:v>107</x:v>
       </x:c>
       <x:c r="E86" s="1" t="s">
-        <x:v>109</x:v>
+        <x:v>107</x:v>
       </x:c>
     </x:row>
     <x:row r="87">
       <x:c r="A87" s="1" t="s">
-        <x:v>411</x:v>
+        <x:v>409</x:v>
       </x:c>
       <x:c r="B87" s="20"/>
       <x:c r="D87" s="1" t="s">
-        <x:v>109</x:v>
+        <x:v>107</x:v>
       </x:c>
       <x:c r="E87" s="1" t="s">
-        <x:v>109</x:v>
+        <x:v>107</x:v>
       </x:c>
     </x:row>
     <x:row r="88">
       <x:c r="A88" s="1" t="s">
-        <x:v>412</x:v>
+        <x:v>410</x:v>
       </x:c>
       <x:c r="B88" s="20"/>
       <x:c r="D88" s="1" t="s">
-        <x:v>109</x:v>
+        <x:v>107</x:v>
       </x:c>
       <x:c r="E88" s="1" t="s">
-        <x:v>109</x:v>
+        <x:v>107</x:v>
       </x:c>
     </x:row>
     <x:row r="89">
       <x:c r="A89" s="1" t="s">
-        <x:v>413</x:v>
+        <x:v>411</x:v>
       </x:c>
       <x:c r="B89" s="20"/>
       <x:c r="D89" s="1" t="s">
-        <x:v>109</x:v>
+        <x:v>107</x:v>
       </x:c>
       <x:c r="E89" s="1" t="s">
-        <x:v>109</x:v>
+        <x:v>107</x:v>
       </x:c>
     </x:row>
     <x:row r="90">
       <x:c r="A90" s="1" t="s">
-        <x:v>414</x:v>
+        <x:v>412</x:v>
       </x:c>
       <x:c r="B90" s="20"/>
       <x:c r="D90" s="1" t="s">
-        <x:v>109</x:v>
+        <x:v>107</x:v>
       </x:c>
       <x:c r="E90" s="1" t="s">
-        <x:v>109</x:v>
+        <x:v>107</x:v>
       </x:c>
     </x:row>
     <x:row r="91">
       <x:c r="A91" s="1" t="s">
-        <x:v>415</x:v>
+        <x:v>413</x:v>
       </x:c>
       <x:c r="B91" s="1" t="s">
         <x:v>27</x:v>
       </x:c>
       <x:c r="C91" s="1" t="s">
-        <x:v>416</x:v>
+        <x:v>414</x:v>
       </x:c>
       <x:c r="D91" s="1" t="s">
         <x:v>28</x:v>
@@ -24897,13 +24891,13 @@
     </x:row>
     <x:row r="92">
       <x:c r="A92" s="1" t="s">
-        <x:v>417</x:v>
+        <x:v>415</x:v>
       </x:c>
       <x:c r="B92" s="1" t="s">
         <x:v>27</x:v>
       </x:c>
       <x:c r="C92" s="1" t="s">
-        <x:v>418</x:v>
+        <x:v>416</x:v>
       </x:c>
       <x:c r="D92" s="1" t="s">
         <x:v>28</x:v>
@@ -24914,36 +24908,36 @@
     </x:row>
     <x:row r="93">
       <x:c r="A93" s="1" t="s">
-        <x:v>419</x:v>
+        <x:v>417</x:v>
       </x:c>
       <x:c r="B93" s="1" t="s">
         <x:v>27</x:v>
       </x:c>
       <x:c r="C93" s="1" t="s">
-        <x:v>420</x:v>
+        <x:v>418</x:v>
       </x:c>
       <x:c r="D93" s="1" t="s">
-        <x:v>98</x:v>
+        <x:v>96</x:v>
       </x:c>
       <x:c r="E93" s="1" t="s">
-        <x:v>98</x:v>
+        <x:v>96</x:v>
       </x:c>
     </x:row>
     <x:row r="94">
       <x:c r="A94" s="1" t="s">
-        <x:v>421</x:v>
+        <x:v>419</x:v>
       </x:c>
       <x:c r="B94" s="1" t="s">
         <x:v>27</x:v>
       </x:c>
       <x:c r="C94" s="1" t="s">
-        <x:v>422</x:v>
+        <x:v>420</x:v>
       </x:c>
       <x:c r="D94" s="1" t="s">
-        <x:v>98</x:v>
+        <x:v>96</x:v>
       </x:c>
       <x:c r="E94" s="1" t="s">
-        <x:v>71</x:v>
+        <x:v>69</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>

<commit_message>
env var changes, workbook update
</commit_message>
<xml_diff>
--- a/apps/it-governance/migrations/IT Governance Intake Request Mapping Workbook.xlsx
+++ b/apps/it-governance/migrations/IT Governance Intake Request Mapping Workbook.xlsx
@@ -2,20 +2,21 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="business_cases" sheetId="1" r:id="Rc7b2f01f33784cba"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="estimated_lifecycle_costs" sheetId="2" r:id="Rf2969f0a5b224510"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="governance_request_feedback" sheetId="3" r:id="Ra0b71d44cc064aaf"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="system_intake_contacts" sheetId="4" r:id="Rb8b03b1ea2b34805"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="system_intake_contract_numbers" sheetId="5" r:id="R7392fc91e840441a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="system_intake_documents" sheetId="6" r:id="R811e4e684535433f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="system_intake_funding_sources" sheetId="7" r:id="Ra3297d96dfbc47e6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="system_intake_systems" sheetId="8" r:id="R85c516b2e59c404a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="system_intakes" sheetId="9" r:id="R9c43572cbcf64583"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="system_intake_grb_reviewers" sheetId="10" r:id="Ra48ab4cc11dc4cde"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="system_intake_grb_presentation_" sheetId="11" r:id="R17c8e4c2e521400c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="system_intake_internal_grb_revi" sheetId="12" r:id="R8f73ed2542904c85"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mapping Governance" sheetId="14" r:id="R9ccec4dd651d4ec1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Migration Next Steps" sheetId="15" r:id="R6b0b34e7a49d4e05"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="business_cases" sheetId="1" r:id="R4c0e05dd8d564456"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="estimated_lifecycle_costs" sheetId="2" r:id="R46d827310cbf4e9e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="governance_request_feedback" sheetId="3" r:id="R0937f9f2af1346f0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="system_intake_contacts" sheetId="4" r:id="R37d521410ed84e4d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="system_intake_contract_numbers" sheetId="5" r:id="Rcd9777f15a784357"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="system_intake_documents" sheetId="6" r:id="Rcbf8aec0b8d2431e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="system_intake_funding_sources" sheetId="7" r:id="R5ad4e746d3b54260"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="system_intake_systems" sheetId="8" r:id="R917a08d3c5494ba5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="system_intakes" sheetId="9" r:id="R157d24d0a21140fa"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="system_intake_grb_reviewers" sheetId="10" r:id="Rc6ee34a584174da3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="system_intake_grb_presentation_" sheetId="11" r:id="R31cd0dc50b0145ea"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="system_intake_internal_grb_revi" sheetId="12" r:id="R5b9b3ce4572b4110"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mapping Governance" sheetId="14" r:id="R37e6118ab8624bb6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Migration Next Steps" sheetId="15" r:id="R1daa560f99b1479d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="notes" sheetId="16" r:id="Rf2741c72856647e7"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1366,7 +1367,7 @@
     <x:numFmt numFmtId="200" formatCode="0"/>
     <x:numFmt numFmtId="201" formatCode="yyyy-mm-dd"/>
   </x:numFmts>
-  <x:fonts count="11">
+  <x:fonts count="14">
     <x:font>
       <x:sz val="10"/>
       <x:color rgb="FF000000"/>
@@ -1425,6 +1426,23 @@
     <x:font>
       <x:sz val="10"/>
       <x:color rgb="FF222222"/>
+      <x:name val="Arial"/>
+    </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="10"/>
+      <x:color rgb="FF000000"/>
+      <x:name val="Arial"/>
+    </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="10"/>
+      <x:color theme="1"/>
+      <x:name val="Arial"/>
+    </x:font>
+    <x:font>
+      <x:sz val="10"/>
+      <x:color theme="1"/>
       <x:name val="Arial"/>
     </x:font>
   </x:fonts>
@@ -1701,7 +1719,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="1" applyAlignment="1"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="132">
+  <x:cellXfs count="165">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <x:alignment vertical="bottom" wrapText="0"/>
     </x:xf>
@@ -2082,6 +2100,103 @@
     <x:xf numFmtId="200" fontId="10" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="center" vertical="top" wrapText="1"/>
     </x:xf>
+    <x:xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="bottom" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="left"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="left" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="bottom" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="left" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="left" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
@@ -2250,6 +2365,25 @@
     <x:tableColumn id="6" name="Downstream finding"/>
     <x:tableColumn id="7" name="Status"/>
     <x:tableColumn id="8" name="Verification"/>
+  </x:tableColumns>
+  <x:tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</x:table>
+</file>
+
+<file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="NotesMappingTable" displayName="NotesMappingTable" ref="A5:K15" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:tableColumns count="11">
+    <x:tableColumn id="1" name="Column"/>
+    <x:tableColumn id="2" name="Staging Column"/>
+    <x:tableColumn id="3" name="Staging Table"/>
+    <x:tableColumn id="4" name="Source Datatype"/>
+    <x:tableColumn id="5" name="Staging Datatype"/>
+    <x:tableColumn id="6" name="Transformed?"/>
+    <x:tableColumn id="7" name="IMPL Max Length"/>
+    <x:tableColumn id="8" name="Staging Text Field Size"/>
+    <x:tableColumn id="9" name="Planned Final Target"/>
+    <x:tableColumn id="10" name="Notes"/>
+    <x:tableColumn id="11" name="Is this Legacy Data?"/>
   </x:tableColumns>
   <x:tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </x:table>
@@ -10374,7 +10508,472 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R910fc0c6de8d4420"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R81f9eb96071e405c"/>
+  </x:tableParts>
+</x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
+    <x:col min="1" max="1" width="22" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="26" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="20" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="22" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="20" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="15" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="18" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="18" hidden="0" customWidth="1"/>
+    <x:col min="9" max="9" width="27" hidden="0" customWidth="1"/>
+    <x:col min="10" max="10" width="58" hidden="0" customWidth="1"/>
+    <x:col min="11" max="11" width="18" hidden="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1">
+      <x:c r="A1" s="154" t="str">
+        <x:v>Postgresql Table</x:v>
+      </x:c>
+      <x:c r="B1" s="155" t="str">
+        <x:v>notes</x:v>
+      </x:c>
+      <x:c r="C1" s="142"/>
+      <x:c r="D1" s="142"/>
+      <x:c r="E1" s="142"/>
+      <x:c r="F1" s="156"/>
+      <x:c r="G1" s="156"/>
+      <x:c r="H1" s="157"/>
+      <x:c r="I1" s="157"/>
+      <x:c r="J1" s="142"/>
+      <x:c r="K1" s="142"/>
+    </x:row>
+    <x:row r="2">
+      <x:c r="A2" s="154" t="str">
+        <x:v>Staging Table</x:v>
+      </x:c>
+      <x:c r="B2" s="155" t="str">
+        <x:v>new_stagenote</x:v>
+      </x:c>
+      <x:c r="C2" s="142"/>
+      <x:c r="D2" s="142"/>
+      <x:c r="E2" s="142"/>
+      <x:c r="F2" s="156"/>
+      <x:c r="G2" s="156"/>
+      <x:c r="H2" s="157"/>
+      <x:c r="I2" s="157"/>
+      <x:c r="J2" s="142"/>
+      <x:c r="K2" s="142"/>
+    </x:row>
+    <x:row r="3" ht="32" customHeight="1">
+      <x:c r="A3" s="154" t="str">
+        <x:v>Notes</x:v>
+      </x:c>
+      <x:c r="B3" s="158" t="str">
+        <x:v>Stage Notes loads source rows into new_stagenote. Power Automate later creates native Notes and associates them with Reviews. NotesQA flags blank, archived, and suspicious content.</x:v>
+      </x:c>
+      <x:c r="C3" s="151"/>
+      <x:c r="D3" s="158"/>
+      <x:c r="E3" s="158"/>
+      <x:c r="F3" s="158"/>
+      <x:c r="G3" s="158"/>
+      <x:c r="H3" s="159"/>
+      <x:c r="I3" s="159"/>
+      <x:c r="J3" s="151"/>
+      <x:c r="K3" s="151"/>
+    </x:row>
+    <x:row r="4">
+      <x:c r="A4" s="142"/>
+      <x:c r="B4" s="154"/>
+      <x:c r="C4" s="154"/>
+      <x:c r="D4" s="154"/>
+      <x:c r="E4" s="154"/>
+      <x:c r="F4" s="154"/>
+      <x:c r="G4" s="154"/>
+      <x:c r="H4" s="160"/>
+      <x:c r="I4" s="161"/>
+      <x:c r="J4" s="154"/>
+      <x:c r="K4" s="142"/>
+    </x:row>
+    <x:row r="5" ht="32" customHeight="1">
+      <x:c r="A5" s="148" t="str">
+        <x:v>Column</x:v>
+      </x:c>
+      <x:c r="B5" s="162" t="str">
+        <x:v>Staging Column</x:v>
+      </x:c>
+      <x:c r="C5" s="162" t="str">
+        <x:v>Staging Table</x:v>
+      </x:c>
+      <x:c r="D5" s="162" t="str">
+        <x:v>Source Datatype</x:v>
+      </x:c>
+      <x:c r="E5" s="162" t="str">
+        <x:v>Staging Datatype</x:v>
+      </x:c>
+      <x:c r="F5" s="162" t="str">
+        <x:v>Transformed?</x:v>
+      </x:c>
+      <x:c r="G5" s="162" t="str">
+        <x:v>IMPL Max Length</x:v>
+      </x:c>
+      <x:c r="H5" s="162" t="str">
+        <x:v>Staging Text Field Size</x:v>
+      </x:c>
+      <x:c r="I5" s="163" t="str">
+        <x:v>Planned Final Target</x:v>
+      </x:c>
+      <x:c r="J5" s="163" t="str">
+        <x:v>Notes</x:v>
+      </x:c>
+      <x:c r="K5" s="162" t="str">
+        <x:v>Is this Legacy Data?</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6" ht="42" customHeight="1">
+      <x:c r="A6" s="164" t="str">
+        <x:v>id</x:v>
+      </x:c>
+      <x:c r="B6" s="164" t="str">
+        <x:v>new_legacynoteid</x:v>
+      </x:c>
+      <x:c r="C6" s="164" t="str">
+        <x:v>new_stagenote</x:v>
+      </x:c>
+      <x:c r="D6" s="164" t="str">
+        <x:v>uuid</x:v>
+      </x:c>
+      <x:c r="E6" s="164" t="str">
+        <x:v>text (required)</x:v>
+      </x:c>
+      <x:c r="F6" s="142"/>
+      <x:c r="G6" s="142" t="n">
+        <x:v>36</x:v>
+      </x:c>
+      <x:c r="H6" s="157" t="n">
+        <x:v>100</x:v>
+      </x:c>
+      <x:c r="I6" s="157" t="str">
+        <x:v>annotation.subject marker</x:v>
+      </x:c>
+      <x:c r="J6" s="151" t="str">
+        <x:v>Primary name column. Used for QA and planned migration idempotency marker.</x:v>
+      </x:c>
+      <x:c r="K6" s="142" t="str">
+        <x:v>yes</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7" ht="42" customHeight="1">
+      <x:c r="A7" s="164" t="str">
+        <x:v>system_intake</x:v>
+      </x:c>
+      <x:c r="B7" s="164" t="str">
+        <x:v>new_systemintakeid</x:v>
+      </x:c>
+      <x:c r="C7" s="164" t="str">
+        <x:v>new_stagenote</x:v>
+      </x:c>
+      <x:c r="D7" s="164" t="str">
+        <x:v>uuid</x:v>
+      </x:c>
+      <x:c r="E7" s="164" t="str">
+        <x:v>text</x:v>
+      </x:c>
+      <x:c r="F7" s="142"/>
+      <x:c r="G7" s="142" t="n">
+        <x:v>36</x:v>
+      </x:c>
+      <x:c r="H7" s="157" t="n">
+        <x:v>100</x:v>
+      </x:c>
+      <x:c r="I7" s="157" t="str">
+        <x:v>annotation.objectid (Review)</x:v>
+      </x:c>
+      <x:c r="J7" s="151" t="str">
+        <x:v>Power Automate resolves the legacy System Intake to the migrated Request and related Review.</x:v>
+      </x:c>
+      <x:c r="K7" s="142" t="str">
+        <x:v>yes</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8" ht="42" customHeight="1">
+      <x:c r="A8" s="164" t="str">
+        <x:v>created_at</x:v>
+      </x:c>
+      <x:c r="B8" s="164" t="str">
+        <x:v>new_createdatlegacy</x:v>
+      </x:c>
+      <x:c r="C8" s="164" t="str">
+        <x:v>new_stagenote</x:v>
+      </x:c>
+      <x:c r="D8" s="164" t="str">
+        <x:v>timestamp with time zone</x:v>
+      </x:c>
+      <x:c r="E8" s="164" t="str">
+        <x:v>date and time</x:v>
+      </x:c>
+      <x:c r="F8" s="164" t="str">
+        <x:v>yes</x:v>
+      </x:c>
+      <x:c r="G8" s="142" t="n">
+        <x:v>29</x:v>
+      </x:c>
+      <x:c r="H8" s="157" t="str">
+        <x:v>n/a</x:v>
+      </x:c>
+      <x:c r="I8" s="157" t="str">
+        <x:v>annotation.overriddencreatedon</x:v>
+      </x:c>
+      <x:c r="J8" s="151" t="str">
+        <x:v>Parsed safely as UTC. Invalid or pre-1753 values are reported by NotesQA.</x:v>
+      </x:c>
+      <x:c r="K8" s="142" t="str">
+        <x:v>yes</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9" ht="42" customHeight="1">
+      <x:c r="A9" s="164" t="str">
+        <x:v>eua_user_id</x:v>
+      </x:c>
+      <x:c r="B9" s="164" t="str">
+        <x:v>new_euauserid</x:v>
+      </x:c>
+      <x:c r="C9" s="164" t="str">
+        <x:v>new_stagenote</x:v>
+      </x:c>
+      <x:c r="D9" s="164" t="str">
+        <x:v>text</x:v>
+      </x:c>
+      <x:c r="E9" s="164" t="str">
+        <x:v>text</x:v>
+      </x:c>
+      <x:c r="F9" s="142"/>
+      <x:c r="G9" s="142" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="H9" s="157" t="n">
+        <x:v>100</x:v>
+      </x:c>
+      <x:c r="I9" s="157" t="str">
+        <x:v>Pending migration policy</x:v>
+      </x:c>
+      <x:c r="J9" s="151" t="str">
+        <x:v>Original author identifier. Native annotation.createdby cannot be set directly.</x:v>
+      </x:c>
+      <x:c r="K9" s="142" t="str">
+        <x:v>yes</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="10" ht="42" customHeight="1">
+      <x:c r="A10" s="164" t="str">
+        <x:v>author_name</x:v>
+      </x:c>
+      <x:c r="B10" s="164" t="str">
+        <x:v>new_authorname</x:v>
+      </x:c>
+      <x:c r="C10" s="164" t="str">
+        <x:v>new_stagenote</x:v>
+      </x:c>
+      <x:c r="D10" s="164" t="str">
+        <x:v>text</x:v>
+      </x:c>
+      <x:c r="E10" s="164" t="str">
+        <x:v>text</x:v>
+      </x:c>
+      <x:c r="F10" s="142"/>
+      <x:c r="G10" s="142" t="n">
+        <x:v>310</x:v>
+      </x:c>
+      <x:c r="H10" s="157" t="n">
+        <x:v>500</x:v>
+      </x:c>
+      <x:c r="I10" s="157" t="str">
+        <x:v>Pending migration policy</x:v>
+      </x:c>
+      <x:c r="J10" s="151" t="str">
+        <x:v>IMPL includes formula-style and HTML security-test values; NotesQA flags suspicious content.</x:v>
+      </x:c>
+      <x:c r="K10" s="142" t="str">
+        <x:v>yes</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="11" ht="42" customHeight="1">
+      <x:c r="A11" s="164" t="str">
+        <x:v>content</x:v>
+      </x:c>
+      <x:c r="B11" s="164" t="str">
+        <x:v>new_content</x:v>
+      </x:c>
+      <x:c r="C11" s="164" t="str">
+        <x:v>new_stagenote</x:v>
+      </x:c>
+      <x:c r="D11" s="164" t="str">
+        <x:v>text</x:v>
+      </x:c>
+      <x:c r="E11" s="164" t="str">
+        <x:v>multiline plain text</x:v>
+      </x:c>
+      <x:c r="F11" s="142"/>
+      <x:c r="G11" s="142" t="n">
+        <x:v>768</x:v>
+      </x:c>
+      <x:c r="H11" s="157" t="n">
+        <x:v>20000</x:v>
+      </x:c>
+      <x:c r="I11" s="157" t="str">
+        <x:v>annotation.notetext</x:v>
+      </x:c>
+      <x:c r="J11" s="151" t="str">
+        <x:v>Stored as raw plain text in staging. IMPL has 14 blank values and encoded or HTML security-test content.</x:v>
+      </x:c>
+      <x:c r="K11" s="142" t="str">
+        <x:v>yes</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="12" ht="42" customHeight="1">
+      <x:c r="A12" s="164" t="str">
+        <x:v>modified_by</x:v>
+      </x:c>
+      <x:c r="B12" s="164" t="str">
+        <x:v>new_modifiedbylegacy</x:v>
+      </x:c>
+      <x:c r="C12" s="164" t="str">
+        <x:v>new_stagenote</x:v>
+      </x:c>
+      <x:c r="D12" s="164" t="str">
+        <x:v>text</x:v>
+      </x:c>
+      <x:c r="E12" s="164" t="str">
+        <x:v>text</x:v>
+      </x:c>
+      <x:c r="F12" s="164"/>
+      <x:c r="G12" s="142" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="H12" s="157" t="n">
+        <x:v>100</x:v>
+      </x:c>
+      <x:c r="I12" s="157" t="str">
+        <x:v>No direct system-field mapping</x:v>
+      </x:c>
+      <x:c r="J12" s="151" t="str">
+        <x:v>Preserved for traceability; populated on 7 IMPL rows.</x:v>
+      </x:c>
+      <x:c r="K12" s="142" t="str">
+        <x:v>yes</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="13" ht="42" customHeight="1">
+      <x:c r="A13" s="164" t="str">
+        <x:v>modified_at</x:v>
+      </x:c>
+      <x:c r="B13" s="164" t="str">
+        <x:v>new_modifiedatlegacy</x:v>
+      </x:c>
+      <x:c r="C13" s="164" t="str">
+        <x:v>new_stagenote</x:v>
+      </x:c>
+      <x:c r="D13" s="164" t="str">
+        <x:v>timestamp with time zone</x:v>
+      </x:c>
+      <x:c r="E13" s="164" t="str">
+        <x:v>date and time</x:v>
+      </x:c>
+      <x:c r="F13" s="142" t="str">
+        <x:v>yes</x:v>
+      </x:c>
+      <x:c r="G13" s="142" t="n">
+        <x:v>29</x:v>
+      </x:c>
+      <x:c r="H13" s="157" t="str">
+        <x:v>n/a</x:v>
+      </x:c>
+      <x:c r="I13" s="157" t="str">
+        <x:v>No direct system-field mapping</x:v>
+      </x:c>
+      <x:c r="J13" s="151" t="str">
+        <x:v>Parsed safely as UTC when populated; populated on 7 IMPL rows.</x:v>
+      </x:c>
+      <x:c r="K13" s="142" t="str">
+        <x:v>yes</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="14" ht="42" customHeight="1">
+      <x:c r="A14" s="164" t="str">
+        <x:v>is_archived</x:v>
+      </x:c>
+      <x:c r="B14" s="164" t="str">
+        <x:v>new_isarchived</x:v>
+      </x:c>
+      <x:c r="C14" s="164" t="str">
+        <x:v>new_stagenote</x:v>
+      </x:c>
+      <x:c r="D14" s="164" t="str">
+        <x:v>boolean</x:v>
+      </x:c>
+      <x:c r="E14" s="164" t="str">
+        <x:v>yes/no</x:v>
+      </x:c>
+      <x:c r="F14" s="142" t="str">
+        <x:v>yes</x:v>
+      </x:c>
+      <x:c r="G14" s="142" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="H14" s="157" t="str">
+        <x:v>n/a</x:v>
+      </x:c>
+      <x:c r="I14" s="157" t="str">
+        <x:v>Migration inclusion rule</x:v>
+      </x:c>
+      <x:c r="J14" s="151" t="str">
+        <x:v>IMPL contains 2 archived Notes. NotesQA flags them for an explicit migrate-or-skip decision.</x:v>
+      </x:c>
+      <x:c r="K14" s="142" t="str">
+        <x:v>yes</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="15" ht="42" customHeight="1">
+      <x:c r="A15" s="164" t="str">
+        <x:v>migrate_batch_id</x:v>
+      </x:c>
+      <x:c r="B15" s="164" t="str">
+        <x:v>new_batchid</x:v>
+      </x:c>
+      <x:c r="C15" s="164" t="str">
+        <x:v>new_stagenote</x:v>
+      </x:c>
+      <x:c r="D15" s="164" t="str">
+        <x:v>generated</x:v>
+      </x:c>
+      <x:c r="E15" s="164" t="str">
+        <x:v>text</x:v>
+      </x:c>
+      <x:c r="F15" s="142" t="str">
+        <x:v>yes</x:v>
+      </x:c>
+      <x:c r="G15" s="142" t="str">
+        <x:v>n/a</x:v>
+      </x:c>
+      <x:c r="H15" s="157" t="n">
+        <x:v>100</x:v>
+      </x:c>
+      <x:c r="I15" s="157" t="str">
+        <x:v>Rollback control</x:v>
+      </x:c>
+      <x:c r="J15" s="151" t="str">
+        <x:v>Generated from the active Migration Run. Used by the dashboard and staging rollback flow.</x:v>
+      </x:c>
+      <x:c r="K15" s="142" t="str">
+        <x:v>no</x:v>
+      </x:c>
+    </x:row>
+  </x:sheetData>
+  <x:mergeCells>
+    <x:mergeCell ref="B3:K3"/>
+  </x:mergeCells>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <x:tableParts count="1">
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf043b29abf0542b1"/>
   </x:tableParts>
 </x:worksheet>
 </file>

</xml_diff>

<commit_message>
adding images to hide puzzle pieces. updated the mapping workbook with recent changes
</commit_message>
<xml_diff>
--- a/apps/it-governance/migrations/IT Governance Intake Request Mapping Workbook.xlsx
+++ b/apps/it-governance/migrations/IT Governance Intake Request Mapping Workbook.xlsx
@@ -2,21 +2,21 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="business_cases" sheetId="1" r:id="R4c0e05dd8d564456"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="estimated_lifecycle_costs" sheetId="2" r:id="R46d827310cbf4e9e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="governance_request_feedback" sheetId="3" r:id="R0937f9f2af1346f0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="system_intake_contacts" sheetId="4" r:id="R37d521410ed84e4d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="system_intake_contract_numbers" sheetId="5" r:id="Rcd9777f15a784357"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="system_intake_documents" sheetId="6" r:id="Rcbf8aec0b8d2431e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="system_intake_funding_sources" sheetId="7" r:id="R5ad4e746d3b54260"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="system_intake_systems" sheetId="8" r:id="R917a08d3c5494ba5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="system_intakes" sheetId="9" r:id="R157d24d0a21140fa"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="system_intake_grb_reviewers" sheetId="10" r:id="Rc6ee34a584174da3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="system_intake_grb_presentation_" sheetId="11" r:id="R31cd0dc50b0145ea"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="system_intake_internal_grb_revi" sheetId="12" r:id="R5b9b3ce4572b4110"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mapping Governance" sheetId="14" r:id="R37e6118ab8624bb6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Migration Next Steps" sheetId="15" r:id="R1daa560f99b1479d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="notes" sheetId="16" r:id="Rf2741c72856647e7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="business_cases" sheetId="1" r:id="Rdc3693df614340e0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="estimated_lifecycle_costs" sheetId="2" r:id="R47099db223d74b0b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="governance_request_feedback" sheetId="3" r:id="Ree6ed805cd884d5b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="system_intake_contacts" sheetId="4" r:id="R9b7d2288d96442c2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="system_intake_contract_numbers" sheetId="5" r:id="R21f8411c4e76402b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="system_intake_documents" sheetId="6" r:id="R5c435bcbaeff4674"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="system_intake_funding_sources" sheetId="7" r:id="R4a1c555814064ba3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="system_intake_systems" sheetId="8" r:id="Rf9eaf25189994a2f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="system_intakes" sheetId="9" r:id="Re2401646dacb4bc2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="system_intake_grb_reviewers" sheetId="10" r:id="R0cfdf06928154560"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="system_intake_grb_presentation_" sheetId="11" r:id="Rc43c1b2f3f8a4bd1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="system_intake_internal_grb_revi" sheetId="12" r:id="R45def60a3dfc4c47"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mapping Governance" sheetId="14" r:id="Rc63b27af731847fc"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Migration Next Steps" sheetId="15" r:id="R7ecba3a13e4849d4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="notes" sheetId="16" r:id="R2e8a752d9362489b"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -9704,25 +9704,25 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="B2" s="113" t="str">
-        <x:v>DEV schema</x:v>
+        <x:v>UAT deployment</x:v>
       </x:c>
       <x:c r="C2" s="113" t="str">
-        <x:v>Staging Business Case</x:v>
+        <x:v>Migration solution</x:v>
       </x:c>
       <x:c r="D2" s="113" t="str">
-        <x:v>Preferred / Alternative A / Alternative B Summary</x:v>
+        <x:v>Dataflows and configuration</x:v>
       </x:c>
       <x:c r="E2" s="113" t="str">
-        <x:v>Keep all three staging summary fields at 4,000; export 1.0.0.138 confirms the family is aligned.</x:v>
+        <x:v>Deploy, then restore environment-specific dataflow configuration and connections.</x:v>
       </x:c>
       <x:c r="F2" s="113" t="str">
-        <x:v>All three map to Business Case Solution cr69a_Sumary, which already supports 4,000.</x:v>
+        <x:v>Dataflow IDs/configuration can reset during deployment.</x:v>
       </x:c>
       <x:c r="G2" s="113" t="str">
-        <x:v>Verified</x:v>
+        <x:v>In progress</x:v>
       </x:c>
       <x:c r="H2" s="114" t="str">
-        <x:v>Published managed export 1.0.0.138: Preferred, Alternative A, and Alternative B staging summaries are each 4,000; shared destination summary is 4,000.</x:v>
+        <x:v>Migration solution is deployed and all 13 staging dataflows are configured/published. Downstream migration dataflows still need connection configuration; regenerate migration IDs only after that configuration is complete.</x:v>
       </x:c>
     </x:row>
     <x:row r="3" ht="60" hidden="0" customHeight="1">
@@ -9730,25 +9730,25 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="B3" s="113" t="str">
-        <x:v>DEV schema</x:v>
+        <x:v>UAT run</x:v>
       </x:c>
       <x:c r="C3" s="113" t="str">
-        <x:v>Staging Business Case</x:v>
+        <x:v>Staging tables</x:v>
       </x:c>
       <x:c r="D3" s="113" t="str">
-        <x:v>Preferred / Alternative A / Alternative B Acquisition Approach</x:v>
+        <x:v>Fresh batch</x:v>
       </x:c>
       <x:c r="E3" s="113" t="str">
-        <x:v>Keep all three related staging fields at 20,000; export 1.0.0.138 confirms the family is aligned.</x:v>
+        <x:v>Complete rollback, then refresh staging dataflows in dependency order.</x:v>
       </x:c>
       <x:c r="F3" s="113" t="str">
-        <x:v>The shared Business Case Solution multiline destination supports 20,000; Preferred has a 10,000-character IMPL value.</x:v>
+        <x:v>A fresh batch avoids mixing partial attempts.</x:v>
       </x:c>
       <x:c r="G3" s="113" t="str">
-        <x:v>Verified</x:v>
+        <x:v>Partially verified</x:v>
       </x:c>
       <x:c r="H3" s="114" t="str">
-        <x:v>Published managed export 1.0.0.138: cr69a_preferredacquisitionapproach, cr69a_alternativeaacquisitionapproachmulti, and cr69a_alternativebacquisitionapproachmulti are each 20,000.</x:v>
+        <x:v>All staging dataflows succeeded except one System Intake row: 1,035 of 1,036 loaded. The remaining project_acronym value is invalid source data and has been cleared in a corrected source copy.</x:v>
       </x:c>
     </x:row>
     <x:row r="4" ht="48" hidden="0" customHeight="1">
@@ -9756,25 +9756,25 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="B4" s="113" t="str">
-        <x:v>DEV schema</x:v>
+        <x:v>UAT QA</x:v>
       </x:c>
       <x:c r="C4" s="113" t="str">
-        <x:v>Staging Business Case</x:v>
+        <x:v>All staged text</x:v>
       </x:c>
       <x:c r="D4" s="113" t="str">
-        <x:v>Preferred / Alternative A / Alternative B Pros</x:v>
+        <x:v>Length reconciliation</x:v>
       </x:c>
       <x:c r="E4" s="113" t="str">
-        <x:v>Map preferred, Alternative A, and Alternative B Pros only to their 20,000-character *ProsMulti staging fields; set the old single-line mappings to None. Update the downstream M inputs.</x:v>
+        <x:v>Compare source maximum lengths with staged values for every widened/replacement field.</x:v>
       </x:c>
       <x:c r="F4" s="113" t="str">
-        <x:v>Create Business Cases &amp; Solutions keeps one common Pros output and maps it to Business Case Solution cr69a_ProsMulti.</x:v>
+        <x:v>Proves values were preserved rather than silently truncated.</x:v>
       </x:c>
       <x:c r="G4" s="113" t="str">
-        <x:v>Verified</x:v>
+        <x:v>To do</x:v>
       </x:c>
       <x:c r="H4" s="114" t="str">
-        <x:v>DEV full migration succeeded after Pros mappings were moved to cr69a_preferredprosmulti, cr69a_alternativeaprosmulti, and cr69a_alternativebprosmulti. UAT staging completed without Business Case errors.</x:v>
+        <x:v>Max length and representative long values match source.</x:v>
       </x:c>
     </x:row>
     <x:row r="5" ht="48" hidden="0" customHeight="1">
@@ -9782,733 +9782,359 @@
         <x:v>4</x:v>
       </x:c>
       <x:c r="B5" s="113" t="str">
-        <x:v>DEV schema</x:v>
+        <x:v>UAT run</x:v>
       </x:c>
       <x:c r="C5" s="113" t="str">
-        <x:v>Staging Business Case</x:v>
+        <x:v>Migration dataflows</x:v>
       </x:c>
       <x:c r="D5" s="113" t="str">
-        <x:v>Preferred / Alternative A / Alternative B Cons</x:v>
+        <x:v>Create/link/update phases</x:v>
       </x:c>
       <x:c r="E5" s="113" t="str">
-        <x:v>Map preferred, Alternative A, and Alternative B Cons only to their 20,000-character *ConsMulti staging fields; set the old single-line mappings to None.</x:v>
+        <x:v>Run downstream migration only after staging passes.</x:v>
       </x:c>
       <x:c r="F5" s="113" t="str">
-        <x:v>Create Business Cases &amp; Solutions already reads the three multiline Cons staging fields and maps the common Cons output to cr69a_ConsMulti.</x:v>
+        <x:v>Destination increases are required before Request and LCID writes.</x:v>
       </x:c>
       <x:c r="G5" s="113" t="str">
-        <x:v>Verified</x:v>
+        <x:v>To do</x:v>
       </x:c>
       <x:c r="H5" s="114" t="str">
-        <x:v>DEV full migration succeeded with all three multiline Cons fields. UAT staging completed without Business Case errors.</x:v>
+        <x:v>All outputs and QA queries succeed.</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="48" hidden="0" customHeight="1">
-      <x:c r="A6" s="120" t="n">
+      <x:c r="A6" s="121" t="n">
         <x:v>5</x:v>
       </x:c>
-      <x:c r="B6" s="113" t="str">
-        <x:v>DEV schema</x:v>
-      </x:c>
-      <x:c r="C6" s="113" t="str">
-        <x:v>Staging GRB Presentation Links</x:v>
-      </x:c>
-      <x:c r="D6" s="113" t="str">
-        <x:v>cr69a_transcriptlink</x:v>
-      </x:c>
-      <x:c r="E6" s="113" t="str">
-        <x:v>Keep staging cr69a_transcriptlink at 2,000.</x:v>
-      </x:c>
-      <x:c r="F6" s="113" t="str">
-        <x:v>new_GRBPresentationLink.new_transcriptlink is already 2,000; migration flow is not implemented.</x:v>
-      </x:c>
-      <x:c r="G6" s="113" t="str">
-        <x:v>Verified</x:v>
-      </x:c>
-      <x:c r="H6" s="114" t="str">
-        <x:v>Published managed export 1.0.0.138: staging cr69a_transcriptlink and destination new_transcriptlink are both 2,000. Presentation-link migration flow remains unimplemented.</x:v>
+      <x:c r="B6" s="116" t="str">
+        <x:v>UAT QA</x:v>
+      </x:c>
+      <x:c r="C6" s="116" t="str">
+        <x:v>Migration batch</x:v>
+      </x:c>
+      <x:c r="D6" s="116" t="str">
+        <x:v>Counts and golden records</x:v>
+      </x:c>
+      <x:c r="E6" s="116" t="str">
+        <x:v>Reconcile source, staging, output, relationships, long text, and invalid-date nulling.</x:v>
+      </x:c>
+      <x:c r="F6" s="116" t="str">
+        <x:v>This is the release evidence for IMPL-sized data.</x:v>
+      </x:c>
+      <x:c r="G6" s="116" t="str">
+        <x:v>To do</x:v>
+      </x:c>
+      <x:c r="H6" s="117" t="str">
+        <x:v>Record results in Mapping Governance and cutover notes.</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="24" hidden="0" customHeight="1">
-      <x:c r="A7" s="120" t="n">
+      <x:c r="A7" s="131" t="n">
         <x:v>6</x:v>
       </x:c>
-      <x:c r="B7" s="113" t="str">
-        <x:v>DEV schema</x:v>
-      </x:c>
-      <x:c r="C7" s="113" t="str">
-        <x:v>Staging System Intake</x:v>
-      </x:c>
-      <x:c r="D7" s="113" t="str">
-        <x:v>cr69a_business_need</x:v>
-      </x:c>
-      <x:c r="E7" s="113" t="str">
-        <x:v>Keep staging cr69a_business_need at 4,000.</x:v>
-      </x:c>
-      <x:c r="F7" s="113" t="str">
-        <x:v>Request cr69a_business_need is already 4,000.</x:v>
-      </x:c>
-      <x:c r="G7" s="113" t="str">
-        <x:v>Verified</x:v>
-      </x:c>
-      <x:c r="H7" s="114" t="str">
-        <x:v>Published managed export 1.0.0.138: staging and Request cr69a_business_need are both 4,000.</x:v>
+      <x:c r="B7" s="116" t="str">
+        <x:v>Source cleanup</x:v>
+      </x:c>
+      <x:c r="C7" s="116" t="str">
+        <x:v>system_intakes.csv</x:v>
+      </x:c>
+      <x:c r="D7" s="116" t="str">
+        <x:v>project_acronym on 422cb351-4767-4c95-9915-a746e9ab371a</x:v>
+      </x:c>
+      <x:c r="E7" s="116" t="str">
+        <x:v>Clear the invalid 226-character formula-style test payload; do not widen the 100-character acronym schema.</x:v>
+      </x:c>
+      <x:c r="F7" s="116" t="str">
+        <x:v>All other nonblank IMPL acronyms are 15 characters or fewer.</x:v>
+      </x:c>
+      <x:c r="G7" s="116" t="str">
+        <x:v>Ready for PO</x:v>
+      </x:c>
+      <x:c r="H7" s="117" t="str">
+        <x:v>Corrected source copy contains 1,036 rows and changes only this one cell to blank.</x:v>
       </x:c>
     </x:row>
     <x:row r="8" ht="36" hidden="0" customHeight="1">
-      <x:c r="A8" s="120" t="n">
+      <x:c r="A8" s="131" t="n">
         <x:v>7</x:v>
       </x:c>
-      <x:c r="B8" s="113" t="str">
-        <x:v>DEV schema</x:v>
-      </x:c>
-      <x:c r="C8" s="113" t="str">
-        <x:v>Staging System Intake</x:v>
-      </x:c>
-      <x:c r="D8" s="113" t="str">
-        <x:v>cr69a_decision_next_steps</x:v>
-      </x:c>
-      <x:c r="E8" s="113" t="str">
-        <x:v>Keep staging cr69a_decision_next_steps at 4,000.</x:v>
-      </x:c>
-      <x:c r="F8" s="113" t="str">
-        <x:v>Request cr3ee_nextsteps is also 4,000 in export 1.0.0.138.</x:v>
-      </x:c>
-      <x:c r="G8" s="113" t="str">
-        <x:v>Verified</x:v>
-      </x:c>
-      <x:c r="H8" s="114" t="str">
-        <x:v>Published managed export 1.0.0.138: staging cr69a_decision_next_steps and Request cr3ee_nextsteps are both 4,000.</x:v>
+      <x:c r="B8" s="116" t="str">
+        <x:v>UAT run</x:v>
+      </x:c>
+      <x:c r="C8" s="116" t="str">
+        <x:v>Migration dataflows</x:v>
+      </x:c>
+      <x:c r="D8" s="116" t="str">
+        <x:v>Connections and environment variable IDs</x:v>
+      </x:c>
+      <x:c r="E8" s="116" t="str">
+        <x:v>Configure and publish every downstream migration dataflow, then query operational IDs and update the migration configuration environment variable.</x:v>
+      </x:c>
+      <x:c r="F8" s="116" t="str">
+        <x:v>Connection configuration may create or replace operational IDs, so capture IDs only after configuration is complete.</x:v>
+      </x:c>
+      <x:c r="G8" s="116" t="str">
+        <x:v>To do</x:v>
+      </x:c>
+      <x:c r="H8" s="117" t="str">
+        <x:v>User is reconfiguring connections; ID generation is the next step.</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="36" hidden="0" customHeight="1">
-      <x:c r="A9" s="120" t="n">
-        <x:v>8</x:v>
-      </x:c>
-      <x:c r="B9" s="113" t="str">
-        <x:v>DEV schema</x:v>
-      </x:c>
-      <x:c r="C9" s="113" t="str">
-        <x:v>Request</x:v>
-      </x:c>
-      <x:c r="D9" s="113" t="str">
-        <x:v>cr3ee_nextsteps</x:v>
-      </x:c>
-      <x:c r="E9" s="113" t="str">
-        <x:v>Keep Request cr3ee_nextsteps at 4,000.</x:v>
-      </x:c>
-      <x:c r="F9" s="113" t="str">
-        <x:v>Required to receive decision_next_steps without truncation.</x:v>
-      </x:c>
-      <x:c r="G9" s="113" t="str">
-        <x:v>Verified</x:v>
-      </x:c>
-      <x:c r="H9" s="114" t="str">
-        <x:v>Published managed export 1.0.0.138: Request cr3ee_nextsteps is 4,000. Runtime migration of the 2,342-character value remains a UAT QA check.</x:v>
-      </x:c>
+      <x:c r="A9"/>
+      <x:c r="B9"/>
+      <x:c r="C9"/>
+      <x:c r="D9"/>
+      <x:c r="E9"/>
+      <x:c r="F9"/>
+      <x:c r="G9"/>
+      <x:c r="H9"/>
     </x:row>
     <x:row r="10" ht="36" hidden="0" customHeight="1">
-      <x:c r="A10" s="120" t="n">
-        <x:v>9</x:v>
-      </x:c>
-      <x:c r="B10" s="113" t="str">
-        <x:v>DEV schema</x:v>
-      </x:c>
-      <x:c r="C10" s="113" t="str">
-        <x:v>Staging System Intake</x:v>
-      </x:c>
-      <x:c r="D10" s="113" t="str">
-        <x:v>cr69a_lcid_scope</x:v>
-      </x:c>
-      <x:c r="E10" s="113" t="str">
-        <x:v>Keep staging cr69a_lcid_scope at 4,000.</x:v>
-      </x:c>
-      <x:c r="F10" s="113" t="str">
-        <x:v>LCID cr3ee_scope is also 4,000 in export 1.0.0.138.</x:v>
-      </x:c>
-      <x:c r="G10" s="113" t="str">
-        <x:v>Verified</x:v>
-      </x:c>
-      <x:c r="H10" s="114" t="str">
-        <x:v>Published managed export 1.0.0.138: staging cr69a_lcid_scope and LCID cr3ee_scope are both 4,000.</x:v>
-      </x:c>
+      <x:c r="A10"/>
+      <x:c r="B10"/>
+      <x:c r="C10"/>
+      <x:c r="D10"/>
+      <x:c r="E10"/>
+      <x:c r="F10"/>
+      <x:c r="G10"/>
+      <x:c r="H10"/>
     </x:row>
     <x:row r="11" ht="36" hidden="0" customHeight="1">
-      <x:c r="A11" s="120" t="n">
-        <x:v>10</x:v>
-      </x:c>
-      <x:c r="B11" s="113" t="str">
-        <x:v>DEV schema</x:v>
-      </x:c>
-      <x:c r="C11" s="113" t="str">
-        <x:v>Life Cycle ID</x:v>
-      </x:c>
-      <x:c r="D11" s="113" t="str">
-        <x:v>cr3ee_Scope</x:v>
-      </x:c>
-      <x:c r="E11" s="113" t="str">
-        <x:v>Keep LCID cr3ee_scope at 4,000.</x:v>
-      </x:c>
-      <x:c r="F11" s="113" t="str">
-        <x:v>Required to receive lcid_scope without truncation.</x:v>
-      </x:c>
-      <x:c r="G11" s="113" t="str">
-        <x:v>Verified</x:v>
-      </x:c>
-      <x:c r="H11" s="114" t="str">
-        <x:v>Published managed export 1.0.0.138: LCID cr3ee_scope is 4,000. Runtime migration of the 2,342-character value remains a UAT QA check.</x:v>
-      </x:c>
+      <x:c r="A11"/>
+      <x:c r="B11"/>
+      <x:c r="C11"/>
+      <x:c r="D11"/>
+      <x:c r="E11"/>
+      <x:c r="F11"/>
+      <x:c r="G11"/>
+      <x:c r="H11"/>
     </x:row>
     <x:row r="12" ht="48" hidden="0" customHeight="1">
-      <x:c r="A12" s="120" t="n">
-        <x:v>11</x:v>
-      </x:c>
-      <x:c r="B12" s="113" t="str">
-        <x:v>DEV schema</x:v>
-      </x:c>
-      <x:c r="C12" s="113" t="str">
-        <x:v>Staging System Intake</x:v>
-      </x:c>
-      <x:c r="D12" s="113" t="str">
-        <x:v>cr69a_grt_review_email_body</x:v>
-      </x:c>
-      <x:c r="E12" s="113" t="str">
-        <x:v>Keep staging cr69a_grt_review_email_body at 2,000.</x:v>
-      </x:c>
-      <x:c r="F12" s="113" t="str">
-        <x:v>No destination mapping exists.</x:v>
-      </x:c>
-      <x:c r="G12" s="113" t="str">
-        <x:v>Verified</x:v>
-      </x:c>
-      <x:c r="H12" s="114" t="str">
-        <x:v>Published managed export 1.0.0.139: staging cr69a_grt_review_email_body is 2,000. No destination mapping currently exists, so omission remains intentional unless scope changes.</x:v>
-      </x:c>
+      <x:c r="A12"/>
+      <x:c r="B12"/>
+      <x:c r="C12"/>
+      <x:c r="D12"/>
+      <x:c r="E12"/>
+      <x:c r="F12"/>
+      <x:c r="G12"/>
+      <x:c r="H12"/>
     </x:row>
     <x:row r="13" ht="48" hidden="0" customHeight="1">
-      <x:c r="A13" s="120" t="n">
-        <x:v>12</x:v>
-      </x:c>
-      <x:c r="B13" s="113" t="str">
-        <x:v>DEV review</x:v>
-      </x:c>
-      <x:c r="C13" s="113" t="str">
-        <x:v>Staging System Intake</x:v>
-      </x:c>
-      <x:c r="D13" s="113" t="str">
-        <x:v>Pre-1753 date normalization</x:v>
-      </x:c>
-      <x:c r="E13" s="113" t="str">
-        <x:v>Remove any active customization from the UAT Stage System Intakes dataflow, confirm the managed query contains the pre-1753 guard, then publish and refresh.</x:v>
-      </x:c>
-      <x:c r="F13" s="113" t="str">
-        <x:v>The local query normalizes every typed System Intake date/date-time column before loading Dataverse.</x:v>
-      </x:c>
-      <x:c r="G13" s="113" t="str">
-        <x:v>Verified</x:v>
-      </x:c>
-      <x:c r="H13" s="114" t="str">
-        <x:v>UAT operational Stage System Intakes contains DataverseMinimumDate = #date(1753, 1, 1). The fresh UAT staging run produced no pre-1753 date errors.</x:v>
-      </x:c>
+      <x:c r="A13"/>
+      <x:c r="B13"/>
+      <x:c r="C13"/>
+      <x:c r="D13"/>
+      <x:c r="E13"/>
+      <x:c r="F13"/>
+      <x:c r="G13"/>
+      <x:c r="H13"/>
     </x:row>
     <x:row r="14" ht="24" hidden="0" customHeight="1">
-      <x:c r="A14" s="120" t="n">
-        <x:v>13</x:v>
-      </x:c>
-      <x:c r="B14" s="113" t="str">
-        <x:v>DEV review</x:v>
-      </x:c>
-      <x:c r="C14" s="113" t="str">
-        <x:v>Activity Log</x:v>
-      </x:c>
-      <x:c r="D14" s="113" t="str">
-        <x:v>new_recommendationsforthegrb</x:v>
-      </x:c>
-      <x:c r="E14" s="113" t="str">
-        <x:v>Confirm the field is 2,000 and included in the exported solution.</x:v>
-      </x:c>
-      <x:c r="F14" s="113" t="str">
-        <x:v>Earlier DEV change is not reflected in the checked-in solution XML yet.</x:v>
-      </x:c>
-      <x:c r="G14" s="113" t="str">
-        <x:v>Verified</x:v>
-      </x:c>
-      <x:c r="H14" s="114" t="str">
-        <x:v>Published managed export 1.0.0.138: Activity Log new_recommendationsforthegrb is 2,000.</x:v>
-      </x:c>
+      <x:c r="A14"/>
+      <x:c r="B14"/>
+      <x:c r="C14"/>
+      <x:c r="D14"/>
+      <x:c r="E14"/>
+      <x:c r="F14"/>
+      <x:c r="G14"/>
+      <x:c r="H14"/>
     </x:row>
     <x:row r="15" ht="24" hidden="0" customHeight="1">
-      <x:c r="A15" s="120" t="n">
-        <x:v>14</x:v>
-      </x:c>
-      <x:c r="B15" s="113" t="str">
-        <x:v>DEV review</x:v>
-      </x:c>
-      <x:c r="C15" s="113" t="str">
-        <x:v>Staging Contact</x:v>
-      </x:c>
-      <x:c r="D15" s="113" t="str">
-        <x:v>cr69a_roles</x:v>
-      </x:c>
-      <x:c r="E15" s="113" t="str">
-        <x:v>Confirm 1,000-character staging size.</x:v>
-      </x:c>
-      <x:c r="F15" s="113" t="str">
-        <x:v>Destination is multi-select choice; no target length change.</x:v>
-      </x:c>
-      <x:c r="G15" s="113" t="str">
-        <x:v>Verified</x:v>
-      </x:c>
-      <x:c r="H15" s="114" t="str">
-        <x:v>Published managed export 1.0.0.138: staging contact cr69a_roles is 1,000.</x:v>
-      </x:c>
+      <x:c r="A15"/>
+      <x:c r="B15"/>
+      <x:c r="C15"/>
+      <x:c r="D15"/>
+      <x:c r="E15"/>
+      <x:c r="F15"/>
+      <x:c r="G15"/>
+      <x:c r="H15"/>
     </x:row>
     <x:row r="16" ht="48" hidden="0" customHeight="1">
-      <x:c r="A16" s="120" t="n">
-        <x:v>15</x:v>
-      </x:c>
-      <x:c r="B16" s="113" t="str">
-        <x:v>DEV review</x:v>
-      </x:c>
-      <x:c r="C16" s="113" t="str">
-        <x:v>Staging Edit Requests</x:v>
-      </x:c>
-      <x:c r="D16" s="113" t="str">
-        <x:v>new_requesterfeedbackmultitext</x:v>
-      </x:c>
-      <x:c r="E16" s="113" t="str">
-        <x:v>Confirm 2,000-character replacement field and mapping; old field remains unmapped.</x:v>
-      </x:c>
-      <x:c r="F16" s="113" t="str">
-        <x:v>Edit Request destination supports 4,000.</x:v>
-      </x:c>
-      <x:c r="G16" s="113" t="str">
-        <x:v>Verified</x:v>
-      </x:c>
-      <x:c r="H16" s="114" t="str">
-        <x:v>Replacement field and mapping passed DEV staging and the full DEV migration.</x:v>
-      </x:c>
+      <x:c r="A16"/>
+      <x:c r="B16"/>
+      <x:c r="C16"/>
+      <x:c r="D16"/>
+      <x:c r="E16"/>
+      <x:c r="F16"/>
+      <x:c r="G16"/>
+      <x:c r="H16"/>
     </x:row>
     <x:row r="17" ht="24" hidden="0" customHeight="1">
-      <x:c r="A17" s="120" t="n">
-        <x:v>16</x:v>
-      </x:c>
-      <x:c r="B17" s="113" t="str">
-        <x:v>DEV review</x:v>
-      </x:c>
-      <x:c r="C17" s="113" t="str">
-        <x:v>Staging GRB Discussion</x:v>
-      </x:c>
-      <x:c r="D17" s="113" t="str">
-        <x:v>cr69a_content</x:v>
-      </x:c>
-      <x:c r="E17" s="113" t="str">
-        <x:v>Confirm 1,000-character staging size.</x:v>
-      </x:c>
-      <x:c r="F17" s="113" t="str">
-        <x:v>Destination migration remains out of scope/not implemented.</x:v>
-      </x:c>
-      <x:c r="G17" s="113" t="str">
-        <x:v>Verified</x:v>
-      </x:c>
-      <x:c r="H17" s="114" t="str">
-        <x:v>Published managed export 1.0.0.138: staging GRB discussion cr69a_content is 1,000.</x:v>
-      </x:c>
+      <x:c r="A17"/>
+      <x:c r="B17"/>
+      <x:c r="C17"/>
+      <x:c r="D17"/>
+      <x:c r="E17"/>
+      <x:c r="F17"/>
+      <x:c r="G17"/>
+      <x:c r="H17"/>
     </x:row>
     <x:row r="18" ht="24" hidden="0" customHeight="1">
-      <x:c r="A18" s="120" t="n">
-        <x:v>17</x:v>
-      </x:c>
-      <x:c r="B18" s="113" t="str">
-        <x:v>DEV review</x:v>
-      </x:c>
-      <x:c r="C18" s="113" t="str">
-        <x:v>Staging GRB Presentation Links</x:v>
-      </x:c>
-      <x:c r="D18" s="113" t="str">
-        <x:v>cr69a_recordinglink</x:v>
-      </x:c>
-      <x:c r="E18" s="113" t="str">
-        <x:v>Confirm 2,000-character staging size.</x:v>
-      </x:c>
-      <x:c r="F18" s="113" t="str">
-        <x:v>Presentation-link migration remains not implemented.</x:v>
-      </x:c>
-      <x:c r="G18" s="113" t="str">
-        <x:v>Verified</x:v>
-      </x:c>
-      <x:c r="H18" s="114" t="str">
-        <x:v>Published managed export 1.0.0.138: staging GRB presentation cr69a_recordinglink is 2,000.</x:v>
-      </x:c>
+      <x:c r="A18"/>
+      <x:c r="B18"/>
+      <x:c r="C18"/>
+      <x:c r="D18"/>
+      <x:c r="E18"/>
+      <x:c r="F18"/>
+      <x:c r="G18"/>
+      <x:c r="H18"/>
     </x:row>
     <x:row r="19" ht="48" hidden="0" customHeight="1">
-      <x:c r="A19" s="120" t="n">
-        <x:v>18</x:v>
-      </x:c>
-      <x:c r="B19" s="113" t="str">
-        <x:v>DEV review</x:v>
-      </x:c>
-      <x:c r="C19" s="113" t="str">
-        <x:v>Staging Business Case</x:v>
-      </x:c>
-      <x:c r="D19" s="113" t="str">
-        <x:v>new_requestphonenumbertext</x:v>
-      </x:c>
-      <x:c r="E19" s="113" t="str">
-        <x:v>Confirm text replacement field, 50-character size, and dataflow mapping; old float field unmapped.</x:v>
-      </x:c>
-      <x:c r="F19" s="113" t="str">
-        <x:v>Request new_requesterphonenumberlegacy must be present and text-capable.</x:v>
-      </x:c>
-      <x:c r="G19" s="113" t="str">
-        <x:v>Verified</x:v>
-      </x:c>
-      <x:c r="H19" s="114" t="str">
-        <x:v>Replacement phone field and mapping passed DEV staging and the full DEV migration.</x:v>
-      </x:c>
+      <x:c r="A19"/>
+      <x:c r="B19"/>
+      <x:c r="C19"/>
+      <x:c r="D19"/>
+      <x:c r="E19"/>
+      <x:c r="F19"/>
+      <x:c r="G19"/>
+      <x:c r="H19"/>
     </x:row>
     <x:row r="20" ht="60" hidden="0" customHeight="1">
-      <x:c r="A20" s="120" t="n">
-        <x:v>19</x:v>
-      </x:c>
-      <x:c r="B20" s="113" t="str">
-        <x:v>DEV deployment</x:v>
-      </x:c>
-      <x:c r="C20" s="113" t="str">
-        <x:v>Application solution</x:v>
-      </x:c>
-      <x:c r="D20" s="113" t="str">
-        <x:v>All schema changes</x:v>
-      </x:c>
-      <x:c r="E20" s="113" t="str">
-        <x:v>Publish all customizations, export the managed solution, and unpack/pull it locally.</x:v>
-      </x:c>
-      <x:c r="F20" s="113" t="str">
-        <x:v>Prevents unpublished definitions from being omitted.</x:v>
-      </x:c>
-      <x:c r="G20" s="113" t="str">
-        <x:v>Verified</x:v>
-      </x:c>
-      <x:c r="H20" s="114" t="str">
-        <x:v>UAT reports managed InitialITGO 1.0.0.140. Read-only effective-metadata verification passed after active customizations were removed.</x:v>
-      </x:c>
+      <x:c r="A20"/>
+      <x:c r="B20"/>
+      <x:c r="C20"/>
+      <x:c r="D20"/>
+      <x:c r="E20"/>
+      <x:c r="F20"/>
+      <x:c r="G20"/>
+      <x:c r="H20"/>
     </x:row>
     <x:row r="21" ht="15" hidden="0" customHeight="1">
-      <x:c r="A21" s="120" t="n">
-        <x:v>20</x:v>
-      </x:c>
-      <x:c r="B21" s="113" t="str">
-        <x:v>UAT deployment</x:v>
-      </x:c>
-      <x:c r="C21" s="113" t="str">
-        <x:v>Application solution</x:v>
-      </x:c>
-      <x:c r="D21" s="113" t="str">
-        <x:v>Managed upgrade</x:v>
-      </x:c>
-      <x:c r="E21" s="113" t="str">
-        <x:v>Deploy the application solution before the migration solution.</x:v>
-      </x:c>
-      <x:c r="F21" s="113" t="str">
-        <x:v>Migration mappings require the new fields and capacities.</x:v>
-      </x:c>
-      <x:c r="G21" s="113" t="str">
-        <x:v>Verified</x:v>
-      </x:c>
-      <x:c r="H21" s="114" t="str">
-        <x:v>Removed active customizations from the seven affected columns. UAT API verification passed 7/7: Alternative A/B Summary 4,000; transcript link 2,000; business need, decision next steps, and LCID scope 4,000; GRT review email body 2,000.</x:v>
-      </x:c>
+      <x:c r="A21"/>
+      <x:c r="B21"/>
+      <x:c r="C21"/>
+      <x:c r="D21"/>
+      <x:c r="E21"/>
+      <x:c r="F21"/>
+      <x:c r="G21"/>
+      <x:c r="H21"/>
     </x:row>
     <x:row r="22" ht="24" hidden="0" customHeight="1">
-      <x:c r="A22" s="120" t="n">
-        <x:v>21</x:v>
-      </x:c>
-      <x:c r="B22" s="113" t="str">
-        <x:v>UAT deployment</x:v>
-      </x:c>
-      <x:c r="C22" s="113" t="str">
-        <x:v>Affected columns</x:v>
-      </x:c>
-      <x:c r="D22" s="113" t="str">
-        <x:v>Solution layers</x:v>
-      </x:c>
-      <x:c r="E22" s="113" t="str">
-        <x:v>Inspect each changed column for unmanaged layers and remove only confirmed blockers.</x:v>
-      </x:c>
-      <x:c r="F22" s="113" t="str">
-        <x:v>Column-level layers previously overrode managed MaxLength changes.</x:v>
-      </x:c>
-      <x:c r="G22" s="113" t="str">
-        <x:v>Verified</x:v>
-      </x:c>
-      <x:c r="H22" s="114" t="str">
-        <x:v>Confirmed blocking column-level unmanaged layers were removed and effective UAT schema values matched the managed definitions before the latest staging run.</x:v>
-      </x:c>
+      <x:c r="A22"/>
+      <x:c r="B22"/>
+      <x:c r="C22"/>
+      <x:c r="D22"/>
+      <x:c r="E22"/>
+      <x:c r="F22"/>
+      <x:c r="G22"/>
+      <x:c r="H22"/>
     </x:row>
     <x:row r="23" ht="24" hidden="0" customHeight="1">
-      <x:c r="A23" s="120" t="n">
-        <x:v>22</x:v>
-      </x:c>
-      <x:c r="B23" s="113" t="str">
-        <x:v>UAT deployment</x:v>
-      </x:c>
-      <x:c r="C23" s="113" t="str">
-        <x:v>Migration solution</x:v>
-      </x:c>
-      <x:c r="D23" s="113" t="str">
-        <x:v>Dataflows and configuration</x:v>
-      </x:c>
-      <x:c r="E23" s="113" t="str">
-        <x:v>Deploy, then restore environment-specific dataflow configuration and connections.</x:v>
-      </x:c>
-      <x:c r="F23" s="113" t="str">
-        <x:v>Dataflow IDs/configuration can reset during deployment.</x:v>
-      </x:c>
-      <x:c r="G23" s="113" t="str">
-        <x:v>In progress</x:v>
-      </x:c>
-      <x:c r="H23" s="114" t="str">
-        <x:v>Migration solution is deployed and all 13 staging dataflows are configured/published. Downstream migration dataflows still need connection configuration; regenerate migration IDs only after that configuration is complete.</x:v>
-      </x:c>
+      <x:c r="A23"/>
+      <x:c r="B23"/>
+      <x:c r="C23"/>
+      <x:c r="D23"/>
+      <x:c r="E23"/>
+      <x:c r="F23"/>
+      <x:c r="G23"/>
+      <x:c r="H23"/>
     </x:row>
     <x:row r="24" ht="24" hidden="0" customHeight="1">
-      <x:c r="A24" s="120" t="n">
-        <x:v>23</x:v>
-      </x:c>
-      <x:c r="B24" s="113" t="str">
-        <x:v>UAT validation</x:v>
-      </x:c>
-      <x:c r="C24" s="113" t="str">
-        <x:v>Stage System Intakes</x:v>
-      </x:c>
-      <x:c r="D24" s="113" t="str">
-        <x:v>Main output query</x:v>
-      </x:c>
-      <x:c r="E24" s="113" t="str">
-        <x:v>Remove any active customization from Stage System Intakes, verify the managed output is based on Normalized Dataverse dates, publish, and rerun the staging flow.</x:v>
-      </x:c>
-      <x:c r="F24" s="113" t="str">
-        <x:v>The failed UAT run allowed 47 pre-1753 values to reach Dataverse even though the repository query contains the complete guard.</x:v>
-      </x:c>
-      <x:c r="G24" s="113" t="str">
-        <x:v>Verified</x:v>
-      </x:c>
-      <x:c r="H24" s="114" t="str">
-        <x:v>Fresh UAT staging produced no 1111/0021 date payload errors; the managed date guard is executing correctly.</x:v>
-      </x:c>
+      <x:c r="A24"/>
+      <x:c r="B24"/>
+      <x:c r="C24"/>
+      <x:c r="D24"/>
+      <x:c r="E24"/>
+      <x:c r="F24"/>
+      <x:c r="G24"/>
+      <x:c r="H24"/>
     </x:row>
     <x:row r="25" ht="24" hidden="0" customHeight="1">
-      <x:c r="A25" s="120" t="n">
-        <x:v>24</x:v>
-      </x:c>
-      <x:c r="B25" s="113" t="str">
-        <x:v>UAT run</x:v>
-      </x:c>
-      <x:c r="C25" s="113" t="str">
-        <x:v>Staging tables</x:v>
-      </x:c>
-      <x:c r="D25" s="113" t="str">
-        <x:v>Fresh batch</x:v>
-      </x:c>
-      <x:c r="E25" s="113" t="str">
-        <x:v>Complete rollback, then refresh staging dataflows in dependency order.</x:v>
-      </x:c>
-      <x:c r="F25" s="113" t="str">
-        <x:v>A fresh batch avoids mixing partial attempts.</x:v>
-      </x:c>
-      <x:c r="G25" s="113" t="str">
-        <x:v>Partially verified</x:v>
-      </x:c>
-      <x:c r="H25" s="114" t="str">
-        <x:v>All staging dataflows succeeded except one System Intake row: 1,035 of 1,036 loaded. The remaining project_acronym value is invalid source data and has been cleared in a corrected source copy.</x:v>
-      </x:c>
+      <x:c r="A25"/>
+      <x:c r="B25"/>
+      <x:c r="C25"/>
+      <x:c r="D25"/>
+      <x:c r="E25"/>
+      <x:c r="F25"/>
+      <x:c r="G25"/>
+      <x:c r="H25"/>
     </x:row>
     <x:row r="26" ht="24" hidden="0" customHeight="1">
-      <x:c r="A26" s="120" t="n">
-        <x:v>25</x:v>
-      </x:c>
-      <x:c r="B26" s="113" t="str">
-        <x:v>UAT QA</x:v>
-      </x:c>
-      <x:c r="C26" s="113" t="str">
-        <x:v>All staged text</x:v>
-      </x:c>
-      <x:c r="D26" s="113" t="str">
-        <x:v>Length reconciliation</x:v>
-      </x:c>
-      <x:c r="E26" s="113" t="str">
-        <x:v>Compare source maximum lengths with staged values for every widened/replacement field.</x:v>
-      </x:c>
-      <x:c r="F26" s="113" t="str">
-        <x:v>Proves values were preserved rather than silently truncated.</x:v>
-      </x:c>
-      <x:c r="G26" s="113" t="str">
-        <x:v>To do</x:v>
-      </x:c>
-      <x:c r="H26" s="114" t="str">
-        <x:v>Max length and representative long values match source.</x:v>
-      </x:c>
+      <x:c r="A26"/>
+      <x:c r="B26"/>
+      <x:c r="C26"/>
+      <x:c r="D26"/>
+      <x:c r="E26"/>
+      <x:c r="F26"/>
+      <x:c r="G26"/>
+      <x:c r="H26"/>
     </x:row>
     <x:row r="27" ht="15" hidden="0" customHeight="1">
-      <x:c r="A27" s="120" t="n">
-        <x:v>26</x:v>
-      </x:c>
-      <x:c r="B27" s="113" t="str">
-        <x:v>UAT run</x:v>
-      </x:c>
-      <x:c r="C27" s="113" t="str">
-        <x:v>Migration dataflows</x:v>
-      </x:c>
-      <x:c r="D27" s="113" t="str">
-        <x:v>Create/link/update phases</x:v>
-      </x:c>
-      <x:c r="E27" s="113" t="str">
-        <x:v>Run downstream migration only after staging passes.</x:v>
-      </x:c>
-      <x:c r="F27" s="113" t="str">
-        <x:v>Destination increases are required before Request and LCID writes.</x:v>
-      </x:c>
-      <x:c r="G27" s="113" t="str">
-        <x:v>To do</x:v>
-      </x:c>
-      <x:c r="H27" s="114" t="str">
-        <x:v>All outputs and QA queries succeed.</x:v>
-      </x:c>
+      <x:c r="A27"/>
+      <x:c r="B27"/>
+      <x:c r="C27"/>
+      <x:c r="D27"/>
+      <x:c r="E27"/>
+      <x:c r="F27"/>
+      <x:c r="G27"/>
+      <x:c r="H27"/>
     </x:row>
     <x:row r="28" ht="24" hidden="0" customHeight="1">
-      <x:c r="A28" s="121" t="n">
-        <x:v>27</x:v>
-      </x:c>
-      <x:c r="B28" s="116" t="str">
-        <x:v>UAT QA</x:v>
-      </x:c>
-      <x:c r="C28" s="116" t="str">
-        <x:v>Migration batch</x:v>
-      </x:c>
-      <x:c r="D28" s="116" t="str">
-        <x:v>Counts and golden records</x:v>
-      </x:c>
-      <x:c r="E28" s="116" t="str">
-        <x:v>Reconcile source, staging, output, relationships, long text, and invalid-date nulling.</x:v>
-      </x:c>
-      <x:c r="F28" s="116" t="str">
-        <x:v>This is the release evidence for IMPL-sized data.</x:v>
-      </x:c>
-      <x:c r="G28" s="116" t="str">
-        <x:v>To do</x:v>
-      </x:c>
-      <x:c r="H28" s="117" t="str">
-        <x:v>Record results in Mapping Governance and cutover notes.</x:v>
-      </x:c>
+      <x:c r="A28"/>
+      <x:c r="B28"/>
+      <x:c r="C28"/>
+      <x:c r="D28"/>
+      <x:c r="E28"/>
+      <x:c r="F28"/>
+      <x:c r="G28"/>
+      <x:c r="H28"/>
     </x:row>
     <x:row r="29" ht="24" hidden="0" customHeight="1">
-      <x:c r="A29" s="131" t="n">
-        <x:v>28</x:v>
-      </x:c>
-      <x:c r="B29" s="116" t="str">
-        <x:v>DEV/UAT schema</x:v>
-      </x:c>
-      <x:c r="C29" s="116" t="str">
-        <x:v>Staging System Intake</x:v>
-      </x:c>
-      <x:c r="D29" s="116" t="str">
-        <x:v>new_solutionmultitext / new_lcidcostbaselinemultitext</x:v>
-      </x:c>
-      <x:c r="E29" s="116" t="str">
-        <x:v>Use 4,000-character replacement staging fields; leave the two legacy 100-character staging fields unmapped.</x:v>
-      </x:c>
-      <x:c r="F29" s="116" t="str">
-        <x:v>Create Requests reads new_solutionmultitext; Create LCIDs reads new_lcidcostbaselinemultitext.</x:v>
-      </x:c>
-      <x:c r="G29" s="116" t="str">
-        <x:v>Verified</x:v>
-      </x:c>
-      <x:c r="H29" s="117" t="str">
-        <x:v>DEV staging and full migration completed successfully. UAT staging also completed for these mappings.</x:v>
-      </x:c>
+      <x:c r="A29"/>
+      <x:c r="B29"/>
+      <x:c r="C29"/>
+      <x:c r="D29"/>
+      <x:c r="E29"/>
+      <x:c r="F29"/>
+      <x:c r="G29"/>
+      <x:c r="H29"/>
     </x:row>
     <x:row r="30" ht="24" hidden="0" customHeight="1">
-      <x:c r="A30" s="131" t="n">
-        <x:v>29</x:v>
-      </x:c>
-      <x:c r="B30" s="116" t="str">
-        <x:v>DEV migration</x:v>
-      </x:c>
-      <x:c r="C30" s="116" t="str">
-        <x:v>Historical GRB Activity Logs</x:v>
-      </x:c>
-      <x:c r="D30" s="116" t="str">
-        <x:v>UnmappedIssues filter</x:v>
-      </x:c>
-      <x:c r="E30" s="116" t="str">
-        <x:v>Filter clean preparation rows with [UnmappedIssues] = null, not an empty string.</x:v>
-      </x:c>
-      <x:c r="F30" s="116" t="str">
-        <x:v>The empty-string comparison silently produced zero final rows despite 206 valid preparation rows.</x:v>
-      </x:c>
-      <x:c r="G30" s="116" t="str">
-        <x:v>Verified</x:v>
-      </x:c>
-      <x:c r="H30" s="117" t="str">
-        <x:v>After correction, DEV created all 206 expected Activity Logs.</x:v>
-      </x:c>
+      <x:c r="A30"/>
+      <x:c r="B30"/>
+      <x:c r="C30"/>
+      <x:c r="D30"/>
+      <x:c r="E30"/>
+      <x:c r="F30"/>
+      <x:c r="G30"/>
+      <x:c r="H30"/>
     </x:row>
     <x:row r="31" ht="24" hidden="0" customHeight="1">
-      <x:c r="A31" s="131" t="n">
-        <x:v>30</x:v>
-      </x:c>
-      <x:c r="B31" s="116" t="str">
-        <x:v>Source cleanup</x:v>
-      </x:c>
-      <x:c r="C31" s="116" t="str">
-        <x:v>system_intakes.csv</x:v>
-      </x:c>
-      <x:c r="D31" s="116" t="str">
-        <x:v>project_acronym on 422cb351-4767-4c95-9915-a746e9ab371a</x:v>
-      </x:c>
-      <x:c r="E31" s="116" t="str">
-        <x:v>Clear the invalid 226-character formula-style test payload; do not widen the 100-character acronym schema.</x:v>
-      </x:c>
-      <x:c r="F31" s="116" t="str">
-        <x:v>All other nonblank IMPL acronyms are 15 characters or fewer.</x:v>
-      </x:c>
-      <x:c r="G31" s="116" t="str">
-        <x:v>Ready for PO</x:v>
-      </x:c>
-      <x:c r="H31" s="117" t="str">
-        <x:v>Corrected source copy contains 1,036 rows and changes only this one cell to blank.</x:v>
-      </x:c>
+      <x:c r="A31"/>
+      <x:c r="B31"/>
+      <x:c r="C31"/>
+      <x:c r="D31"/>
+      <x:c r="E31"/>
+      <x:c r="F31"/>
+      <x:c r="G31"/>
+      <x:c r="H31"/>
     </x:row>
     <x:row r="32" ht="36" hidden="0" customHeight="1">
-      <x:c r="A32" s="131" t="n">
-        <x:v>31</x:v>
-      </x:c>
-      <x:c r="B32" s="116" t="str">
-        <x:v>UAT run</x:v>
-      </x:c>
-      <x:c r="C32" s="116" t="str">
-        <x:v>Migration dataflows</x:v>
-      </x:c>
-      <x:c r="D32" s="116" t="str">
-        <x:v>Connections and environment variable IDs</x:v>
-      </x:c>
-      <x:c r="E32" s="116" t="str">
-        <x:v>Configure and publish every downstream migration dataflow, then query operational IDs and update the migration configuration environment variable.</x:v>
-      </x:c>
-      <x:c r="F32" s="116" t="str">
-        <x:v>Connection configuration may create or replace operational IDs, so capture IDs only after configuration is complete.</x:v>
-      </x:c>
-      <x:c r="G32" s="116" t="str">
-        <x:v>To do</x:v>
-      </x:c>
-      <x:c r="H32" s="117" t="str">
-        <x:v>User is reconfiguring connections; ID generation is the next step.</x:v>
-      </x:c>
+      <x:c r="A32"/>
+      <x:c r="B32"/>
+      <x:c r="C32"/>
+      <x:c r="D32"/>
+      <x:c r="E32"/>
+      <x:c r="F32"/>
+      <x:c r="G32"/>
+      <x:c r="H32"/>
+    </x:row>
+    <x:row r="33">
+      <x:c r="A33"/>
+      <x:c r="B33"/>
+      <x:c r="C33"/>
+      <x:c r="D33"/>
+      <x:c r="E33"/>
+      <x:c r="F33"/>
+      <x:c r="G33"/>
+      <x:c r="H33"/>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R81f9eb96071e405c"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R879481733b3c4057"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -10973,7 +10599,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf043b29abf0542b1"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7bc23cc80e134741"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -25524,7 +25150,7 @@
         <x:v>4000</x:v>
       </x:c>
       <x:c r="J23" t="str">
-        <x:v>Staging must increase from 100 to 4,000. Destination cr69a_business_need already supports 4,000.</x:v>
+        <x:v>Business need text length aligned. Verified in DEV Web API metadata on 2026-10-26.</x:v>
       </x:c>
     </x:row>
     <x:row r="24">
@@ -25553,7 +25179,7 @@
         <x:v>4000</x:v>
       </x:c>
       <x:c r="J24" t="str">
-        <x:v>Stage source solution through replacement staging field new_solutionmultitext (4,000); leave legacy cr69a_solution staging mapping at None. 03-create-requests.m reads the replacement field and emits the Request solution value. DEV staging and the full DEV migration completed successfully.</x:v>
+        <x:v>Mapped replacement staging field new_solutionmultitext and Request destination are both 4,000. The legacy staging field is also now 4,000. Verified in DEV Web API metadata on 2026-10-26.</x:v>
       </x:c>
     </x:row>
     <x:row r="25">
@@ -25696,7 +25322,7 @@
         <x:v>n/a</x:v>
       </x:c>
       <x:c r="J32" t="str">
-        <x:v>Published managed export 1.0.0.139 confirms the staging field is 2,000. No destination mapping exists; preserve as staging-only unless the legacy email body is added to migration scope.</x:v>
+        <x:v>Staging review email body supports 2,000 characters; no destination field is mapped. Verified in DEV Web API metadata on 2026-10-26.</x:v>
       </x:c>
     </x:row>
     <x:row r="33">
@@ -25844,10 +25470,10 @@
         <x:v>4000</x:v>
       </x:c>
       <x:c r="I40" s="1" t="n">
-        <x:v>2000</x:v>
+        <x:v>4000</x:v>
       </x:c>
       <x:c r="J40" t="str">
-        <x:v>Staging must increase from 100 to 4,000. Destination cr69a_LifeCycleIDs.cr3ee_Scope must increase from 2,000 to 4,000 to prevent truncation/failure.</x:v>
+        <x:v>LCID scope text length aligned. Verified in DEV Web API metadata on 2026-10-26.</x:v>
       </x:c>
     </x:row>
     <x:row r="41">
@@ -26097,10 +25723,10 @@
         <x:v>4000</x:v>
       </x:c>
       <x:c r="I53" t="n">
-        <x:v>2000</x:v>
+        <x:v>4000</x:v>
       </x:c>
       <x:c r="J53" t="str">
-        <x:v>03-create-requests.m emits next_steps_dataverse_format for finished requests. Increase destination cr3ee_nextsteps from 2,000 to 4,000.</x:v>
+        <x:v>Decision/next steps text length aligned. Verified in DEV Web API metadata on 2026-10-26.</x:v>
       </x:c>
     </x:row>
     <x:row r="54">
@@ -26250,9 +25876,11 @@
       <x:c r="H61" t="n">
         <x:v>4000</x:v>
       </x:c>
-      <x:c r="I61" s="1"/>
+      <x:c r="I61" s="1" t="n">
+        <x:v>4000</x:v>
+      </x:c>
       <x:c r="J61" t="str">
-        <x:v>Stage source lcid_cost_baseline through replacement staging field new_lcidcostbaselinemultitext (4,000); leave legacy cr69a_lcid_cost_baseline staging mapping at None. 01-create-lcids.m reads the replacement field and emits cr3ee_costbaseline. DEV staging and the full DEV migration completed successfully; confirm the longest IMPL value during UAT migration QA.</x:v>
+        <x:v>Mapped replacement staging field new_lcidcostbaselinemultitext and LCID destination cr3ee_CostBaseline are both 4,000. Verified in DEV Web API metadata on 2026-10-28.</x:v>
       </x:c>
     </x:row>
     <x:row r="62">

</xml_diff>